<commit_message>
Replace the storyboard draft with the critic-checked version
Four family critics traced every claim to the catalogue and tightened the
copy; 15 pages, 105 blocks, 0 brevity violations. story-scroll.html is the
published roadmap and prompt page.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
+++ b/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
@@ -50535,7 +50535,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five sessions in one box, visible from the first treatment.</t>
+          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five ampoules and five gel-mask sachets in one box, hydration and radiance visible from the first treatment.</t>
         </is>
       </c>
       <c r="E2" s="5" t="n">
@@ -50583,7 +50583,7 @@
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>Start: block-0 hero (gold carton right, vials in front). Camera pushes slowly toward the mirror-gold face of the carton; its reflection ripples and brightens until the frame is pure gold light (1.5 s). The light cools and resolves into the block-1 macro: a microneedling pen tip gliding across a cheek under warm rim light, the tip leaving the frame at the end. 4 s, dolly-in then settle. The product becomes the light that reveals the problem.</t>
+          <t>Start: block-0 hero (gold carton right, vials in front). Camera pushes slowly toward the mirror-gold face of the carton; its reflection ripples and brightens until the frame is pure gold light (1.5 s). The light cools and resolves into the block-1 macro: a champagne-gold cordless microneedling pen tip gliding across a cheek under warm rim light, the tip leaving the frame at the end. 4 s, dolly-in then settle. The product becomes the light that reveals the problem.</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
@@ -50610,7 +50610,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five sessions in one box, visible from the first treatment.</t>
+          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five ampoules and five gel-mask sachets in one box, hydration and radiance visible from the first treatment.</t>
         </is>
       </c>
       <c r="E3" s="5" t="n">
@@ -50653,12 +50653,12 @@
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic close-up, 16:9. A gloved practitioner's hand holds a slim cordless microneedling pen just above a woman's cheek; macro view of skin texture with faint dots of temporary micro-channels catching warm light. The woman's face is in soft focus, eyes closed, relaxed. Environment: dark treatment room in black and deep bronze tones, a thin warm gold edge light along the jawline. Camera: 100 mm macro, f/2.8, focus on the pen tip and the skin, the image occupies the left two-thirds and the right third falls to near-black for text. Mood: precise, clinical, luxurious. No overlay text, no logos.</t>
+          <t>Photoreal cinematic close-up, 16:9. A gloved practitioner's hand holds a slim cordless microneedling pen — champagne-gold body, rose-gold grip ring, clear needle cartridge at the tip — just above a woman's cheek; macro view of skin texture with faint dots of temporary micro-channels catching warm light. The woman's face is in soft focus, eyes closed, relaxed. Environment: dark treatment room in black and deep bronze tones, a thin warm gold edge light along the jawline. Camera: 100 mm macro, f/2.8, focus on the pen tip and the skin, the image occupies the left two-thirds and the right third falls to near-black for text. Mood: precise, clinical, luxurious. No overlay text, no logos.</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>Start: block-1 skin macro, pen gone. An amber vial enters from the right and tilts; one golden drop falls in slow motion onto the skin. The camera follows the drop down into the surface as it swells into a translucent golden sphere drifting in dark liquid, particles glowing inside. End: block-2 vesicle frame, sphere centre-right, vial soft on the left. 5 s, continuous tracking shot, no cuts.</t>
+          <t>Start: block-1 skin macro, pen gone. An amber vial with a white cap enters from the right and tilts; one golden drop falls in slow motion onto the skin. The camera follows the drop down into the surface as it swells into a translucent golden sphere drifting in dark liquid, particles glowing inside. End: block-2 vesicle frame, sphere centre-right, vial soft on the left. 5 s, continuous tracking shot, no cuts.</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
@@ -50685,7 +50685,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five sessions in one box, visible from the first treatment.</t>
+          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five ampoules and five gel-mask sachets in one box, hydration and radiance visible from the first treatment.</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
@@ -50728,7 +50728,7 @@
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>Photoreal macro, 16:9. An open amber glass vial lying on black slate on the left, a single golden drop suspended at its mouth; centre-right an enlarged translucent golden sphere (an engineered vesicle) floating in dark liquid, its shell catching light, soft strands and particles glowing inside it. Lighting: dark background (#0E0C0A), warm gold backlight (#E8C87E) through the sphere, cool highlights on the glass. Camera: 100 mm macro, f/4, sphere sharp, vial slightly soft. Scientific but warm. No overlay text, no logos, no labels.</t>
+          <t>Photoreal macro, 16:9. An open amber glass vial with its white cap beside it, lying on black slate on the left, a single golden drop suspended at its mouth; centre-right an enlarged translucent golden sphere (an engineered vesicle) floating in dark liquid, its shell catching light, soft strands and particles glowing inside it. Lighting: dark background (#0E0C0A), warm gold backlight (#E8C87E) through the sphere, cool highlights on the glass. Camera: 100 mm macro, f/4, sphere sharp, vial slightly soft. Scientific but warm. No overlay text, no logos, no labels.</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
@@ -50760,7 +50760,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five sessions in one box, visible from the first treatment.</t>
+          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five ampoules and five gel-mask sachets in one box, hydration and radiance visible from the first treatment.</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
@@ -50788,7 +50788,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Hydration &amp; radiance · Texture &amp; density · Firming &amp; elasticity · Even tone</t>
+          <t>Hydration &amp; radiance · Structure &amp; density · Firming &amp; elasticity · Even tone</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -50803,12 +50803,12 @@
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic portrait, 16:9. A woman in her forties sits in a treatment chair facing the camera as if looking into a mirror, skin slightly flushed and dewy after microneedling; a practitioner's gloved hands press a clear golden gel from a gold foil sachet onto her cheek. Her eyes meet the lens, calm. Environment: dark clinic room with black walls, a warm gold key light from the front-left and a soft gold rim; a hint of the gold carton on a shelf behind, out of focus. Camera: 85 mm, f/2, eye level, the woman in the left two-thirds, the right third darker for text. No overlay text, no logos.</t>
+          <t>Photoreal cinematic portrait, 16:9. A woman in her forties sits in a treatment chair facing the camera as if looking into a mirror, skin slightly flushed and dewy after microneedling; a practitioner's gloved hands press a clear golden gel from a flat gold-foil sachet onto her cheek. Her eyes meet the lens, calm. Environment: dark clinic room with black walls, a warm gold key light from the front-left and a soft gold rim; a hint of the tall gold carton on a shelf behind, out of focus. Camera: 85 mm, f/2, eye level, the woman in the left two-thirds, the right third darker for text. No overlay text, no logos.</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>Start: block-3 portrait. She closes her eyes; the camera tilts down past her shoulder to the treatment trolley and continues to a straight-overhead view; items slide into one row: pen, vial, sachet, folded mask on a teal card, sunscreen. A thin gold line draws from left to right beneath them. End: block-4 flat lay. 4 s, tilt-down to overhead, objects glide into place.</t>
+          <t>Start: block-3 portrait. She closes her eyes; the camera tilts down past her shoulder to the treatment trolley and continues to a straight-overhead view; items slide into one row: champagne-gold pen, amber vial, gold sachet, folded pale-blue mask in front of a small teal carton, plain white sunscreen tube. A thin gold line draws from left to right beneath them. End: block-4 flat lay. 4 s, tilt-down to overhead, objects glide into place.</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr">
@@ -50835,7 +50835,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five sessions in one box, visible from the first treatment.</t>
+          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five ampoules and five gel-mask sachets in one box, hydration and radiance visible from the first treatment.</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
@@ -50878,12 +50878,12 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Photoreal top-down flat lay, 16:9. On matte black slate, left to right: a slim cordless microneedling pen, an amber glass vial with a white cap, a gold foil sachet, a folded translucent pale-blue bio-cellulose sheet mask on a teal card, and a small white sunscreen tube. Items in one straight row with generous black space between them for step numbers. Lighting: a thin warm gold rim light from the top, soft fill, long soft shadows. Camera: directly overhead, 50 mm, f/8, everything sharp. No overlay text, no logos; pack faces clean.</t>
+          <t>Photoreal top-down flat lay, 16:9. On matte black slate, left to right: a slim cordless microneedling pen with a champagne-gold body, rose-gold grip ring and clear needle cartridge; an amber glass vial with a white cap; a flat gold-foil sachet; a folded translucent pale-blue bio-cellulose sheet mask lying in front of a small matte teal carton; and a plain white unbranded sunscreen tube. Items in one straight row with generous black space between them for step numbers. Lighting: a thin warm gold rim light from the top, soft fill, long soft shadows. Camera: directly overhead, 50 mm, f/8, everything sharp. No overlay text, no logos; pack faces clean.</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>Start: block-4 flat lay. Items lift and slide left into the tall gold carton, which rotates up from flat to standing in three-quarter view, lid flap opening; from inside, five vials and five sachets slide out onto the lacquer in two neat rows. End: block-5 kit shot. 5 s, camera rises from overhead to 20° above eye level.</t>
+          <t>Start: block-4 flat lay. Pen, mask, teal carton and sunscreen slide off-frame left; the tall gold carton glides in and rises from lying flat to standing in three-quarter view as the camera lifts from overhead to 20° above eye level; five amber vials and five gold sachets glide in from the right and settle in two neat rows on the lacquer beside the closed carton. End: block-5 kit shot. 5 s, continuous camera lift.</t>
         </is>
       </c>
       <c r="O6" s="5" t="inlineStr">
@@ -50910,7 +50910,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five sessions in one box, visible from the first treatment.</t>
+          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five ampoules and five gel-mask sachets in one box, hydration and radiance visible from the first treatment.</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
@@ -50933,7 +50933,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Five 5 ml serum ampoules and five 5 ml gel-mask sachets: one course of four treatments, then maintenance every six months.</t>
+          <t>Five 5 ml serum ampoules and five 5 ml gel-mask sachets. Recommended course: at least four treatments; maintenance every six months.</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -50948,17 +50948,17 @@
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>Split 1/2–1/2. Left: the open carton with the 5 + 5 items laid out (real packshot composited for the carton). Right: four big numbers that count up on scroll (5 · 5 ml · 4 · 2 wk) with their labels; a small line 'Face · Neck · Décolleté · Hands'. Gold hairline frame.</t>
+          <t>Split 1/2–1/2. Left: the closed carton in three-quarter view with the 5 + 5 items laid out in two rows beside it (real packshot composited for the carton; the catalogue shows no box interior, so the lid stays closed). Right: four big numbers that count up on scroll (5 · 5 ml · 4 · 2 wk) with their labels; a small line 'Face · Neck · Décolleté · Hands'. Gold hairline frame.</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>Photoreal product shot, 16:9. The tall gold-foil carton with black top and bottom bands, lid flap open, standing in three-quarter view on the left; next to it on black lacquer, neatly in two rows: five amber glass vials with white caps and five flat gold foil sachets. Lighting: warm gold key from the upper right, black background (#0E0C0A), soft gold glow behind the carton only, crisp reflections in the surface. Camera: 70 mm, slightly above eye level, f/5.6, all items sharp, right third empty for numbers. No overlay text, no logos; pack faces clean.</t>
+          <t>Photoreal product shot, 16:9. The tall mirror-gold carton with thin black top and bottom bands, closed, standing in three-quarter view on the left; beside it on black lacquer, neatly in two rows: five amber glass vials with white caps and five flat gold-foil sachets. Lighting: warm gold key from the upper right, black background (#0E0C0A), soft gold glow behind the carton only, crisp reflections in the surface. Camera: 70 mm, slightly above eye level, f/5.6, all items sharp, right third empty for numbers. No overlay text, no logos; pack faces clean.</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>Start: block-5 open carton with items. The lid closes, the items glide back to the hero arrangement (vials and sachet in front), the carton turns to face us and drifts to the right third; the gold glow fades up behind it and a hairline reflection draws across the surface. End: block-6 closing hero. 3 s, gentle dolly-out, light rises.</t>
+          <t>Start: block-5 kit shot. Four sachets slide behind the carton; the five vials close ranks and one sachet settles beside them, re-forming the hero arrangement; the carton turns to face us and drifts to the right third; the gold glow fades up behind it and a hairline reflection draws across the surface. End: block-6 closing hero. 3 s, gentle dolly-out, light rises.</t>
         </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
@@ -50985,7 +50985,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five sessions in one box, visible from the first treatment.</t>
+          <t>V-TECH turns the microneedling you already do into a dermal-regeneration course: synthetic-exosome serum plus a no-rinse gel mask, five ampoules and five gel-mask sachets in one box, hydration and radiance visible from the first treatment.</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
@@ -51028,7 +51028,7 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic hero, 16:9, closing frame. The tall mirror-gold carton with black bands stands on the right third on black lacquer, five amber vials and the gold sachet in front, the set lit by a warm gold glow (#D4A853) behind the carton and a thin gold hairline reflection on the surface; the left two-thirds pure near-black for the offer and buttons. Camera: 85 mm, eye level, f/4. Calm, premium, final. No overlay text, no logos; pack faces clean.</t>
+          <t>Photoreal cinematic hero, 16:9, closing frame. The tall mirror-gold carton with thin black top and bottom bands stands on the right third on black lacquer, five amber vials with white caps and the flat gold-foil sachet in front, the set lit by a warm gold glow (#D4A853) behind the carton and a thin gold hairline reflection on the surface; the left two-thirds pure near-black for the offer and buttons. Camera: 85 mm, eye level, f/4. Calm, premium, final. No overlay text, no logos; pack faces clean.</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
@@ -51108,7 +51108,7 @@
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>Start: block-0 hero (black box right, ampoules in front). The camera slides along the gold lettering and up past the ampoule necks into the black; a circular scope light opens in the dark and reveals a ×50 scalp view: follicle openings, thin hairs. End: block-1 trichoscope macro. 4 s, lateral dolly then push-in, black to scope circle.</t>
+          <t>Start: block-0 hero (black box right, ampoules in front). The camera slides along the box face and up past the ampoule necks into the black; a circular scope light opens in the dark and reveals a ×50 scalp view: follicle openings, thin hairs. End: block-1 trichoscope macro. 4 s, lateral dolly then push-in, black to scope circle.</t>
         </is>
       </c>
       <c r="O9" s="5" t="inlineStr">
@@ -51253,7 +51253,7 @@
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>Photoreal macro, 16:9. A clear glass ampoule with its neck snapped open, tilted, a single clear drop falling from it on the left; centre-right the drop enlarged into a translucent sphere (an engineered vesicle) with glowing strands and particles inside, warm gold (#C9A24A) backlight on matte black (#111111). Camera: 100 mm macro, f/4, sphere sharp, ampoule slightly soft. No overlay text, no logos, no labels.</t>
+          <t>Photoreal macro, 16:9. A clear glass snap-neck ampoule with its neck snapped open, tilted, a single clear drop falling from it on the left; centre-right the drop enlarged into a translucent sphere (an engineered vesicle) with glowing strands and particles inside, warm gold (#C9A24A) backlight on matte black (#111111). Camera: 100 mm macro, f/4, sphere sharp, ampoule slightly soft. No overlay text, no logos, no labels.</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
@@ -51323,17 +51323,17 @@
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>Full-bleed mirror scene: the client faces the camera, the practitioner behind her applying the ampoule along the parting; a faint screen glow at the right edge (the MITOSCAN, planted for the next transition). Text in the right 1/3 over a dark gradient; the four labels appear as gold pins on the scalp line, crown, temple and parting. No before/after — the catalogue has no case images (see notes).</t>
+          <t>Full-bleed mirror scene: the client faces the camera, the practitioner behind her applying the ampoule along the parting; a faint glow from a white tablet screen at the right edge (the MITOSCAN, planted for the next transition). Text in the right 1/3 over a dark gradient; the four labels appear as gold pins on the scalp line, crown, temple and parting. No before/after — the catalogue has no case images (see notes).</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic portrait, 16:9. A woman in her thirties with fine, thinning hair sits facing the camera as if into a mirror; behind her a practitioner dressed in black parts her hair and applies a clear serum from a glass ampoule along the parting with gloved fingers. Her eyes meet the lens, hopeful and calm. Environment: dark trichology room with matte black walls, a warm gold key light from the front-left, a faint cool glow from a screen at the right edge. Camera: 85 mm, f/2, eye level, subject in the left two-thirds, right third dark for text. No overlay text, no logos.</t>
+          <t>Photoreal cinematic portrait, 16:9. A woman in her thirties with fine, thinning hair sits facing the camera as if into a mirror; behind her a practitioner dressed in black parts her hair and applies a clear serum from a glass snap-neck ampoule along the parting with gloved fingers. Her eyes meet the lens, hopeful and calm. Environment: dark trichology room with matte black walls, a warm gold key light from the front-left, a faint cool glow from a white tablet screen on a stand at the right edge. Camera: 85 mm, f/2, eye level, subject in the left two-thirds, right third dark for text. No overlay text, no logos.</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>Start: block-3 portrait. The small screen glow at the right edge grows and swings into frame: a scalp camera's screen showing the scope circle; the camera pans along the counter past the microneedling pen and the ampoule to the spray bottle; a gold line draws beneath them. End: block-4 counter scene. 4 s, pan left to right.</t>
+          <t>Start: block-3 portrait. The screen glow at the right edge grows and swings into frame: a white tablet on a white stand showing the scope circle, a corded white handheld scope resting in front of it; the camera pans along the counter past the champagne-gold microneedling pen and the standing ampoule to a small clear glass spray bottle with a tall gold cap; a gold line draws beneath them. End: block-4 counter scene. 4 s, pan left to right.</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
@@ -51398,17 +51398,17 @@
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>Full-width counter scene as background with a three-step strip plus a fourth 'at home' card; the gold line draws on scroll; each object lights up as its step is reached; the MITOSCAN screen in step 1 plays a 3 s loop of the scope circle. Small device cards (MITOPEN, MITOSCAN) with 'View' links under the strip.</t>
+          <t>Full-width counter scene as background with a three-step strip plus a fourth 'at home' card; the gold line draws on scroll; each object lights up as its step is reached; the MITOSCAN tablet screen in step 1 plays a 3 s loop of the scope circle. Small device cards (MITOPEN, MITOSCAN) with 'View' links under the strip.</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>Photoreal counter scene, 16:9. On a black satin counter, left to right with space between: a handheld scalp camera with a small screen showing an abstract magnified scalp circle, a slim cordless microneedling pen, a clear glass ampoule standing in a small holder, and a small spray bottle at the far right. Lighting: thin warm gold rim light from above, soft fill, matte black background (#111111). Camera: 50 mm, slightly above eye level, f/8, all items sharp, the row centred with margins. No overlay text, no logos, screen content abstract, pack faces clean.</t>
+          <t>Photoreal counter scene, 16:9. On a black satin counter, left to right with space between: a white tablet-style screen on a white stand with a silver cylindrical base, the screen showing an abstract magnified scalp circle, with a corded white handheld scope camera resting in front of it; a slim cordless microneedling pen with a champagne-gold body, rose-gold grip ring and clear needle cartridge; a clear glass snap-neck ampoule standing in a small holder; and a small clear glass spray bottle with a tall gold cap at the far right. Lighting: thin warm gold rim light from above, soft fill, matte black background (#111111). Camera: 50 mm, slightly above eye level, f/8, all items sharp, the row centred with margins. No overlay text, no logos, screen content abstract, pack faces clean.</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>Start: block-4 counter. The devices slide out of frame, the ampoule glides left into the black box as its lid lifts; five ampoules stand up in the tray inside, one lies down in front. End: block-5 open box. 4 s, orbit 30° around the box.</t>
+          <t>Start: block-4 counter. Tablet, scope, pen and spray slide out of frame; the matte black box glides in from the right and settles in three-quarter view behind the standing ampoule; four more ampoules rise one by one beside it into a row, and the last tips gently over to lie in front. End: block-5 kit shot. 4 s, orbit 30° around the box.</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
@@ -51473,17 +51473,17 @@
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>Split 1/2–1/2. Left: the open box with ampoules in the tray (real packshot composited for the box). Right: four large numbers counting up on scroll with labels; a quiet caption 'Designed for men and women · Before / after hair transplant'. Gold hairline frame.</t>
+          <t>Split 1/2–1/2. Left: the closed box in three-quarter view with the five ampoules in a row before it, one lying down (real packshot composited for the box; the catalogue shows no box interior, so no open lid or tray). Right: four large numbers counting up on scroll with labels; a quiet caption 'Designed for men and women · Before / after hair transplant'. Gold hairline frame.</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Photoreal product shot, 16:9. The matte black landscape carton, lid lifted, in three-quarter view on the left, revealing five clear glass ampoules standing in a black tray inside; one ampoule taken out and lying in front. Lighting: warm gold key from the upper right, cool highlight on the glass necks, matte black background, a soft gold glow behind the box only. Camera: 70 mm, f/5.6, right third empty for numbers. No overlay text, no logos; pack faces clean.</t>
+          <t>Photoreal product shot, 16:9. The matte black landscape carton, closed, in three-quarter view on the left; in front of it five clear glass snap-neck ampoules with colourless liquid, four standing in a row and one lying on its side in front. Lighting: warm gold key from the upper right, cool highlight on the glass necks, matte black background, a soft gold glow behind the box only. Camera: 70 mm, f/5.6, right third empty for numbers. No overlay text, no logos; pack faces clean.</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>Start: block-5 open box. The lid closes; the ampoules line up in front; the box turns to face us and settles on the right third; a warm gold glow rises behind it and a reflection line draws. End: block-6 closing hero. 3 s, dolly-out.</t>
+          <t>Start: block-5 kit shot. The lying ampoule rights itself; the row closes ranks in front; the box turns to face us and settles on the right third; a warm gold glow rises behind it and a reflection line draws. End: block-6 closing hero. 3 s, dolly-out.</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -51553,7 +51553,7 @@
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic closing hero, 16:9. The matte black landscape carton on the right third on black satin, five clear ampoules lined up in front, a warm gold glow (#C9A24A) behind the box and a thin gold reflection line on the surface; the left two-thirds matte black for the offer and buttons. Camera: 85 mm, eye level, f/4. Quiet, premium, final. No overlay text, no logos; pack faces clean.</t>
+          <t>Photoreal cinematic closing hero, 16:9. The matte black landscape carton on the right third on black satin, five clear snap-neck ampoules lined up in front, a warm gold glow (#C9A24A) behind the box and a thin gold reflection line on the surface; the left two-thirds matte black for the offer and buttons. Camera: 85 mm, eye level, f/4. Quiet, premium, final. No overlay text, no logos; pack faces clean.</t>
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr">
@@ -52148,17 +52148,17 @@
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>Full-bleed black. Left 5/12: eyebrow 'HOME CARE · SYNTHETIC EXOSOME LINE', title, line, four chips, ghost CTA. Right 7/12: the catalogue packshot of the mirror-gold sphere jar, large, floating just above a dark reflective surface; the black/gold cube box 30% faded behind-left. One warm gold light sweep crosses the sphere on load (1.2 s). Logo reserved top-left.</t>
+          <t>Full-bleed black. Left 5/12: eyebrow 'HOME CARE · SYNTHETIC EXOSOME LINE', title, line, four chips, ghost CTA. Right 7/12: the catalogue packshot of the mirror-gold sphere jar, large, floating just above a dark reflective surface; the black cube box (mirror-gold front face, black diagonal wedge at the left, black top) 30% faded behind-left. One warm gold light sweep crosses the sphere on load (1.2 s). Logo reserved top-left.</t>
         </is>
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>Background plate for compositing: a near-black studio tabletop with a faint mirror reflection, deep charcoal-bronze gradient rising to pure black at the top, one warm gold light sweep entering from the upper right, soft volumetric haze, very subtle gold dust suspended in the air, the right third kept empty for a mirror-polished gold sphere jar (two hemispheres meeting at a thin equator seam) and a matte-black cube box with a mirror-gold diagonal panel, photoreal cinematic product photography, 85 mm lens, f/4, low camera at jar height, 16:9, no text, no captions, no logos.</t>
+          <t>Background plate for compositing: a near-black studio tabletop with a faint mirror reflection, deep charcoal-bronze gradient rising to pure black at the top, one warm gold light sweep entering from the upper right, soft volumetric haze, very subtle gold dust suspended in the air, the right third kept empty for a mirror-polished gold sphere jar with a thin seam just below its equator and a black cube box whose front face is mirror-gold foil with a black diagonal wedge at the left edge, photoreal cinematic product photography, 85 mm lens, f/4, low camera at jar height, 16:9, no text, no captions, no logos.</t>
         </is>
       </c>
       <c r="N23" s="5" t="inlineStr">
         <is>
-          <t>Start frame: the gold sphere at rest on the right, reflection beneath. Camera orbits 30° left while the sphere turns on its axis; the equator seam catches a glint and a hairline of light opens along it. End frame: the upper hemisphere has lifted 2 cm, a sliver of translucent pale-gold gel visible in the gap, the sphere drifted to centre frame, background warmed to bronze. 4 s, scroll-scrubbed.</t>
+          <t>Start frame: the gold sphere at rest on the right, reflection beneath. Camera orbits 30° left while the sphere turns on its axis; the seam catches a glint and a hairline of light opens along it. End frame: the upper hemisphere has lifted 2 cm, a sliver of translucent gel visible in the gap, the sphere drifted to centre frame, background warmed to bronze. 4 s, scroll-scrubbed.</t>
         </is>
       </c>
       <c r="O23" s="5" t="inlineStr">
@@ -52223,7 +52223,7 @@
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>Half-open sphere at centre-left, now 40% height, lid hovering. Right half: a soft-focus low-key portrait of a woman after a clinic visit, one gold edge light on the cheek, eyes to camera — a mood image, not a skin claim. Copy over the dark left third; chips fade in one by one on scroll.</t>
+          <t>Half-open sphere at centre-left, now 40% height, upper hemisphere hovering. Right half: a soft-focus low-key portrait of a woman after a clinic visit, one gold edge light on the cheek, eyes to camera — a mood image, not a skin claim. Copy over the dark left third; chips fade in one by one on scroll.</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
@@ -52233,7 +52233,7 @@
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>Start frame: half-open sphere, portrait soft behind. The portrait dims to black; the camera pushes into the gap between the hemispheres as the upper half floats up and out of frame. End frame: macro of the gel surface filling the screen — translucent pale-gold gel with a glossy meniscus, tiny suspended gold flecks and faint spherical vesicle shapes under the surface, one slow ripple. 5 s, scroll-scrubbed.</t>
+          <t>Start frame: half-open sphere, portrait soft behind. The portrait dims to black; the camera pushes into the gap between the hemispheres as the upper half floats up and out of frame. End frame: macro of the gel surface filling the screen — translucent gel with a glossy meniscus, faint spherical droplets under the surface catching warm gold reflections, one slow ripple. 5 s, scroll-scrubbed.</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr">
@@ -52283,7 +52283,7 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Five actives in one gel: synthetic exosomes, PDRN, biomimetic peptides with gold and copper, hyaluronic acid, snail-derived polysaccharides.</t>
+          <t>Five actives: synthetic exosomes, PDRN, biomimetic peptides with gold and copper, hyaluronic acid, snail-derived polysaccharides.</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
@@ -52293,7 +52293,7 @@
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>none; micro-interaction: hover/tap a chip and the matching particle in the macro lights up</t>
+          <t>none; micro-interaction: hover/tap a chip and the matching droplet in the macro lights up</t>
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr">
@@ -52303,7 +52303,7 @@
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>Extreme macro of a translucent pale-gold cosmetic gel surface, glossy meniscus, tiny suspended gold flecks and faint spherical vesicle-like droplets just below the surface, one gentle ripple, lit from behind with warm gold rim light against black, deep black vignette on the left third, scientific-yet-luxurious mood for a black-and-gold page, 100 mm macro, f/5.6, photoreal, cinematic, 16:9, no text, no diagrams, no logos.</t>
+          <t>Extreme macro of a translucent cosmetic gel surface, glossy meniscus, faint spherical vesicle-like droplets just below the surface catching warm gold reflections, one gentle ripple, lit from behind with warm gold rim light against black, deep black vignette on the left third, scientific-yet-luxurious mood for a black-and-gold page, 100 mm macro, f/5.6, photoreal, cinematic, 16:9, no text, no diagrams, no logos.</t>
         </is>
       </c>
       <c r="N25" s="5" t="inlineStr">
@@ -52373,7 +52373,7 @@
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>Mirror scene: she faces the camera as if it were her mirror and massages the gel into her cheek with upward strokes — the screen is the mirror. She fills the left two thirds, copy on the right; the four chips rise along her jawline with each stroke. No before/after: the catalogue has none for this product.</t>
+          <t>Mirror scene: she faces the camera as if it were her mirror and massages the gel into her cheek until absorbed — the screen is the mirror. She fills the left two thirds, copy on the right; the four chips rise along her jawline with each stroke. No before/after: the catalogue has none for this product.</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
@@ -52448,7 +52448,7 @@
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>Closed sphere centred on a shelf in morning light; three numbered step cards in a horizontal timeline beneath it, each lighting as it enters the viewport; the 'works with' row shows three small catalogue packshots (V-TECH, EXO-NAD, BIOSPICULE™ range) with names.</t>
+          <t>Closed sphere centred on a shelf in morning light; three numbered step cards in a horizontal timeline beneath it, each lighting as it enters the viewport; the 'works with' row shows three small catalogue packshots (V-TECH SYSTEM, EXO-NAD, BIOSPICULE™ range) with names.</t>
         </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
@@ -52458,7 +52458,7 @@
       </c>
       <c r="N27" s="5" t="inlineStr">
         <is>
-          <t>Start frame: closed sphere on the shelf. The shelf dissolves; the matte-black cube box slides in from the left, its mirror-gold diagonal panel catching light; the lid lifts and the sphere lowers itself into the box's cradle. End frame: open box with the sphere nested inside, 3/4 top angle, lid floating above. 4 s.</t>
+          <t>Start frame: closed sphere on the shelf. The shelf dissolves to black; the black cube box slides in from the left, its mirror-gold front face catching light; the sphere rolls once and settles in front of the box. End frame: box and sphere together on a black reflective surface, 3/4 top angle. 4 s.</t>
         </is>
       </c>
       <c r="O27" s="5" t="inlineStr">
@@ -52523,17 +52523,17 @@
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>Open box with the sphere nested inside, 3/4 top view, right side. Left: four stat tiles in a 2×2 grid (the spec stats), number + one-word label, counting up on entry. Indication chips (normal–combination, dry, tired, fine lines, after treatments) as a quiet row underneath.</t>
+          <t>Closed box with the sphere standing in front of it, 3/4 top view, right side. Left: four stat tiles in a 2×2 grid (the spec stats), number + one-word label, counting up on entry. Indication chips (normal–combination, dry, tired, fine lines, after treatments) as a quiet row underneath. The box interior is not shown in the catalogue, so the box stays closed.</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>Top-down 3/4 view of an open matte-black cube gift box with a mirror-gold diagonal foil panel, lid floating just above, a mirror-polished gold sphere jar nested inside on a black satin cradle, on a black reflective surface, warm gold key light from the upper left, deep black surroundings, luxury unboxing mood for a black-and-gold page, 50 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Top-down 3/4 view of a black cube box with a mirror-gold foil front face and a black diagonal wedge at its left edge, a mirror-polished gold sphere jar standing in front of it, both on a black reflective surface, warm gold key light from the upper left, deep black surroundings, luxury still-life mood for a black-and-gold page, 50 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos.</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>Start frame: open box with sphere. The lid lowers and closes; the camera drops to table level and pulls back; the sphere rises out and lands beside the closed box. End frame: the block-0 composition again — closed box and sphere side by side on the right, now in full warm gold light, the left half open for the offer. 3 s.</t>
+          <t>Start frame: box and sphere, 3/4 top angle. The camera drops to table level and pulls back while the gold light widens. End frame: the block-0 composition again — closed box and sphere side by side on the right, now in full warm gold light, the left half open for the offer. 3 s.</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr">
@@ -52588,7 +52588,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Partner clinics · Training &amp; protocols · Synthetic exosome line · Contact</t>
+          <t>Partner clinics · Ask your specialist · Synthetic exosome line · Contact</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
@@ -52603,7 +52603,7 @@
       </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>Mirror-polished gold sphere jar standing beside its matte-black cube box with a mirror-gold diagonal panel, both on a black reflective surface, generous warm gold light from the upper right, soft gold haze, deep black surroundings, left half of the frame empty and dark for copy, premium closing shot for a black-and-gold page, 85 mm, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Mirror-polished gold sphere jar standing beside a black cube box whose front face is mirror-gold foil with a black diagonal wedge at the left edge, both on a black reflective surface, generous warm gold light from the upper right, soft gold haze, deep black surroundings, left half of the frame empty and dark for copy, premium closing shot for a black-and-gold page, 85 mm, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
         </is>
       </c>
       <c r="N29" s="5" t="inlineStr">
@@ -52673,17 +52673,17 @@
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>Full-bleed black. Left: eyebrow 'HOME CARE · SCALP', title, line, chips, ghost CTA. Right: the slim clear 15 ml spray bottle standing tall, its brushed-silver cap lit by a cool rim light, the tall matte-black carton behind-right at 40%; a frozen fine mist hangs above the nozzle.</t>
+          <t>Full-bleed black. Left: eyebrow 'HOME CARE · SCALP', title, line, chips, ghost CTA. Right: the slim frosted-glass 15 ml spray bottle standing tall, its tall polished-gold cap lit by a warm rim light, the tall matte-black carton behind-right at 40%; a frozen fine mist hangs above the cap.</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>Background plate for compositing: a near-black studio with a cool silver-white rim light from the upper right, a barely visible reflective black surface, a frozen cloud of fine mist droplets suspended in the light at the right third of the frame (where a slim clear-glass 15 ml spray bottle with a tall brushed-silver cap and its tall matte-black carton will be composited), very faint haze, monochrome black-and-white grade with a silver tint, 85 mm, f/4, low camera, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Background plate for compositing: a near-black studio with a warm gold rim light from the upper right, a barely visible reflective black surface, a frozen cloud of fine mist droplets suspended in the light at the right third of the frame (where a slim frosted-glass 15 ml spray bottle with a tall polished-gold cap and its tall matte-black rectangular carton will be composited), very faint haze, black-and-gold grade with frosted-white highlights, 85 mm, f/4, low camera, photoreal, cinematic, 16:9, no text, no logos.</t>
         </is>
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>Start frame: bottle at rest, mist frozen. The silver cap depresses; a fine mist blooms in slow motion in the rim light and drifts left across the frame; the camera follows the mist. End frame: the mist dissolves into a top-down close-up of dark hair parted to expose the scalp, lit by the same cool light; the bottle now small at the lower right. 4 s.</t>
+          <t>Start frame: bottle at rest, mist frozen. The gold cap lifts away and the pump head presses; a fine mist blooms in slow motion in the gold rim light and drifts left across the frame; the camera follows the mist. End frame: the mist dissolves into a top-down close-up of dark hair parted to expose the scalp, lit by the same warm light; the bottle now small at the lower right. 4 s.</t>
         </is>
       </c>
       <c r="O30" s="5" t="inlineStr">
@@ -52733,7 +52733,7 @@
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>EXOSIGNAL HAIR works in the clinic. Hair thinning, brittle hair and scalp imbalance need support on the days in between.</t>
+          <t>EXOSIGNAL HAIR is the clinic treatment. Hair thinning, brittle hair and scalp imbalance need support on the days in between.</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
@@ -52748,22 +52748,22 @@
       </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>Top-down close-up of a hair parting as the background (right two thirds); copy on the dark left third. A thin silver strip of 14 day-ticks draws under the line: only the first and last tick glow (clinic visits), the middle ticks stay empty — a picture of 'the days in between', no numbers claimed.</t>
+          <t>Top-down close-up of a hair parting as the background (right two thirds); copy on the dark left third. A thin gold line draws under the copy between two glowing end points — two clinic visits — with no ticks and no numbers: the interval is the clinic's protocol, not a claim.</t>
         </is>
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>Top-down close-up of a person's dark hair parted with a comb to expose a clean line of scalp, cool silver-white directional light from the upper right, deep black surroundings, monochrome black-and-white grade with silver tint, clinical and intimate, left third of the frame dark and empty for copy, 100 mm macro, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Top-down close-up of a person's dark hair parted with a comb to expose a clean line of scalp, warm gold directional light from the upper right, deep black surroundings, black-and-gold grade, clinical and intimate, left third of the frame dark and empty for copy, 100 mm macro, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
         </is>
       </c>
       <c r="N31" s="5" t="inlineStr">
         <is>
-          <t>Start frame: hair parting from above. The bottle rises from the lower right into frame and sprays once toward the parting; the camera dives with the mist down to the scalp. End frame: extreme macro of droplets settling between hair strands on the scalp, catching silver light. 4 s.</t>
+          <t>Start frame: hair parting from above. The bottle rises from the lower right into frame and sprays once toward the parting; the camera dives with the mist down to the scalp. End frame: extreme macro of droplets settling between hair strands on the scalp, catching warm gold light. 4 s.</t>
         </is>
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>Parting image full-width behind the copy at 50% opacity; the 14-day strip becomes a 7-day strip to fit 390 px.</t>
+          <t>Parting image full-width behind the copy at 50% opacity; the two-point visit line shortens to fit 390 px.</t>
         </is>
       </c>
     </row>
@@ -52828,12 +52828,12 @@
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>Extreme macro of fine clear droplets settling on scalp skin between dark hair strands, droplets catching cool silver-white light, shallow depth of field, deep black background, monochrome grade with silver tint, clinical-scientific mood for a black-white-silver page, 100 mm macro, f/4, photoreal, cinematic, 16:9, no text, no diagrams, no logos.</t>
+          <t>Extreme macro of fine clear droplets settling on scalp skin between dark hair strands, droplets catching warm gold rim light, shallow depth of field, deep black background, black-and-gold grade, clinical-scientific mood for a black-and-gold page, 100 mm macro, f/4, photoreal, cinematic, 16:9, no text, no diagrams, no logos.</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>Start frame: droplet macro. The droplets sink into the skin and vanish; the camera pulls back fast out of the hair, rises, and we find ourselves as a bathroom mirror. End frame: medium shot, a woman in her 30s facing the camera, one hand parting her hair, the spray bottle in the other raised to the scalp, cool white bathroom light, the black carton on the shelf. 5 s.</t>
+          <t>Start frame: droplet macro. The droplets sink into the skin and vanish; the camera pulls back fast out of the hair, rises, and we find ourselves as a bathroom mirror. End frame: medium shot, a woman in her 30s facing the camera, one hand parting her hair, the spray bottle in the other raised to the scalp, one warm practical light, the matte-black carton on the shelf. 5 s.</t>
         </is>
       </c>
       <c r="O32" s="5" t="inlineStr">
@@ -52903,12 +52903,12 @@
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>Medium close-up of a woman in her 30s facing the camera as if it were her bathroom mirror, one hand parting her dark hair to expose the scalp, the other holding a slim clear-glass spray bottle with a tall brushed-silver cap at the parting, calm expression, cool white bathroom light, black tiled wall, a tall matte-black carton on the shelf, monochrome black-and-white grade with silver tint, 50 mm, f/2.8, photoreal, cinematic, natural skin and hair, 16:9, no text, no logos.</t>
+          <t>Medium close-up of a woman in her 30s facing the camera as if it were her bathroom mirror, one hand parting her dark hair to expose the scalp, the other holding a slim frosted-glass spray bottle with a tall polished-gold cap at the parting, calm expression, one warm practical light, dark tiled wall, a tall matte-black carton on the shelf, black-and-gold grade, 50 mm, f/2.8, photoreal, cinematic, natural skin and hair, 16:9, no text, no logos.</t>
         </is>
       </c>
       <c r="N33" s="5" t="inlineStr">
         <is>
-          <t>Start frame: fingertips massaging the parting. She lowers her hands and lets the hair fall back; the camera tilts down to her hand placing the bottle on the shelf. End frame: the bottle standing on the shelf beside the carton, 3/4 top-down, cool light, copy space on the left. 3 s.</t>
+          <t>Start frame: fingertips massaging the parting. She lowers her hands and lets the hair fall back; the camera tilts down to her hand placing the bottle on the shelf. End frame: the bottle standing on the shelf beside the carton, 3/4 top-down, warm light, copy space on the left. 3 s.</t>
         </is>
       </c>
       <c r="O33" s="5" t="inlineStr">
@@ -52973,22 +52973,22 @@
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>Bottle on the shelf, centred; three step cards in a horizontal timeline with line icons (comb / mist / fingertips) lighting on entry. 'Works with' shows the EXOSIGNAL HAIR catalogue packshot (black box with ampoules) and a MITOSCAN thumbnail labelled 'tracked with' — the spec lists MITOSCAN as working with the spray.</t>
+          <t>Bottle on the shelf, centred; three step cards in a horizontal timeline with line icons (comb / mist / fingertips) lighting on entry. 'Works with' shows the EXOSIGNAL HAIR catalogue packshot (black box with ampoules).</t>
         </is>
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>A slim clear-glass 15 ml spray bottle with a tall brushed-silver cap standing on a black stone bathroom shelf beside its tall matte-black carton, cool morning window light from the left, soft reflection, black background, calm daily-ritual mood for a black-white-silver page, 50 mm, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>A slim frosted-glass 15 ml spray bottle with a tall polished-gold cap standing on a black stone bathroom shelf beside its tall matte-black rectangular carton, warm morning window light from the left, soft reflection, black background, calm daily-ritual mood for a black-and-gold page, 50 mm, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
         </is>
       </c>
       <c r="N34" s="5" t="inlineStr">
         <is>
-          <t>Start frame: bottle and carton on the shelf. The carton turns to face us and its top flap opens; the bottle lifts and slides down into the carton's cradle; the camera moves to a 3/4 top angle. End frame: open carton with the bottle seated inside, flap raised, on black. 4 s.</t>
+          <t>Start frame: bottle and carton on the shelf. The carton turns to face us and its top flap opens; the bottle lifts and lowers halfway into the carton; the camera moves to a 3/4 top angle. End frame: open carton with the bottle standing half-inside, flap raised, on black. 4 s.</t>
         </is>
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
-          <t>Bottle 40% width centred; steps stack as three rows; 'works with' as a horizontal scroll row.</t>
+          <t>Bottle 40% width centred; steps stack as three rows; 'works with' as a single packshot card.</t>
         </is>
       </c>
     </row>
@@ -53048,17 +53048,17 @@
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>Open carton with the bottle inside, right. Left: 2×2 stat tiles from the spec (15 ml / Daily / No rinsing / Scalp). Indication chips underneath (hair thinning, fine brittle hair, scalp imbalance, hair-loss programmes, between treatments, after a course, after transplantation).</t>
+          <t>Open carton with the bottle half-inside, right. Left: 2×2 stat tiles from the spec (15 ml / Daily / No rinsing / Scalp). Indication chips underneath (hair thinning, fine brittle hair, scalp imbalance, hair-loss programmes, between treatments, after a course, after transplantation).</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr">
         <is>
-          <t>Top-down 3/4 view of a tall matte-black rectangular carton opened at the top, a slim clear-glass spray bottle with a brushed-silver cap seated inside on a black insert, on a black reflective surface, cool silver-white key light from the upper left, deep black surroundings, precise unboxing mood for a black-white-silver page, 50 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Top-down 3/4 view of a tall matte-black rectangular carton opened at the top, a slim frosted-glass spray bottle with a tall polished-gold cap standing half-inside it, on a black reflective surface, warm gold key light from the upper left, deep black surroundings, precise unboxing mood for a black-and-gold page, 50 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos.</t>
         </is>
       </c>
       <c r="N35" s="5" t="inlineStr">
         <is>
-          <t>Start frame: open carton. The flap closes; the bottle rises out and stands beside the carton; the camera drops to table level and pulls back to the block-0 composition, rim light brighter, the copy side empty. 3 s.</t>
+          <t>Start frame: open carton with the bottle half-inside. The bottle rises out and stands beside the carton; the flap closes; the camera drops to table level and pulls back. End frame: the block-0 composition — bottle and carton side by side on the right, gold rim light brighter, the left half empty for the offer. 3 s.</t>
         </is>
       </c>
       <c r="O35" s="5" t="inlineStr">
@@ -53113,27 +53113,27 @@
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>Partner clinics · Hair-loss programmes · After hair transplantation · Training &amp; protocols</t>
+          <t>Partner clinics · Hair-loss programmes · After hair transplantation · Between EXOSIGNAL HAIR treatments</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>Primary: 'Where to buy' (white fill, black text). Secondary: 'Ask a specialist' (ghost) → contact form / WhatsApp. Mobile: sticky bottom bar 'Where to buy'.</t>
+          <t>Primary: 'Where to buy' (gold fill, black text). Secondary: 'Ask a specialist' (ghost) → contact form / WhatsApp. Mobile: sticky bottom bar 'Where to buy'.</t>
         </is>
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>Bottle + carton on the right in full rim light; left: title, line, buttons; related row: EXOSIGNAL HAIR (clinic treatment) and MITOSCAN (diagnostics).</t>
+          <t>Bottle + carton on the right in full rim light; left: title, line, buttons; related row: EXOSIGNAL HAIR (clinic treatment) and MITOSCAN (diagnostics — its spec lists the spray under 'works with').</t>
         </is>
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>A slim clear-glass 15 ml spray bottle with a tall brushed-silver cap standing beside its tall matte-black carton on a black reflective surface, a fine frozen mist above the nozzle, bright cool silver-white rim light from the upper right, deep black surroundings, left half of the frame empty and dark for copy, premium closing shot for a black-white-silver page, 85 mm, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>A slim frosted-glass 15 ml spray bottle with a tall polished-gold cap standing beside its tall matte-black rectangular carton on a black reflective surface, a fine frozen mist above the cap, bright warm gold rim light from the upper right, deep black surroundings, left half of the frame empty and dark for copy, premium closing shot for a black-and-gold page, 85 mm, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>End of page — no next block. Idle loop (6 s): a single mist puff every few seconds dissolving in the rim light; 'back to top' flies the bottle to its block-0 position.</t>
+          <t>End of page — no next block. Idle loop (6 s): a single mist puff every few seconds dissolving in the gold rim light; 'back to top' flies the bottle to its block-0 position.</t>
         </is>
       </c>
       <c r="O36" s="5" t="inlineStr">
@@ -54778,7 +54778,7 @@
       </c>
       <c r="M58" s="5" t="inlineStr">
         <is>
-          <t>Background plate for compositing: a warm champagne-gold brushed-metal studio surface with a soft horizon gradient from pale champagne to deeper sand, one large soft key light from the upper left and a subtle warm rim from the right, faint metallic sheen, the right third kept empty for a slender champagne-gold cordless microneedling pen with a ribbed rose-copper adjustment ring and a clear needle cartridge, precision-instrument mood, 85 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Background plate for compositing: a warm champagne-gold brushed-metal studio surface with a soft horizon gradient from pale champagne to deeper sand, one large soft key light from the upper left and a subtle warm rim from the right, faint metallic sheen, the right third kept empty for a slender champagne-gold cordless microneedling pen with a ribbed rose-copper adjustment ring, a small rose-copper button near the top and a clear needle cartridge at the tip, precision-instrument mood, 85 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos.</t>
         </is>
       </c>
       <c r="N58" s="5" t="inlineStr">
@@ -54858,7 +54858,7 @@
       </c>
       <c r="N59" s="5" t="inlineStr">
         <is>
-          <t>Start frame: triptych of areas. The three images slide apart and dim; the pen's cartridge enters at macro scale from the left; the camera orbits the ring as it turns one more step and the small LED near the top lights. End frame: macro of the clear cartridge with needles extended, the rose-copper ring sharp in the foreground, champagne background. 4 s.</t>
+          <t>Start frame: triptych of areas. The three images slide apart and dim; the pen's cartridge enters at macro scale from the left; the camera orbits the ring as it turns one more step and the small dot above the button catches the light. End frame: macro of the clear cartridge with needles extended, the rose-copper ring sharp in the foreground, champagne background. 4 s.</t>
         </is>
       </c>
       <c r="O59" s="5" t="inlineStr">
@@ -55073,7 +55073,7 @@
       </c>
       <c r="L62" s="5" t="inlineStr">
         <is>
-          <t>Top-down tray: pen centred, three step cards along the bottom lighting in sequence on scroll. 'Works with' shows the catalogue packshots of V-TECH SYSTEM (gold box + ampoules), EXOSIGNAL HAIR (black box + ampoules) and the MICRO BOOST 10% vial; area chips face / neck &amp; décolleté / scalp.</t>
+          <t>Top-down tray: pen centred, three step cards along the bottom lighting in sequence on scroll. 'Works with' shows the catalogue packshots of V-TECH SYSTEM (gold box + ampoules), EXOSIGNAL HAIR (black box + ampoules) and the MICRO BOOST 10% syringe; area chips face / neck &amp; décolleté / scalp.</t>
         </is>
       </c>
       <c r="M62" s="5" t="inlineStr">
@@ -55083,7 +55083,7 @@
       </c>
       <c r="N62" s="5" t="inlineStr">
         <is>
-          <t>Start frame: tray top-down. The tray fades; the pen rises to a 20° diagonal and the camera orbits 180° around it, showing the full barrel, the small rose-copper button and LED near the top, the ring and the cartridge. End frame: pen standing on a brushed-champagne plinth, 3/4 view, four empty slots beside it for stat tiles. 4 s.</t>
+          <t>Start frame: tray top-down. The tray fades; the pen rises to a 20° diagonal and the camera orbits 180° around it, showing the full barrel, the small rose-copper button and the dot above it near the top, the ring and the cartridge. End frame: pen standing on a brushed-champagne plinth, 3/4 view, four empty slots beside it for stat tiles. 4 s.</t>
         </is>
       </c>
       <c r="O62" s="5" t="inlineStr">
@@ -55158,7 +55158,7 @@
       </c>
       <c r="N63" s="5" t="inlineStr">
         <is>
-          <t>Start frame: pen on the plinth. The plinth sinks away; the pen tilts back to its block-0 diagonal and the camera pulls back to the hero framing, key light warmer and brighter, the left half open for the offer. 3 s.</t>
+          <t>Start frame: pen upright on the plinth. The plinth sinks away; the pen tilts back to its 20° diagonal and the camera pulls back. End frame: the block-0 hero framing — pen on the right on the brushed-champagne surface, key light warmer and brighter, the left half empty for the offer. 3 s.</t>
         </is>
       </c>
       <c r="O63" s="5" t="inlineStr">
@@ -55223,7 +55223,7 @@
       </c>
       <c r="L64" s="5" t="inlineStr">
         <is>
-          <t>Pen on the right in hero framing; left: title, line, buttons; related row: V-TECH SYSTEM, EXOSIGNAL HAIR, MITOSCAN.</t>
+          <t>Pen on the right in hero framing; left: title, line, buttons; related row: V-TECH SYSTEM, EXOSIGNAL HAIR, MITOSCAN (its spec lists MITOPEN under 'works with').</t>
         </is>
       </c>
       <c r="M64" s="5" t="inlineStr">
@@ -55233,7 +55233,7 @@
       </c>
       <c r="N64" s="5" t="inlineStr">
         <is>
-          <t>End of page — no next block. Idle loop (6 s): the LED near the top pulses once every few seconds and the ring glints; 'back to top' flies the pen to its block-0 position.</t>
+          <t>End of page — no next block. Idle loop (6 s): the rose-copper ring glints once every few seconds; 'back to top' flies the pen to its block-0 position.</t>
         </is>
       </c>
       <c r="O64" s="5" t="inlineStr">
@@ -55358,7 +55358,7 @@
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>To the naked eye, density, follicle count and hair diameter stay invisible — so goals, expectations and the course rest on impression alone.</t>
+          <t>To the naked eye, density, follicle count and hair diameter stay invisible — so goals and the course rest on impression alone.</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
@@ -55383,7 +55383,7 @@
       </c>
       <c r="N66" s="5" t="inlineStr">
         <is>
-          <t>Start frame: consultation room, probe on the desk. A practitioner's hand picks up the probe and brings its lens toward the camera; the ring light around the lens flares white-blue and fills the frame. End frame: the flare resolves into a full-screen ×50 scalp image (hair shafts, follicle openings); one scroll step later it jumps to ×200 — individual follicles and the scalp surface fill the frame. 5 s.</t>
+          <t>Start frame: consultation room, probe on the desk. A practitioner's hand picks up the probe and brings its lens toward the camera; the probe's lens light flares white-blue and fills the frame. End frame: the flare resolves into a full-screen ×50 scalp image (hair shafts, follicle openings); one scroll step later it jumps to ×200 — individual follicles and the scalp surface fill the frame. 5 s.</t>
         </is>
       </c>
       <c r="O66" s="5" t="inlineStr">
@@ -55658,7 +55658,7 @@
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>1× MITOSCAN — advanced hair &amp; scalp diagnostic system with HD display and handheld scan probe. For professional use only.</t>
+          <t>1× MITOSCAN — advanced hair &amp; scalp diagnostic system: ×50 and ×200 magnification, HD imaging. For professional use only.</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
@@ -55683,7 +55683,7 @@
       </c>
       <c r="N70" s="5" t="inlineStr">
         <is>
-          <t>Start frame: system on a plinth. The plinth sinks away; the camera drops to table level and pulls back to the block-0 hero framing, screen brighter, the left half open for the offer. 3 s.</t>
+          <t>Start frame: system on the plinth, 3/4 view. The plinth sinks away; the camera drops to table level and pulls back. End frame: the block-0 hero framing — monitor, docked probe and base on the right, screen brighter, the left half empty for the offer. 3 s.</t>
         </is>
       </c>
       <c r="O70" s="5" t="inlineStr">
@@ -55808,12 +55808,12 @@
       </c>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>An Israeli company bringing advanced Italian and Korean laboratory technologies to professional skin and scalp care.</t>
+          <t>An Israeli company bringing advanced Italian and South Korean laboratory technologies to professional skin and scalp care.</t>
         </is>
       </c>
       <c r="J72" s="5" t="inlineStr">
         <is>
-          <t>MITO - cellular energy · DERM - the skin · Israel · Italy · Korea · Professional aesthetics</t>
+          <t>MITO - cellular energy · DERM - the skin · Israel · Italy · South Korea · Professional aesthetics</t>
         </is>
       </c>
       <c r="K72" s="5" t="inlineStr">
@@ -55823,12 +55823,12 @@
       </c>
       <c r="L72" s="5" t="inlineStr">
         <is>
-          <t>Full-viewport split 1/2 + 1/2 on the dark gold band #1C1510. Left: eyebrow ABOUT, the wordmark animates in as two halves - MITO slides from the left, DERM from the right, meeting at the centre, then the two labels 'cellular energy' / 'the skin' fade under them. Right: the 'product' = the brand emblem as a physical object: a thick polished-gold medallion standing on a dark lacquered surface, soft glow behind it, slow 6-degree idle rotation; the real logo is composited onto its face. Below the emblem, out of focus, the five portfolio objects (real packshots) hint at what is coming.</t>
+          <t>Full-viewport split 1/2 + 1/2 on the dark gold band #1C1510. Left: eyebrow ABOUT, the wordmark animates in as two halves - MITO slides from the left, DERM from the right, meeting at the centre, then the two labels 'cellular energy' / 'the skin' fade under them. Right: the 'product' = the brand emblem as a physical object: a thick polished-gold medallion standing on a dark lacquered surface, soft glow behind it, slow 6-degree idle rotation; the real logo SVG is composited onto its face. Below the emblem, out of focus, the real packshots (vtech-system.webp, exo-nad.webp, micro-boost-10.webp) hint at what is coming.</t>
         </is>
       </c>
       <c r="M72" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product still, 16:9. A thick round polished-gold medallion with a blank brushed face stands upright on a dark lacquered walnut surface in a dim studio; deep warm bronze-black background #1C1510, soft golden rim light from the upper right, a faint warm glow halo behind the medallion only, gentle reflection on the surface. Out of focus in the lower right, three small glass ampoules and a white syringe cap catch gold highlights. 85 mm lens, f/2.8, shallow depth of field, slight low angle, subject in the right third, empty negative space on the left. No text, no logos, no engravings on the medallion.</t>
+          <t>Photoreal cinematic product still, 16:9. A thick round polished-gold medallion with a blank brushed face stands upright on a dark lacquered walnut surface in a dim studio; deep warm bronze-black background #1C1510, soft golden rim light from the upper right, a faint warm glow halo behind the medallion only, gentle reflection on the surface. Out of focus in the lower right, three small clear glass ampoules and a small syringe catch gold highlights. 85 mm lens, f/2.8, shallow depth of field, slight low angle, subject in the right third, empty negative space on the left. No text, no logos, no engravings on the medallion.</t>
         </is>
       </c>
       <c r="N72" s="5" t="inlineStr">
@@ -55908,7 +55908,7 @@
       </c>
       <c r="N73" s="5" t="inlineStr">
         <is>
-          <t>4 s. Start: the closed carton on the trolley. The lid lifts as the camera cranes up and over; the inside glows warm gold, and five objects rise out of it in sequence and spread into an arc on an ivory studio surface: the V-TECH SYSTEM kit, the EXO-NAD kit, the MICRO BOOST 10% syringe, the MITOPEN pen, the MITOSCAN device. The carton fades away. End: block 2 - the gold medallion at the centre of the arc, the five real packshots around it.</t>
+          <t>4 s. Start: the closed carton on the trolley. The lid lifts as the camera cranes up and over; the inside glows warm gold, and five objects rise out together and spread into an arc on an ivory studio surface: the V-TECH SYSTEM kit, the EXO-NAD kit, the MICRO BOOST 10% syringe, the MITOPEN pen, the MITOSCAN device (real packshots composited). The carton fades away. End: block 2 - the gold medallion at the centre of the arc, the five real packshots around it.</t>
         </is>
       </c>
       <c r="O73" s="5" t="inlineStr">
@@ -55958,7 +55958,7 @@
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>Synthetic exosomes, peptides and PDRN, NAD+ and biomimetic ingredients, BIOSPICULE™ purified spicules, and the MITOPEN and MITOSCAN devices.</t>
+          <t>Synthetic exosomes, peptides and PDRN, NAD+ and biomimetic ingredients, BIOSPICULE™ spicules, and the MITOPEN and MITOSCAN devices.</t>
         </is>
       </c>
       <c r="J74" s="5" t="inlineStr">
@@ -55968,7 +55968,7 @@
       </c>
       <c r="K74" s="5" t="inlineStr">
         <is>
-          <t>Each label is a chip-link to its page (Synthetic exosomes, BIOSPICULE™, MITOPEN, MITOSCAN)</t>
+          <t>Chips link to a page where one exists (Synthetic exosomes, BIOSPICULE™, MITOPEN, MITOSCAN); the peptides chip is static</t>
         </is>
       </c>
       <c r="L74" s="5" t="inlineStr">
@@ -55983,7 +55983,7 @@
       </c>
       <c r="N74" s="5" t="inlineStr">
         <is>
-          <t>4 s. Start: the arc of five products on ivory. The camera dollies right along the arc, past the MITOPEN and through a glass partition; the ivory studio becomes a warm modern clinic. A practitioner in white picks one object from the arc - the V-TECH ampoule - turns toward the camera and raises her eyes to it as to a mirror. End: block 3 full-bleed portrait frozen.</t>
+          <t>4 s. Start: the arc of five products on ivory. The camera dollies right along the arc, past the MITOPEN and through a glass partition; the ivory studio becomes a warm modern clinic. A practitioner in white picks one object from the arc - a V-TECH ampoule - turns toward the camera and raises her eyes to it as to a mirror. End: block 3 full-bleed portrait frozen.</t>
         </is>
       </c>
       <c r="O74" s="5" t="inlineStr">
@@ -56028,7 +56028,7 @@
       </c>
       <c r="H75" s="5" t="inlineStr">
         <is>
-          <t>Your clinic, fully equipped</t>
+          <t>A complete framework for your clinic</t>
         </is>
       </c>
       <c r="I75" s="5" t="inlineStr">
@@ -56048,12 +56048,12 @@
       </c>
       <c r="L75" s="5" t="inlineStr">
         <is>
-          <t>Full-bleed photo, the mirror scene for the brand: the practitioner is the hero. She looks straight into the camera (we are her mirror), the V-TECH ampoule in one hand and a blank protocol card in the other, a client softly blurred in the chair behind. Text 1/3 on the left over a gold-to-transparent gradient; the four labels drop in as she 'reads' them, each pinned to a point on the card. Catalogue has no before/after imagery, so none is shown here.</t>
+          <t>Full-bleed photo, the mirror scene for the brand: the practitioner is the hero. She looks straight into the camera (we are her mirror), a V-TECH ampoule in one hand and a blank protocol card in the other, a client softly blurred in the chair behind. Text 1/3 on the left over a gold-to-transparent gradient; the four labels drop in as she 'reads' them, each pinned to a point on the card. Catalogue has no before/after imagery, so none is shown here.</t>
         </is>
       </c>
       <c r="M75" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic portrait, 16:9. A confident female aesthetic practitioner in her thirties in a white uniform stands in a bright modern clinic and looks directly into the lens as if into a mirror; in her right hand a small clear glass ampoule with an amber serum, in her left a blank white card; behind her, out of focus, a reclining treatment chair with a client and a window with warm afternoon light. Warm ivory and gold palette, skin tones natural, gentle gold rim light on her shoulder. 85 mm lens, f/2, eye level, subject in the right two thirds, soft empty space on the left. No text, no logos, no brand marks on the uniform.</t>
+          <t>Photoreal cinematic portrait, 16:9. A confident female aesthetic practitioner in her thirties in a white uniform stands in a bright modern clinic and looks directly into the lens as if into a mirror; in her right hand a small clear glass ampoule, in her left a blank white card; behind her, out of focus, a reclining treatment chair with a client and a window with warm afternoon light. Warm ivory and gold palette, skin tones natural, gentle gold rim light on her shoulder. 85 mm lens, f/2, eye level, subject in the right two thirds, soft empty space on the left. No text, no logos, no brand marks on the uniform or the ampoule.</t>
         </is>
       </c>
       <c r="N75" s="5" t="inlineStr">
@@ -56123,17 +56123,17 @@
       </c>
       <c r="L76" s="5" t="inlineStr">
         <is>
-          <t>Three step cards on the gold step line that draws on scroll (left to right at 1440, top to bottom on mobile): Knowledge -&gt; Protocols -&gt; Training. Background: top-down photo of the clinic desk from the transition; each card lifts slightly on reveal and shows one sentence from the spec. The fourth label 'Works with' is a quiet caption at the end of the line.</t>
+          <t>Three step cards on the gold step line that draws on scroll (left to right at 1440, top to bottom on mobile): Knowledge -&gt; Protocols -&gt; Training. Background: top-down photo of the clinic desk from the transition; each card lifts slightly on reveal and shows one sentence from the spec steps. The fourth label 'Works with' is a quiet caption at the end of the line.</t>
         </is>
       </c>
       <c r="M76" s="5" t="inlineStr">
         <is>
-          <t>Photoreal top-down (flat-lay) photograph, 16:9. A clean pale-oak clinic desk seen from directly above: an open blank white binder with ring spine, a tablet with a dark blank screen, one clear glass ampoule with amber serum, a steel spatula and a folded white towel, arranged in a loose row from left to right. Soft daylight from the top, warm ivory tones, a faint gold reflection on the ampoule. 35 mm lens, f/8, perfectly perpendicular. No text, no logos, no printed pages.</t>
+          <t>Photoreal top-down (flat-lay) photograph, 16:9. A clean pale-oak clinic desk seen from directly above: an open blank white binder with ring spine, a tablet with a dark blank screen, one small clear glass ampoule, a steel spatula and a folded white towel, arranged in a loose row from left to right. Soft daylight from the top, warm ivory tones, a faint gold reflection on the ampoule. 35 mm lens, f/8, perfectly perpendicular. No text, no logos, no printed pages.</t>
         </is>
       </c>
       <c r="N76" s="5" t="inlineStr">
         <is>
-          <t>3 s. Start: the top-down desk. The camera zooms into the ampoule until its glass fills the frame; the amber liquid brightens and the frame cuts to a gloved hand holding a clear vial up against a bright laboratory window. End: block 5 image frozen with the four stat counters starting at zero.</t>
+          <t>3 s. Start: the top-down desk. The camera zooms into the ampoule until its glass fills the frame; the glass brightens and the frame cuts to a gloved hand holding a clear vial up against a bright laboratory window. End: block 5 image frozen with the four stat counters starting at zero.</t>
         </is>
       </c>
       <c r="O76" s="5" t="inlineStr">
@@ -56193,17 +56193,17 @@
       </c>
       <c r="K77" s="5" t="inlineStr">
         <is>
-          <t>Text link 'Download the catalogue (PDF)' - the existing MITODERM-Catalog-EN.pdf / HE.pdf</t>
+          <t>Text link 'Download the catalogue (PDF)' - the existing pdf/MITODERM-Catalog-EN.pdf (HE version for the Hebrew page)</t>
         </is>
       </c>
       <c r="L77" s="5" t="inlineStr">
         <is>
-          <t>Stat row of the four spec numbers with counters animating on reveal: IL 'Founded in Israel' · IT · KR 'Laboratory partners' · 100+ 'Countries where VM is used' · 4 'Core principles'. Under it the four principle labels as a 4-up with one line each from the spec. Right third: the laboratory vial photo; left two thirds: facts on ivory.</t>
+          <t>Stat row of the four spec numbers with counters animating on reveal: IL 'Founded in Israel' · IT · KR 'Laboratory partners' · 100+ 'Countries where VM is used' · 4 'Core principles'. Under it the four principle labels as a 4-up with one line each from the spec benefits. Right third: the laboratory vial photo; left two thirds: facts on ivory.</t>
         </is>
       </c>
       <c r="M77" s="5" t="inlineStr">
         <is>
-          <t>Photoreal laboratory still, 16:9. A hand in a white nitrile glove holds a small clear glass vial of pale amber liquid up to a bright frosted laboratory window; behind it, out of focus, white lab benches and glassware. Clean white and ivory palette with one warm gold highlight running through the vial. 100 mm macro lens, f/2.8, eye level, vial in the right third, soft empty space on the left. No text, no labels on the vial, no logos.</t>
+          <t>Photoreal laboratory still, 16:9. A hand in a white nitrile glove holds a small clear glass vial of pale liquid up to a bright frosted laboratory window; behind it, out of focus, white lab benches and glassware. Clean white and ivory palette with one warm gold highlight running through the vial. 100 mm macro lens, f/2.8, eye level, vial in the right third, soft empty space on the left. No text, no labels on the vial, no logos.</t>
         </is>
       </c>
       <c r="N77" s="5" t="inlineStr">
@@ -56273,7 +56273,7 @@
       </c>
       <c r="L78" s="5" t="inlineStr">
         <is>
-          <t>Dark gold band #1C1510, the emblem centred above the title with its glow; contact form 1/2 left (4 fields + submit), the three labels as pills on the right with one sentence each from the spec CTA; footer with the real logo, phone, e-mail, address placeholders. No animation beyond the glow breathing and the form fields sliding in.</t>
+          <t>Dark gold band #1C1510, the emblem centred above the title with its glow; contact form 1/2 left (4 fields + submit), the labels as pills on the right; footer with the real logo, phone, e-mail, address placeholders. No animation beyond the glow breathing and the form fields sliding in.</t>
         </is>
       </c>
       <c r="M78" s="5" t="inlineStr">
@@ -56358,7 +56358,7 @@
       </c>
       <c r="N79" s="5" t="inlineStr">
         <is>
-          <t>4 s. Start: the vesicle in the right third. The camera pulls back fast: the sphere shrinks to one of thousands drifting above a curved amber surface - skin at macro scale. The scene tilts into a clean cross-section of skin; larger amber molecules settle on the surface and stop there, unable to pass. End: block 1 frame frozen, bronze reduced to a thin copper line.</t>
+          <t>4 s. Start: the vesicle in the right third. The camera pulls back: the sphere shrinks to one of thousands drifting above a curved pale surface - skin at macro scale. The scene tilts into a clean cross-section of skin; larger amber molecules settle on the surface and stop there, unable to pass. End: block 1 frame frozen, bronze reduced to a thin copper line.</t>
         </is>
       </c>
       <c r="O79" s="5" t="inlineStr">
@@ -56498,7 +56498,7 @@
       </c>
       <c r="L81" s="5" t="inlineStr">
         <is>
-          <t>Darkest block, deep bronze. Centre-right: the vesicle cut open (cutaway / exploded view), its contents floating as distinct amber, copper and pale-gold particles; the four chips on the left are wired to the particles - tap one and it pulses. Secondary caption under the chips: 'also plant stem cells, vitamins and antioxidants'. Scroll parallax: the membrane halves drift apart slowly.</t>
+          <t>Darkest block, deep bronze. Centre-right: the vesicle cut open (cutaway / exploded view), its contents floating as distinct amber, copper and pale-gold particles; the four chips on the left are wired to the particles - tap one and it pulses. The remaining actives are already named in the line, so no extra caption. Scroll parallax: the membrane halves drift apart slowly.</t>
         </is>
       </c>
       <c r="M81" s="5" t="inlineStr">
@@ -56508,7 +56508,7 @@
       </c>
       <c r="N81" s="5" t="inlineStr">
         <is>
-          <t>5 s. Start: the open vesicle. The halves close and the camera rises straight up through the warm dermal layer, breaks the pale skin surface and keeps rising into real light: we are above a client's cheek in a clinic; a practitioner's gloved hand enters with a glass ampoule and touches a drop of amber serum to the skin. The client opens her eyes and looks straight at the camera. End: block 3 mirror portrait frozen.</t>
+          <t>5 s. Start: the open vesicle. The halves close and the camera rises straight up through the warm dermal layer, breaks the pale skin surface and keeps rising into real light: we are above a client's cheek in a clinic; a practitioner's gloved hand enters with a clear glass ampoule and touches a drop of serum to the skin. The client opens her eyes and looks straight at the camera. End: block 3 mirror portrait frozen.</t>
         </is>
       </c>
       <c r="O81" s="5" t="inlineStr">
@@ -56573,17 +56573,17 @@
       </c>
       <c r="L82" s="5" t="inlineStr">
         <is>
-          <t>Full-bleed mirror scene: a client reclined in a warm clinic looks straight at us (the mirror) while a practitioner's gloved hand applies a drop of the exosome serum from a glass ampoule to her cheek after a treatment; her face is fresh, calm. Text 1/3 left over a bronze-to-transparent gradient; the four labels appear along a thin copper path drawn from the ampoule to the cheek (encapsulate -&gt; protect -&gt; deliver -&gt; release). No before/after - the catalogue has none for this page.</t>
+          <t>Full-bleed mirror scene: a client reclined in a warm clinic looks straight at us (the mirror) while a practitioner's gloved hand applies a drop of serum from a clear glass ampoule (V-TECH) to her cheek after a treatment; her face is fresh, calm. Text 1/3 left over a bronze-to-transparent gradient; the four labels appear along a thin copper path drawn from the ampoule to the cheek (encapsulate -&gt; protect -&gt; deliver -&gt; release). No before/after - the catalogue has none for this page.</t>
         </is>
       </c>
       <c r="M82" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic portrait, 16:9. A woman in her forties with natural, freshly treated skin reclines in a treatment chair in a warm modern clinic and looks directly into the lens as if into a mirror; a practitioner's hand in a white nitrile glove, seen from the side, touches a small clear glass ampoule with amber serum to her cheekbone. Warm bronze and ivory palette, soft window light from the left, gentle copper rim light on her hair. 85 mm lens, f/2, eye level, her face in the right two thirds, soft empty space on the left. No text, no logos, no visible brand on the ampoule.</t>
+          <t>Photoreal cinematic portrait, 16:9. A woman in her forties with natural, freshly treated skin reclines in a treatment chair in a warm modern clinic and looks directly into the lens as if into a mirror; a practitioner's hand in a white nitrile glove, seen from the side, touches a small clear glass ampoule to her cheekbone. Warm bronze and ivory palette, soft window light from the left, gentle copper rim light on her hair. 85 mm lens, f/2, eye level, her face in the right two thirds, soft empty space on the left. No text, no logos, no visible brand on the ampoule.</t>
         </is>
       </c>
       <c r="N82" s="5" t="inlineStr">
         <is>
-          <t>3 s. Start: her eyes on the camera. She closes them; the camera pulls back and pans left from the chair to a pale-oak shelf along the clinic wall, where six products stand in a row under warm spot light. Three copper dots light along the shelf edge (clinic - finish - home). End: block 4 shelf plate with the real packshots in place.</t>
+          <t>3 s. Start: her eyes on the camera. She closes them; the camera pulls back and pans left from the chair to a pale-oak shelf along the clinic wall, where the five products with packshots stand in a row under warm spot light. Three copper dots light along the shelf edge (clinic - finish - home). End: block 4 shelf plate with the real packshots in place.</t>
         </is>
       </c>
       <c r="O82" s="5" t="inlineStr">
@@ -56648,7 +56648,7 @@
       </c>
       <c r="L83" s="5" t="inlineStr">
         <is>
-          <t>Three step groups on the copper step line that draws on scroll: 1 Clinic (vtech-system.webp, exo-nad.webp) -&gt; 2 Finish (exocell-mask.webp) -&gt; 3 Home (exotech-gel.webp); a second quieter row for the scalp path: exosignal-hair.webp -&gt; EXOSIGNAL SPRAY (no packshot yet - placeholder) with the caption 'works with MITOPEN'. Packshots rise on reveal; the background is the shelf plate from the transition.</t>
+          <t>Three step groups on the copper step line that draws on scroll: 1 Clinic (vtech-system.webp, exo-nad.webp) -&gt; 2 Finish (exocell-mask.webp) -&gt; 3 Home (exotech-gel.webp); a second quieter row for the scalp path: exosignal-hair.webp -&gt; EXOSIGNAL SPRAY as a text chip linking to its page until a packshot exists (no placeholder graphic), with the caption 'works with MITOPEN'. Packshots rise on reveal; the background is the shelf plate from the transition.</t>
         </is>
       </c>
       <c r="M83" s="5" t="inlineStr">
@@ -56658,7 +56658,7 @@
       </c>
       <c r="N83" s="5" t="inlineStr">
         <is>
-          <t>3 s. Start: the shelf with six products. The camera tracks right past the last product to a wall-mounted rack of glass ampoules in a laboratory; the warm clinic light turns to clean lab daylight with one copper highlight. End: block 5 ampoule-rack plate with the four stat counters at zero.</t>
+          <t>3 s. Start: the shelf with the products. The camera tracks right past the last product to a wall-mounted rack of glass ampoules in a laboratory; the warm clinic light turns to clean lab daylight with one copper highlight. End: block 5 ampoule-rack plate with the four stat counters at zero.</t>
         </is>
       </c>
       <c r="O83" s="5" t="inlineStr">
@@ -56703,12 +56703,12 @@
       </c>
       <c r="H84" s="5" t="inlineStr">
         <is>
-          <t>Made in Italy, used worldwide</t>
+          <t>Developed in Italy, used worldwide</t>
         </is>
       </c>
       <c r="I84" s="5" t="inlineStr">
         <is>
-          <t>Developed by VM Corporation in Italy, used by medical professionals in 100+ countries; MITODERM is the exclusive importer in Israel.</t>
+          <t>Developed by VM Corporation in Italy, marketed to medical professionals in 100+ countries; MITODERM is its exclusive importer in Israel.</t>
         </is>
       </c>
       <c r="J84" s="5" t="inlineStr">
@@ -56718,22 +56718,22 @@
       </c>
       <c r="K84" s="5" t="inlineStr">
         <is>
-          <t>Text link 'Download the catalogue (PDF)'</t>
+          <t>Text link 'Download the catalogue (PDF)' - the existing pdf/MITODERM-Catalog-EN.pdf</t>
         </is>
       </c>
       <c r="L84" s="5" t="inlineStr">
         <is>
-          <t>Stat row with the four spec numbers counting up on reveal (VM · 100+ · Nano · 0) over the four labels; under it, the four 'Why synthetic' advantages from the spec as a compact 4-up with one line each. Right third: the ampoule-rack photo; left two thirds: facts on bronze-tinted ivory.</t>
+          <t>Stat row with the four spec numbers counting up on reveal (VM · 100+ · Nano · 0) over the four labels; under it, the four 'Why synthetic' advantages from the spec benefits as a compact 4-up with one line each. Right third: the ampoule-rack photo; left two thirds: facts on bronze-tinted ivory.</t>
         </is>
       </c>
       <c r="M84" s="5" t="inlineStr">
         <is>
-          <t>Photoreal laboratory still, 16:9. A neat rack of clear glass ampoules filled with pale amber liquid stands on a white laboratory bench in front of a bright frosted window; one ampoule in the front row is in sharp focus, the rest fall softly out of focus. Clean white and ivory palette with one warm copper reflection running through the glass. 100 mm macro lens, f/2.8, eye level, rack in the right third, soft empty space on the left. No text, no labels on the ampoules, no logos.</t>
+          <t>Photoreal laboratory still, 16:9. A neat rack of clear glass ampoules stands on a white laboratory bench in front of a bright frosted window; one ampoule in the front row is in sharp focus, the rest fall softly out of focus. Clean white and ivory palette with one warm copper reflection running through the glass. 100 mm macro lens, f/2.8, eye level, rack in the right third, soft empty space on the left. No text, no labels on the ampoules, no logos.</t>
         </is>
       </c>
       <c r="N84" s="5" t="inlineStr">
         <is>
-          <t>4 s. Start: the ampoule rack in lab light. The front ampoule's amber brightens and the frame dips to deep bronze; from the dark, the single vesicle from the opening returns, centred and glowing, slowly rotating. End: block 6 dark bronze band with the vesicle above the contact form.</t>
+          <t>4 s. Start: the ampoule rack in lab light. The front ampoule's highlight brightens and the frame dips to deep bronze; from the dark, the single vesicle from the opening returns, centred and glowing, slowly rotating. End: block 6 dark bronze band with the vesicle above the contact form.</t>
         </is>
       </c>
       <c r="O84" s="5" t="inlineStr">
@@ -56793,7 +56793,7 @@
       </c>
       <c r="K85" s="5" t="inlineStr">
         <is>
-          <t>Primary button 'Contact us' (copper, opens form: name, phone, clinic, message); secondary 'Request prices'; sticky bottom CTA 'Contact us' on mobile</t>
+          <t>Primary button 'Contact us' (copper, opens form: name, phone, clinic, message); secondary 'See the products' (outline, to the three product pages); sticky bottom CTA 'Contact us' on mobile</t>
         </is>
       </c>
       <c r="L85" s="5" t="inlineStr">
@@ -56883,7 +56883,7 @@
       </c>
       <c r="N86" s="5" t="inlineStr">
         <is>
-          <t>4 s. Start: the single spicule in the right third. The camera pulls back: the needle becomes one of thousands woven into a pale sponge skeleton; keep pulling back through clear green water until the whole sponge sits on a stone in a sunlit lake. Cut on a ripple to a laboratory dish where a heap of grey-green raw sponge powder sits under a loupe. End: block 1 frame frozen, green reduced to a thin line.</t>
+          <t>4 s. Start: the single spicule in the right third. The camera pulls back: the needle becomes one of thousands woven into a pale sponge skeleton, then the whole sponge resting on a stone in clear, sunlit freshwater. Cut on a ripple to a laboratory dish where a heap of raw sponge powder sits under a loupe. End: block 1 frame frozen, green reduced to a thin line.</t>
         </is>
       </c>
       <c r="O86" s="5" t="inlineStr">
@@ -56933,7 +56933,7 @@
       </c>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>Traditional Spongilla powder is one non-uniform mixture of the whole raw material; results depend on purity, spicule size and concentration.</t>
+          <t>Traditional Spongilla powder is one non-uniform mixture of the whole raw material; purity, size ratio and concentration decide everything.</t>
         </is>
       </c>
       <c r="J87" s="5" t="inlineStr">
@@ -56948,17 +56948,17 @@
       </c>
       <c r="L87" s="5" t="inlineStr">
         <is>
-          <t>2/3 image left, 1/3 text right on sage-tinted ivory. Image: a lab dish with a heap of raw, uneven grey-green sponge powder under a loupe - fragments of every size, residue visible. On scroll a thin green line scans across the heap and the three dependency labels light up where the heap fails them; the fourth label 'Non-uniform powder' is the verdict.</t>
+          <t>2/3 image left, 1/3 text right on sage-tinted ivory. Image: a lab dish with a heap of raw, uneven sponge powder under a loupe - fragments of every size, residue visible. On scroll a thin green line scans across the heap and the three dependency labels light up where the heap fails them; the fourth label 'Non-uniform powder' is the verdict.</t>
         </is>
       </c>
       <c r="M87" s="5" t="inlineStr">
         <is>
-          <t>Photoreal laboratory macro photograph, 16:9. A white ceramic laboratory dish holding a loose heap of raw grey-green sponge powder with visibly uneven fragments and fibrous residue, a brass-rimmed loupe lying beside it on a white bench; soft daylight from the left, cool sage-ivory palette, one green reflection in the loupe glass. 100 mm macro lens, f/4, slightly elevated angle, dish in the left two thirds, clean empty space on the right. No text, no labels, no logos.</t>
+          <t>Photoreal laboratory macro photograph, 16:9. A white ceramic laboratory dish holding a loose heap of raw, muted grey-green sponge powder with visibly uneven fragments and fibrous residue, a brass-rimmed loupe lying beside it on a white bench; soft daylight from the left, cool sage-ivory palette, one green reflection in the loupe glass. 100 mm macro lens, f/4, slightly elevated angle, dish in the left two thirds, clean empty space on the right. No text, no labels, no logos.</t>
         </is>
       </c>
       <c r="N87" s="5" t="inlineStr">
         <is>
-          <t>5 s. Start: the raw powder in the dish. The powder lifts into the air as a cloud and streams through four parallel glass channels; residue drops away at the first channel, then the particles sort themselves by length into four clean groups; the camera pushes into the longest group, picks one needle and slices it lengthwise to reveal the hollow inner cavity. End: block 2 - the cutaway spicule on the darkest green.</t>
+          <t>5 s. Start: the raw powder in the dish. The powder lifts into the air as a cloud and streams through a clear glass sorting channel; residue drops away first, then the needles settle into two clean groups, short and long. The camera pushes into the long group, picks one needle and slices it lengthwise to reveal the hollow inner cavity. End: block 2 - the cutaway spicule on the darkest green.</t>
         </is>
       </c>
       <c r="O87" s="5" t="inlineStr">
@@ -57003,7 +57003,7 @@
       </c>
       <c r="H88" s="5" t="inlineStr">
         <is>
-          <t>Inside every needle, a channel</t>
+          <t>Every needle is hollow inside</t>
         </is>
       </c>
       <c r="I88" s="5" t="inlineStr">
@@ -57023,22 +57023,22 @@
       </c>
       <c r="L88" s="5" t="inlineStr">
         <is>
-          <t>Darkest block, deep green. Centre-right: the spicule cut lengthwise, the inner cavity glowing pale amber as it fills with serum on scroll; left: the four chips, and under them four spicules of different lengths lined up side by side (the 'four types', short to long, no lengths shown here). Scroll parallax: the two halves of the cutaway drift apart slowly.</t>
+          <t>Darkest block, deep green. Centre-right: the spicule cut lengthwise, the inner cavity glowing softly as it fills with serum on scroll; left: the four chips, and under them one short and one long spicule side by side (the short/long balance from the catalogue - no lengths, no count shown). Scroll parallax: the two halves of the cutaway drift apart slowly.</t>
         </is>
       </c>
       <c r="M88" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic macro render, 16:9. A translucent silica micro-needle sliced lengthwise, the two halves slightly apart in the centre-right of frame, revealing an elongated hollow inner cavity with a finely porous wall, the cavity lit from inside with a pale amber glow; beside it to the left, four intact needles of increasing length lie in a neat row. Deep forest-green background #1E4634, cool green rim light, soft ivory key light, volumetric haze. 100 mm macro lens, f/2.8, shallow focus on the cavity. No text, no labels, no scale bars, no logos.</t>
+          <t>Photoreal cinematic macro render, 16:9. A translucent silica micro-needle sliced lengthwise, the two halves slightly apart in the centre-right of frame, revealing an elongated hollow inner cavity with a finely porous wall, the cavity lit from inside with a soft warm glow; beside it to the left, two intact needles lie in a neat row, one short and one long. Deep forest-green background #1E4634, cool green rim light, soft ivory key light, volumetric haze. 100 mm macro lens, f/2.8, shallow focus on the cavity. No text, no labels, no scale bars, no logos.</t>
         </is>
       </c>
       <c r="N88" s="5" t="inlineStr">
         <is>
-          <t>5 s. Start: the open spicule with its amber-lit cavity. The halves close, the needle shrinks and joins thousands of others suspended in a drop of amber serum; the camera pulls back until the drop sits on a fingertip; the fingertip rises and touches a cheek. The camera keeps pulling back: a woman at a mirror, fingertips on her cheekbone, looking straight at us. End: block 3 mirror portrait frozen.</t>
+          <t>5 s. Start: the open spicule with its lit cavity. The halves close, the needle shrinks and joins thousands of others suspended in a drop of clear serum; the camera pulls back until the drop sits on a fingertip; the fingertip rises and touches a cheek. The camera keeps pulling back: a woman at a mirror, fingertips on her cheekbone, looking straight at us. End: block 3 mirror portrait frozen.</t>
         </is>
       </c>
       <c r="O88" s="5" t="inlineStr">
         <is>
-          <t>390 px: chips 2x2 above, cutaway render at 4:5 (55vh) below with the cavity centred; the four-length row becomes a small strip under the render; parallax off.</t>
+          <t>390 px: chips 2x2 above, cutaway render at 4:5 (55vh) below with the cavity centred; the short/long pair becomes a small strip under the render; parallax off.</t>
         </is>
       </c>
     </row>
@@ -57108,7 +57108,7 @@
       </c>
       <c r="N89" s="5" t="inlineStr">
         <is>
-          <t>3 s. Start: her eyes on the camera. She lowers her hand; the camera pans right to a pale-oak shelf beside the mirror, where four products stand under three soft spots; three green dots light along the shelf edge (clinic - home - recovery). End: block 4 shelf plate with the real packshots in place.</t>
+          <t>3 s. Start: her eyes on the camera. She lowers her hand; the camera pans right to a pale-oak shelf beside the mirror, where the four products stand under three soft spots; three green dots light along the shelf edge (clinic - home - recovery). End: block 4 shelf plate with the real packshots in place.</t>
         </is>
       </c>
       <c r="O89" s="5" t="inlineStr">
@@ -57233,7 +57233,7 @@
       </c>
       <c r="I91" s="5" t="inlineStr">
         <is>
-          <t>Penetration 80-300 µm into the epidermis, continued stimulation up to 72 h, four spicule types, fourth-generation purification.</t>
+          <t>Penetration 80-300 µm into the epidermis, continued stimulation up to 72 h, four spicule types, fourth-generation technology.</t>
         </is>
       </c>
       <c r="J91" s="5" t="inlineStr">
@@ -57243,12 +57243,12 @@
       </c>
       <c r="K91" s="5" t="inlineStr">
         <is>
-          <t>Text link 'Download the BIOSPICULE™ brochure (PDF)' - the existing MITODERM-BIOSPICULE-EN.pdf</t>
+          <t>Text link 'Download the BIOSPICULE™ brochure (PDF)' - the existing pdf/MITODERM-BIOSPICULE-EN.pdf</t>
         </is>
       </c>
       <c r="L91" s="5" t="inlineStr">
         <is>
-          <t>Stat row with the four spec numbers counting up on reveal over the four labels; under it a compact 2-up from the spec: Resurfacing / Delivery (the two parallel mechanisms), and the indications chips from the template collapsed to one row with 'show all'. Right third: the microscope-style illustration (captioned 'illustration'); left two thirds: facts on sage-tinted ivory.</t>
+          <t>Stat row with the four spec numbers counting up on reveal over the four labels; under it a compact 2-up from the spec benefits: Resurfacing / Delivery (the two parallel mechanisms), and the indications chips from the template collapsed to one row with 'show all'. Right third: the microscope-style illustration (captioned 'illustration'); left two thirds: facts on sage-tinted ivory.</t>
         </is>
       </c>
       <c r="M91" s="5" t="inlineStr">
@@ -57318,7 +57318,7 @@
       </c>
       <c r="K92" s="5" t="inlineStr">
         <is>
-          <t>Primary button 'Contact us' (green, opens form: name, phone, clinic, message); secondary 'Request prices'; sticky bottom CTA 'Contact us' on mobile</t>
+          <t>Primary button 'Contact us' (green, opens form: name, phone, clinic, message); secondary 'See the range' (outline, to the four BIOSPICULE™ product pages); sticky bottom CTA 'Contact us' on mobile</t>
         </is>
       </c>
       <c r="L92" s="5" t="inlineStr">
@@ -57398,12 +57398,12 @@
       </c>
       <c r="L93" s="5" t="inlineStr">
         <is>
-          <t>Split 1/2–1/2 on a champagne gradient. Left: eyebrow 'SYNTHETIC EXOSOMES · SKIN LONGEVITY PEEL', headline, line, 4 chips (black on champagne), buttons. Right: the square champagne-gold box with the amber vial, turquoise vial and gold-capped square bottle in front; real packshot composited. Load: gold flecks drift inside the bottle (particle layer), box fades in, vials rise.</t>
+          <t>Split 1/2–1/2 on a champagne gradient. Left: eyebrow 'SYNTHETIC EXOSOMES · SKIN LONGEVITY PEEL', headline, line, 4 chips (black on champagne), buttons. Right: the near-square champagne-gold box with the amber vial, turquoise vial and gold-capped square bottle in front; real packshot composited. Load: gold flecks drift inside the bottle (particle layer), box fades in, vials rise.</t>
         </is>
       </c>
       <c r="M93" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product hero, 16:9. A square carton finished in a champagne-gold gradient (pale warm ivory at the top left to deep gold at the right) standing on the right third on a warm cream stone surface; in front of it three vessels: a small amber glass vial with a silver cap, a small turquoise-blue glass vial with a silver cap, and a square clear glass bottle with a tall gold cap holding a pale liquid with fine gold flecks. Background: soft champagne (#F3E4C2) gradient, warm sunlight from the upper left, long soft shadows, subtle warm bloom. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds clear for text. No overlay text, no logos; pack faces clean so the real packshot PNG can be composited.</t>
+          <t>Photoreal cinematic product hero, 16:9. A near-square carton, slightly wider than tall, finished in a champagne-gold gradient (pale warm ivory at the top left to deep gold at the right) standing on the right third on a warm cream stone surface; in front of it three vessels: a small amber glass vial with a silver cap, a small turquoise-blue glass vial with a silver cap, and a square clear glass bottle with a tall gold cap holding a pale liquid with fine gold flecks. Background: soft champagne (#F3E4C2) gradient, warm sunlight from the upper left, long soft shadows, subtle warm bloom. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds clear for text. No overlay text, no logos; pack faces clean so the real packshot PNG can be composited.</t>
         </is>
       </c>
       <c r="N93" s="5" t="inlineStr">
@@ -57483,7 +57483,7 @@
       </c>
       <c r="N94" s="5" t="inlineStr">
         <is>
-          <t>Start: block-1 cheek. The square bottle tilts into the frame; its contents separate into two visible layers; the camera glides between the lipid layer and the acid layer, past an amber vial, past a turquoise vial, as each liquid swirls; the three vessels line up. End: block-2 still life. 5 s, lateral glide through three liquids.</t>
+          <t>Start: block-1 cheek. The square gold-capped bottle tilts into the frame, gold flecks drifting; the camera dives into its liquid, where an oily phase floats over a watery, fleck-filled phase, then glides on past an amber vial and a turquoise vial as each liquid swirls; the three vessels line up on cream stone. End: block-2 still life. 5 s, lateral glide through three liquids.</t>
         </is>
       </c>
       <c r="O94" s="5" t="inlineStr">
@@ -57548,17 +57548,17 @@
       </c>
       <c r="L95" s="5" t="inlineStr">
         <is>
-          <t>Three columns, one per vessel, each with a macro swirl of its liquid behind it; columns reveal left to right on scroll (1 → 2 → 3), the biphasic bottle shows its two layers separating as it enters. Labels sit under each column; the fourth label is a footnote under column 1. Headline and line above the columns.</t>
+          <t>Three columns, one per vessel, each with a macro swirl of its liquid behind it; columns reveal left to right on scroll (1 → 2 → 3); the macro swirl behind column 1 shows an oily phase floating over the acid phase (the bottle itself stays as on the packshot: pale liquid with gold flecks). Labels sit under each column; the fourth label is a footnote under column 1. Headline and line above the columns.</t>
         </is>
       </c>
       <c r="M95" s="5" t="inlineStr">
         <is>
-          <t>Photoreal macro still life, 16:9. Three liquids in a row on warm cream stone under sunlight: left, a square clear glass bottle with a gold cap, its contents visibly separated into two layers — a clear oily phase floating over a pale fleck-filled phase; centre, an amber vial with a silver cap; right, a turquoise-blue vial with a silver cap; behind each an out-of-focus macro swirl of its liquid. Lighting: warm champagne (#F3E4C2) backdrop, strong sun from the left, gold flecks sparkling. Camera: 100 mm macro, f/4, vessels sharp. No overlay text, no logos; pack faces clean.</t>
+          <t>Photoreal macro still life, 16:9. Three vessels in a row on warm cream stone under sunlight: left, a square clear glass bottle with a tall gold cap holding a pale liquid with fine gold flecks; centre, a small amber glass vial with a silver cap; right, a small turquoise-blue glass vial with a silver cap; behind each an out-of-focus macro swirl of its liquid — behind the bottle, a clear oily phase floating over a watery, fleck-filled phase. Lighting: warm champagne (#F3E4C2) backdrop, strong sun from the left, gold flecks sparkling. Camera: 100 mm macro, f/4, vessels sharp. No overlay text, no logos; pack faces clean.</t>
         </is>
       </c>
       <c r="N95" s="5" t="inlineStr">
         <is>
-          <t>Start: block-2 vessels. Pull back; a woman faces us as into a mirror; a fan brush sweeps the two-phase peel over her cheek, then gloved fingers press a drop of pale serum into the cheekbone; her skin brightens in the sun and her eyes meet the lens. End: block-3 mirror portrait. 5 s, reverse dolly, bloom rises.</t>
+          <t>Start: block-2 vessels. Pull back; a woman faces us as into a mirror; a fan brush sweeps the peel over her cheek, then gloved fingers press a drop of pale serum into the cheekbone; sunlight warms across her face and her eyes meet the lens. End: block-3 mirror portrait. 5 s, reverse dolly, bloom rises.</t>
         </is>
       </c>
       <c r="O95" s="5" t="inlineStr">
@@ -57633,7 +57633,7 @@
       </c>
       <c r="N96" s="5" t="inlineStr">
         <is>
-          <t>Start: block-3 portrait. She closes her eyes; tilt down to the tray and continue to overhead; bottle, fan brush, amber vial, turquoise vial, folded mask, sunscreen glide into one row; a gold line draws and three dots pulse beneath. End: block-4 flat lay. 4 s, tilt-down to overhead.</t>
+          <t>Start: block-3 portrait. She closes her eyes; tilt down to the tray and continue to overhead; gold-capped bottle, fan brush, amber vial, turquoise vial, folded pale-blue mask in front of a small teal carton, plain white sunscreen tube glide into one row; a gold line draws and three dots pulse beneath. End: block-4 flat lay. 4 s, tilt-down to overhead.</t>
         </is>
       </c>
       <c r="O96" s="5" t="inlineStr">
@@ -57703,12 +57703,12 @@
       </c>
       <c r="M97" s="5" t="inlineStr">
         <is>
-          <t>Photoreal top-down flat lay, 16:9. On warm cream stone, left to right in a straight row with space between: a square clear glass bottle with a gold cap and two-layer liquid, a fan brush, an amber vial with a silver cap, a turquoise vial with a silver cap, then a folded translucent pale-blue sheet mask on a teal card and a small white sunscreen tube. Lighting: sunlight from the upper left, long soft shadows, champagne (#F3E4C2) tone. Camera: overhead, 50 mm, f/8, all sharp. No overlay text, no logos; pack faces clean.</t>
+          <t>Photoreal top-down flat lay, 16:9. On warm cream stone, left to right in a straight row with space between: a square clear glass bottle with a tall gold cap and pale gold-flecked liquid, a fan brush, a small amber vial with a silver cap, a small turquoise vial with a silver cap, then a folded translucent pale-blue sheet mask lying in front of a small matte teal carton and a plain white unbranded sunscreen tube. Lighting: sunlight from the upper left, long soft shadows, champagne (#F3E4C2) tone. Camera: overhead, 50 mm, f/8, all sharp. No overlay text, no logos; pack faces clean.</t>
         </is>
       </c>
       <c r="N97" s="5" t="inlineStr">
         <is>
-          <t>Start: block-4 flat lay. Items slide left into the champagne box as it rises to three-quarter view and its lid opens; inside, the 15 ml bottle, five amber vials and five turquoise vials appear and lay themselves out beside it. End: block-5 kit shot. 5 s, camera rises to 20° above eye level.</t>
+          <t>Start: block-4 flat lay. Brush, mask, teal carton and sunscreen slide off-frame; the champagne box glides in and rises to three-quarter view as the camera lifts to 20° above eye level; the gold-capped bottle stays put while five amber vials and five turquoise vials glide in from the right into two rows beside the closed box. End: block-5 kit shot. 5 s, continuous camera lift.</t>
         </is>
       </c>
       <c r="O97" s="5" t="inlineStr">
@@ -57773,17 +57773,17 @@
       </c>
       <c r="L98" s="5" t="inlineStr">
         <is>
-          <t>Split 1/2–1/2. Left: open box with the 1 + 5 + 5 laid out (real packshot composited for the box). Right: four large numbers counting up (15 ml · 5 · 5 · ≈30%) with labels; a caption '3 stages · 3–4 weeks between treatments · Fitzpatrick I–VI'.</t>
+          <t>Split 1/2–1/2. Left: the closed box in three-quarter view with the 1 + 5 + 5 laid out beside it (real packshot composited for the box; the catalogue shows no box interior, so the lid stays closed). Right: four large numbers counting up (15 ml · 5 · 5 · ≈30%) with labels; a caption '3 stages · 3–4 weeks between treatments · Fitzpatrick I–VI'.</t>
         </is>
       </c>
       <c r="M98" s="5" t="inlineStr">
         <is>
-          <t>Photoreal product shot, 16:9. The champagne-gold gradient square carton, lid open, in three-quarter view on the left; beside it on cream stone, laid out neatly: one square clear glass bottle with a gold cap, a row of five amber vials with silver caps and a row of five turquoise-blue vials with silver caps. Lighting: warm sunlight from the upper right, soft champagne backdrop, gentle bloom. Camera: 70 mm, f/5.6, everything sharp, right third clear for numbers. No overlay text, no logos; pack faces clean.</t>
+          <t>Photoreal product shot, 16:9. The champagne-gold gradient near-square carton, closed, in three-quarter view on the left; beside it on cream stone, laid out neatly: one square clear glass bottle with a tall gold cap and gold-flecked liquid, a row of five small amber vials with silver caps and a row of five small turquoise-blue vials with silver caps. Lighting: warm sunlight from the upper right, soft champagne backdrop, gentle bloom. Camera: 70 mm, f/5.6, everything sharp, right third clear for numbers. No overlay text, no logos; pack faces clean.</t>
         </is>
       </c>
       <c r="N98" s="5" t="inlineStr">
         <is>
-          <t>Start: block-5 open box. The lid closes; the three hero vessels step forward; the box drifts to the right third; sunlight warms, bloom rises, a gold reflection line draws. End: block-6 closing hero. 3 s, dolly-out.</t>
+          <t>Start: block-5 kit shot. The rows contract: one amber and one turquoise vial step forward beside the gold-capped bottle while the rest slide behind the box; the box drifts to the right third; sunlight warms, bloom rises, a gold reflection line draws. End: block-6 closing hero. 3 s, dolly-out.</t>
         </is>
       </c>
       <c r="O98" s="5" t="inlineStr">
@@ -57853,7 +57853,7 @@
       </c>
       <c r="M99" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic closing hero, 16:9. The champagne-gold carton on the right third on cream stone, the three vessels (amber vial, turquoise vial, square gold-capped bottle) in front, warm sunlight from the left, soft bloom, a thin gold reflection line; the left two-thirds clean champagne (#F3E4C2) for the offer and buttons. Camera: 85 mm, eye level, f/4. Warm, calm, final. No overlay text, no logos; pack faces clean.</t>
+          <t>Photoreal cinematic closing hero, 16:9. The champagne-gold near-square carton on the right third on cream stone, the three vessels (small amber vial, small turquoise vial, square gold-capped bottle with gold-flecked liquid) in front, warm sunlight from the left, soft bloom, a thin gold reflection line; the left two-thirds clean champagne (#F3E4C2) for the offer and buttons. Camera: 85 mm, eye level, f/4. Warm, calm, final. No overlay text, no logos; pack faces clean.</t>
         </is>
       </c>
       <c r="N99" s="5" t="inlineStr">
@@ -57923,17 +57923,17 @@
       </c>
       <c r="L100" s="5" t="inlineStr">
         <is>
-          <t>Split 1/2–1/2 on turquoise. Left: eyebrow 'SYNTHETIC EXOSOMES · PROFESSIONAL MASK', headline, line, 4 white chips, buttons. Right: the teal box with the folded translucent mask hovering beside it (as in the real packshot, composited). Load: box fades in, mask floats up 16 px and settles, droplets glint (tiny specular layer). The mask stays folded here — it unfolds across the next two transitions.</t>
+          <t>Split 1/2–1/2 on turquoise. Left: eyebrow 'SYNTHETIC EXOSOMES · PROFESSIONAL MASK', headline, line, 4 white chips, buttons. Right: the teal box (real packshot composited for the box only) with a folded translucent mask hovering beside it. Note: the catalogue packshot shows the mask fully open and face-shaped; here it is rendered folded in half so it can unfold across the next two transitions, as the brief asks. Load: box fades in, mask floats up 16 px and settles, droplets glint (tiny specular layer). The mask stays folded here — it unfolds across the next two transitions.</t>
         </is>
       </c>
       <c r="M100" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product hero, 16:9. A matte teal (#6FAEB0) rectangular carton standing on the right third on a wet pale-aqua stone surface; beside it, floating slightly above the surface, a translucent pale-blue bio-cellulose face mask with eye, nose and mouth cut-outs, folded once so its lower half tucks under, tiny water droplets on its surface. Background: cool turquoise gradient (#DDF3F3 to #6FAEB0), soft cool key light from the upper left, a cool rim light on the mask edge, reflections in the wet surface. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds clear for text. No overlay text, no logos; pack faces clean so the real packshot PNG can be composited.</t>
+          <t>Photoreal cinematic product hero, 16:9. A matte teal (#6FAEB0) portrait-format rectangular carton standing on the right third on a wet pale-aqua stone surface; beside it, floating slightly above the surface, a translucent pale-blue bio-cellulose face mask with eye, nose and mouth cut-outs, folded in half along its vertical centre line so one eye cut-out and half the mouth cut-out show, tiny water droplets on its surface. Background: cool turquoise gradient (#DDF3F3 to #6FAEB0), soft cool key light from the upper left, a cool rim light on the mask edge, reflections in the wet surface. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds clear for text. No overlay text, no logos; pack faces clean so the real packshot PNG can be composited.</t>
         </is>
       </c>
       <c r="N100" s="5" t="inlineStr">
         <is>
-          <t>Start: block-0 hero (teal box right, folded mask beside it). The mask lifts off the surface and the first fold opens (one-third unfolded) as the camera slides behind it; through the translucent sheet a woman's post-procedure cheek comes into focus, flushed and tight. End: block-1 close-up with the mask half-unfolded at the right edge. 4 s, lateral dolly behind the sheet.</t>
+          <t>Start: block-0 hero (teal box right, folded mask beside it). The mask lifts off the surface and the fold opens to a third as the camera slides behind it; through the translucent sheet a woman's post-procedure cheek comes into focus, flushed and tight. End: block-1 close-up with the mask half-unfolded at the right edge. 4 s, lateral dolly behind the sheet.</t>
         </is>
       </c>
       <c r="O100" s="5" t="inlineStr">
@@ -57983,7 +57983,7 @@
       </c>
       <c r="I101" s="5" t="inlineStr">
         <is>
-          <t>Microneedling, peels and spicules can leave skin dry, tight and sensitive. The finishing step decides how your client walks out.</t>
+          <t>After microneedling, peels and spicules, skin asks for hydration and barrier support. The finishing step decides how your client walks out.</t>
         </is>
       </c>
       <c r="J101" s="5" t="inlineStr">
@@ -58158,7 +58158,7 @@
       </c>
       <c r="N103" s="5" t="inlineStr">
         <is>
-          <t>Start: block-3 portrait. She peels the mask up from the chin; the camera pulls back and the frame splits into three moments — gloved hands lifting the sheet toward her face, the sheet on her face, the sheet lifted away — sliding in left to right. End: block-4 three-moment scene. 4 s, pull-back and lateral reveal.</t>
+          <t>Start: block-3 portrait, mask on. She lifts the mask from the chin with both hands; the camera pulls back to a wider three-quarter view of the chair as the practitioner's gloved hands enter to take the sheet; hold as the translucent sheet hangs between them in the cool light. End: block-4 centre panel (mask lifted away, skin dewy). 4 s, slow pull-back; the side panels of block 4 then slide in on scroll, not in the video.</t>
         </is>
       </c>
       <c r="O103" s="5" t="inlineStr">
@@ -58223,17 +58223,17 @@
       </c>
       <c r="L104" s="5" t="inlineStr">
         <is>
-          <t>Three equal panels across the width (the three-moment scene), each with its step number and label; a white step line draws between the panels on scroll; the middle panel plays a 3 s loop of droplets forming on the sheet. Under the strip a 'Works with' chip row linking to the three PRO pages and 'Microneedling'. No wear-time shown — the catalogue gives none (see notes).</t>
+          <t>Three equal panels across the width (the three-moment triptych), each with its step number and label; the centre panel is the end frame of the previous transition, the two side panels slide in from the edges on scroll; a white step line draws between the panels; the middle panel plays a 3 s loop of droplets forming on the sheet. Under the strip a 'Works with' chip row linking to the three PRO pages and 'Microneedling'. No wear-time shown — the catalogue gives none (see notes).</t>
         </is>
       </c>
       <c r="M104" s="5" t="inlineStr">
         <is>
-          <t>Photoreal three-moment scene, 16:9, same woman and room as the mirror portrait: left, gloved hands lift an unfolded pale-blue bio-cellulose sheet mask toward her cleansed face; centre, the mask lies flat on her face, translucent, adhering with no air pockets; right, the mask lifted away from the chin, skin dewy and smooth. Cool turquoise light (#6FAEB0), pale-aqua background, soft shadows. Camera: 50 mm, f/4, the three moments spaced evenly across the frame with narrow gaps. No overlay text, no logos.</t>
+          <t>Photoreal triptych in a single 16:9 frame, three evenly spaced moments separated by narrow bands of pale aqua, same woman, chair and room as the mirror portrait: left, gloved hands lift an unfolded pale-blue bio-cellulose sheet mask toward her cleansed face; centre, the mask lies flat on her face, translucent, adhering with no air pockets; right, the mask lifted away from the chin, skin dewy and smooth. Cool turquoise light (#6FAEB0), pale-aqua background, soft shadows. Camera: 50 mm, f/4, eye level in each panel. No overlay text, no logos.</t>
         </is>
       </c>
       <c r="N104" s="5" t="inlineStr">
         <is>
-          <t>Start: block-4 scene. The lifted sheet folds itself back (the unfold in reverse) and slides into a flat pouch, the pouch into the teal box; the box rotates to three-quarter view and its lid lifts; five pouches fan out beside it. End: block-5 kit shot. 5 s, orbit 30° around the box.</t>
+          <t>Start: block-4 triptych, centre panel. The side panels slide away; the lifted sheet floats toward the lens and settles down flat onto wet pale-aqua stone as the teal carton glides in from the right and stops in three-quarter view behind it. End: block-5 kit shot. 4 s, orbit 30° around the carton.</t>
         </is>
       </c>
       <c r="O104" s="5" t="inlineStr">
@@ -58298,17 +58298,17 @@
       </c>
       <c r="L105" s="5" t="inlineStr">
         <is>
-          <t>Split 1/2–1/2. Left: open teal box with five pouches fanned out, one open with the folded mask drawn halfway (real packshot composited for the box). Right: four facts, the first counting up to 5; a caption 'Dry, tired, sensitive or devitalised skin'. Wet-stone reflection under the box.</t>
+          <t>Split 1/2–1/2. Left: the closed teal carton in three-quarter view with one unfolded mask lying flat on the wet stone in front of it (real packshot composited for the carton; the catalogue shows no box interior or pouches, so none are drawn — the count lives in the number). Right: four facts, the first counting up to 5; a caption 'Dry, tired, sensitive or devitalised skin'. Wet-stone reflection under the box.</t>
         </is>
       </c>
       <c r="M105" s="5" t="inlineStr">
         <is>
-          <t>Photoreal product shot, 16:9. The matte teal carton, lid open, in three-quarter view on the left on wet pale-aqua stone; beside it five flat sealed single-use pouches fanned in a row, one open with the folded pale-blue bio-cellulose mask drawn halfway out, droplets on its surface. Lighting: cool key from the upper right, turquoise gradient backdrop, reflections in the wet stone. Camera: 70 mm, f/5.6, all sharp, right third clear for numbers. No overlay text, no logos; pack and pouch faces clean.</t>
+          <t>Photoreal product shot, 16:9. The matte teal portrait-format carton, closed, in three-quarter view on the left on wet pale-aqua stone; in front of it one unfolded translucent pale-blue bio-cellulose face mask with eye, nose and mouth cut-outs lying flat on the stone, droplets on its surface. Lighting: cool key from the upper right, turquoise gradient backdrop, reflections in the wet stone. Camera: 70 mm, f/5.6, all sharp, right third clear for numbers. No overlay text, no logos; pack face clean.</t>
         </is>
       </c>
       <c r="N105" s="5" t="inlineStr">
         <is>
-          <t>Start: block-5 open box. The pouches slide back in; the lid closes; the folded mask floats up beside the box as in the opening frame; the box settles on the right third, cool light rises, a reflection line draws. End: block-6 closing hero. 3 s, dolly-out.</t>
+          <t>Start: block-5 kit shot. The flat mask lifts off the stone, folds in half and floats up beside the carton as in the opening frame; the carton settles on the right third, cool light rises, a reflection line draws. End: block-6 closing hero. 3 s, dolly-out.</t>
         </is>
       </c>
       <c r="O105" s="5" t="inlineStr">
@@ -58363,7 +58363,7 @@
       </c>
       <c r="J106" s="5" t="inlineStr">
         <is>
-          <t>Contact for price · Training &amp; protocols · Finishes every PRO protocol · Exclusive VM importer, Israel</t>
+          <t>Contact for price · Training &amp; protocols · Finishes every advanced protocol · Exclusive VM importer, Israel</t>
         </is>
       </c>
       <c r="K106" s="5" t="inlineStr">
@@ -58378,7 +58378,7 @@
       </c>
       <c r="M106" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic closing hero, 16:9. The matte teal carton on the right third on wet pale-aqua stone, the folded translucent mask floating beside it as in the opening frame, cool key light, a thin cool reflection line on the surface; the left two-thirds clean pale aqua (#DDF3F3) for the offer and buttons. Camera: 85 mm, eye level, f/4. Cool, calm, final. No overlay text, no logos; pack faces clean.</t>
+          <t>Photoreal cinematic closing hero, 16:9. The matte teal portrait-format carton on the right third on wet pale-aqua stone, the translucent pale-blue mask folded in half floating beside it as in the opening frame, cool key light, a thin cool reflection line on the surface; the left two-thirds clean pale aqua (#DDF3F3) for the offer and buttons. Camera: 85 mm, eye level, f/4. Cool, calm, final. No overlay text, no logos; pack faces clean.</t>
         </is>
       </c>
       <c r="N106" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Add the EXOCELL review-board verdict, Board sheet and storyboard page (pre-repair)
Four role judges, synthesis and a skeptic pass; the skeptic's fixes are
being applied in a repair loop and this file will be replaced.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
+++ b/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Old pages (reference)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Make prompt" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Storyboard" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Board" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -66,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -81,6 +82,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -58395,4 +58397,1112 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Block</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Purchase</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Truth</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Brevity</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Meet</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Хедер работает: продукт, «вторая кожа», «после процедуры» прослеживаются к спеке и стр. 10. Натяжка — чип «Instant cooling» (в каталоге immediate — про гидратацию, cooling отдельно); сложенная пополам маска — выдуманный элемент, биоцеллюлоза должна читаться как реальный лист.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Meet</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Строка повторяет eyebrow и hero_sub, чипы повторяют строку — три слоя одного в одном экране. «After every professional treatment» шире каталога (стр. 10: «after professional cosmetic treatments»). Сложенная маска придумана — спорит с реальным пакшотом, где лист раскрыт.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Meet</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>«Your second skin» пишет каждая биоцеллюлозная маска на рынке; наш единственный дифференциатор — синтетические экзосомальные структуры VM — задвинут в чип. «After every» — переобещание, каталог говорит «after professional cosmetic treatments».</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Meet</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Позиционирование и primary CTA на месте, но H1 без имени продукта и без ключа «bio-cellulose mask» — пусто для SEO; имя EXOCELL MASK впервые появляется в последнем блоке. «Every» — усиление спеки. Сложенная маска — осознанно выдуманный элемент, допустимо ради переходов.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Чипы «After V-TECH / EXO-NAD / MICRO BOOST / microneedling» — ровно то, что я проверяю перед заказом, и они прослеживаются (стр. 7, 9, 19). Но покрасневшее лицо с точечными следами на странице про успокоение — риск; маска, висящая в воздухе у лица, странна; «decides how your client walks out» — продающая отсебятина.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Слово «after» шесть раз в блоке; второе предложение — риторика, в каталоге нет; чипы дублируют ряд блока 4. Кадр — медицинская иллюстрация, не продукт-герой. Делать типографикой на бирюзе, чипы = ссылки, без генерации.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Четыре чипа — самое сильное B2B-место страницы (маска продаётся как завершение наших же протоколов), но вторая фраза ничем не подтверждена, а румянец и «pinpoint marks» на генеративном лице рискуют выглядеть как осложнение. Уместнее три реальных пакшота протоколов и лист маски.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Текст говорит с владельцем клиники на его языке, чипы — правильный внутренний граф ссылок на PRO-страницы. Кадр — самый рискованный на странице (медицина / uncanny valley), продукта в кадре фактически нет. Фраза про «walks out» — риторика, не свойство.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Inside</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Состав честный (все 8 ингредиентов из стр. 10) и это то, что я реально читаю, но строка — перечисление, чипы 3 и 4 составные; «сфера-везикула среди волокон» — клише, которому профессионал не верит; единственный кадр без продукта. Концентраций нет — спрошу у поставщика.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Inside</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Состав перечислен трижды (строка, четыре составных чипа, подпись); «adheres with minimal air pockets» повторяется в блоке 4; «soaked» — не из источников (там «active serum»). «Везикула» в макро — псевдонаука. Текстуру дать кропом реального пакшота.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Inside</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Текст дословно из каталога, но блок перегружен; «увеличенная везикула» — научная неточность, которую заметит любой врач: наноразмерные структуры не видны рядом с волокнами целлюлозы. У бренда «where science meets beauty» такого кадра быть не должно.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Inside</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Каждое слово из стр. 10 — плюс, но это стена из 14 ингредиентов, здесь владелец клиники начнёт пролистывать; «Full formula ↓» никуда не ведёт. Оставить два дифференциатора (экзосомы, полинуклеотиды), остальное — в раскрывающийся список. Макро без лиц — снимаемый кадр.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Feel it</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Каждое слово из каталога, но семь прилагательных через запятую дублируют четыре чипа, чипы дублируют хедер; ничто не двигает к заказу. Пин «Smoothing &amp; firming» на шее намекает на шею, чего в каталоге нет. Кадр с маской на лице — лучший на странице, оставить.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Feel it</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Строка — весь абзац Key Benefits через точку с запятой и дублирует чипы и заголовок; одна фраза должна остаться одной. Пины держать на лице — каталог шею не упоминает. Единственный кадр с человеком — оставить: маска на лице = продукт на коже.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Feel it</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Эмоциональная вершина страницы и всё по каталогу, но фраза перечисляет семь прилагательных — список, не фраза. В кадре маска «turned nearly invisible» — продукт должен читаться: края, вырезы, голубой оттенок, капли.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Feel it</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Эмоциональный пик и лучший кадр, все слова из каталога. Но четыре клаузы и четыре лейбла повторяют друг друга. На десктопе на пике убеждения нет ни одной кнопки — добавить secondary «Contact for price». Нужен видимый влажный край листа, иначе продукт исчезает из кадра.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Главный блок для косметолога — без времени экспозиции («сколько держать?» — первый вопрос, в каталоге ответа нет); шаг «Remove» обрывается, хотя каталог на стр. 7, 9, 19 даёт финиш EXOCELL → DERMA RECOVERY → солнцезащита. Триптих одной женщины в одном 16:9 генератор держит плохо.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Строка повторяет блок 2 и блок 3; лейбл 2 — предложение, а не ярлык; «Works with» дублирует чипы блока 1. Триптих в одном 16:9 не сгенерируется стабильно, луп капель — лишняя генерация. Одна сцена (маска снята), три шага — типографикой.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Ключевой блок для владельца клиники (как встроить в рабочий процесс), но без времени экспозиции пуст — каталог его не даёт, нужен ответ редактора, не выдумка. Чипы длинные, четвёртый — предложение; триптих с одной женщиной в трёх позах — зона риска по консистентности.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Самый перегруженный блок: строка из 3 клауз + 4 лейбла + ряд чипов «Works with» + CTA + триптих + луп. Триптих — худшее задание для генератора (разные лица в панелях). «Cleansed skin» есть только в спеке, не в каталоге.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Kit &amp; facts</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>«Факты» без фактов: два чипа из четырёх повторяют хедер; нет того, что нужно для заказа — объёма (на коробке 5 × 25 ml, в каталоге нет), хранения, «professional use only»; «one per client» логично, но не написано в источниках. Одноразовая маска на мокром камне читается негигиенично.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Kit &amp; facts</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>«One per client» и «one finishing step per protocol» — выводы, не факты; «single-use» есть лишь в спеке; чипы «Bio-cellulose» и «Post-procedure finish» повторяют блок 0. Фактов для закупщика (объём, срок, хранение) нет. Кадр — лучший продуктовый still life страницы, годится как hero и финал.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Kit &amp; facts</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>«5 masks per box» — главный B2B-факт (пять клиентов, расчёт себестоимости процедуры), но два чипа из четырёх дословно повторяют блок 0 и место пропадает; сюда просятся «For professional use only» и показания — то, что владелец клиники проверяет перед заказом.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Kit &amp; facts</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Единственный факт для unit-экономики нужен, но блок назван «trust» и доверия не несёт: лейблы повторяют блок 0, «one per client» — вывод, «single-use» только в спеке. Кадр почти дублирует hero, реальный пакшот уже показывает раскрытую маску. Слить в Offer — минус кадр и переход.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Всё прослеживается (training — стр. 3, exclusive VM importer — стр. 5); «Add to a V-TECH / EXO-NAD enquiry» — именно так я буду заказывать. Но три уровня CTA + контакты + четыре чипа + логотип — перегруз; «VM» без «Italy» косметологу ничего не говорит; кадр — зеркало блока 0, генерировать не нужно.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>Строка почти дословно повторяет блок 0 («the soothing finishing step … every …»); «Contact for price» дублирует кнопку, «Finishes every advanced protocol» дублирует строку — живых лейблов два; четыре CTA в блоке «одна фраза». Отдельная генерация не нужна — кадр блока 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Структура оффера верная для B2B (контакт за ценой, обучение, эксклюзивный импортёр VM), но чип «Contact for price» дублирует кнопку, «every» — переобещание, а главный коммерческий ход «Add to a V-TECH / EXO-NAD enquiry» спрятан во вторую кнопку, хотя маска по каталогу — довесок к этим протоколам.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Механика правильная: WhatsApp + форма, вторичный CTA «добавить к запросу» — лучший кросс-селл. Но половина лейблов потрачена впустую (дубли кнопки и строки). Зеркало блока 0 — бесплатный кадр; idle-луп делать CSS. «For professional use only» в каталоге стоит на странице V-TECH, не EXOCELL.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Make image prompts reproduce the real packaging with all its print
The client's test of the EXOCELL hero came out with a blank box: the
prompts asked for plain faces for later compositing. Every product prompt
now attaches the packshot as reference and asks for its colours and every
printed word; compositing stays a fallback. EXOCELL carton colour taken
from the photo (#5ca0a5). Adds the VM flyer as a source and its facts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
+++ b/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
@@ -50580,7 +50580,7 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product hero, 16:9. A tall rectangular carton wrapped in mirror-polished gold foil with a thin black band at the top and bottom edges, standing upright on the right third of the frame on a black lacquered surface; in front of it five small amber-brown glass vials with white plastic caps and one flat gold-foil sachet. Background: near-black (#0E0C0A) studio with a soft warm gold glow (#D4A853) only behind the carton and faint gold specks in the air. Lighting: single warm key from the upper left, gold rim light on the carton edges, reflections of the vials in the surface. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds empty for text. No overlay text, no logos; pack faces clean so the real packshot PNG can be composited.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/vtech-system.webp. Photoreal cinematic product hero, 16:9. A tall rectangular carton wrapped in mirror-polished gold foil with a thin black band at the top and bottom edges, standing upright on the right third of the frame on a black lacquered surface; in front of it five small amber-brown glass vials with white plastic caps and one flat gold-foil sachet. Background: near-black (#0E0C0A) studio with a soft warm gold glow (#D4A853) only behind the carton and faint gold specks in the air. Lighting: single warm key from the upper left, gold rim light on the carton edges, reflections of the vials in the surface. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds empty for text. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/vtech-system.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
@@ -50880,7 +50880,7 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Photoreal top-down flat lay, 16:9. On matte black slate, left to right: a slim cordless microneedling pen with a champagne-gold body, rose-gold grip ring and clear needle cartridge; an amber glass vial with a white cap; a flat gold-foil sachet; a folded translucent pale-blue bio-cellulose sheet mask lying in front of a small matte teal carton; and a plain white unbranded sunscreen tube. Items in one straight row with generous black space between them for step numbers. Lighting: a thin warm gold rim light from the top, soft fill, long soft shadows. Camera: directly overhead, 50 mm, f/8, everything sharp. No overlay text, no logos; pack faces clean.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/vtech-system.webp. Photoreal top-down flat lay, 16:9. On matte black slate, left to right: a slim cordless microneedling pen with a champagne-gold body, rose-gold grip ring and clear needle cartridge; an amber glass vial with a white cap; a flat gold-foil sachet; a folded translucent pale-blue bio-cellulose sheet mask lying in front of a small matte teal carton; and a plain white unbranded sunscreen tube. Items in one straight row with generous black space between them for step numbers. Lighting: a thin warm gold rim light from the top, soft fill, long soft shadows. Camera: directly overhead, 50 mm, f/8, everything sharp. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/vtech-system.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
@@ -50955,7 +50955,7 @@
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>Photoreal product shot, 16:9. The tall mirror-gold carton with thin black top and bottom bands, closed, standing in three-quarter view on the left; beside it on black lacquer, neatly in two rows: five amber glass vials with white caps and five flat gold-foil sachets. Lighting: warm gold key from the upper right, black background (#0E0C0A), soft gold glow behind the carton only, crisp reflections in the surface. Camera: 70 mm, slightly above eye level, f/5.6, all items sharp, right third empty for numbers. No overlay text, no logos; pack faces clean.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/vtech-system.webp. Photoreal product shot, 16:9. The tall mirror-gold carton with thin black top and bottom bands, closed, standing in three-quarter view on the left; beside it on black lacquer, neatly in two rows: five amber glass vials with white caps and five flat gold-foil sachets. Lighting: warm gold key from the upper right, black background (#0E0C0A), soft gold glow behind the carton only, crisp reflections in the surface. Camera: 70 mm, slightly above eye level, f/5.6, all items sharp, right third empty for numbers. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/vtech-system.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
@@ -51030,7 +51030,7 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic hero, 16:9, closing frame. The tall mirror-gold carton with thin black top and bottom bands stands on the right third on black lacquer, five amber vials with white caps and the flat gold-foil sachet in front, the set lit by a warm gold glow (#D4A853) behind the carton and a thin gold hairline reflection on the surface; the left two-thirds pure near-black for the offer and buttons. Camera: 85 mm, eye level, f/4. Calm, premium, final. No overlay text, no logos; pack faces clean.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/vtech-system.webp. Photoreal cinematic hero, 16:9, closing frame. The tall mirror-gold carton with thin black top and bottom bands stands on the right third on black lacquer, five amber vials with white caps and the flat gold-foil sachet in front, the set lit by a warm gold glow (#D4A853) behind the carton and a thin gold hairline reflection on the surface; the left two-thirds pure near-black for the offer and buttons. Camera: 85 mm, eye level, f/4. Calm, premium, final. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/vtech-system.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
@@ -51105,7 +51105,7 @@
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product hero, 16:9. A matte black landscape carton (wider than tall) standing on the right third on a black satin surface; in front of it five clear glass snap-neck ampoules with colourless liquid standing in a loose row, catching a warm gold edge light (#C9A24A). Background: matte black (#111111), a faint warm gold glow only behind the carton, no haze elsewhere. Lighting: warm key from the upper left, a cool white highlight along the ampoule necks. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds empty for text. No overlay text, no logos; pack faces clean so the real packshot PNG can be composited.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exosignal-hair.webp. Photoreal cinematic product hero, 16:9. A matte black landscape carton (wider than tall) standing on the right third on a black satin surface; in front of it five clear glass snap-neck ampoules with colourless liquid standing in a loose row, catching a warm gold edge light (#C9A24A). Background: matte black (#111111), a faint warm gold glow only behind the carton, no haze elsewhere. Lighting: warm key from the upper left, a cool white highlight along the ampoule necks. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds empty for text. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exosignal-hair.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
@@ -51405,7 +51405,7 @@
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>Photoreal counter scene, 16:9. On a black satin counter, left to right with space between: a white tablet-style screen on a white stand with a silver cylindrical base, the screen showing an abstract magnified scalp circle, with a corded white handheld scope camera resting in front of it; a slim cordless microneedling pen with a champagne-gold body, rose-gold grip ring and clear needle cartridge; a clear glass snap-neck ampoule standing in a small holder; and a small clear glass spray bottle with a tall gold cap at the far right. Lighting: thin warm gold rim light from above, soft fill, matte black background (#111111). Camera: 50 mm, slightly above eye level, f/8, all items sharp, the row centred with margins. No overlay text, no logos, screen content abstract, pack faces clean.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exosignal-hair.webp. Photoreal counter scene, 16:9. On a black satin counter, left to right with space between: a white tablet-style screen on a white stand with a silver cylindrical base, the screen showing an abstract magnified scalp circle, with a corded white handheld scope camera resting in front of it; a slim cordless microneedling pen with a champagne-gold body, rose-gold grip ring and clear needle cartridge; a clear glass snap-neck ampoule standing in a small holder; and a small clear glass spray bottle with a tall gold cap at the far right. Lighting: thin warm gold rim light from above, soft fill, matte black background (#111111). Camera: 50 mm, slightly above eye level, f/8, all items sharp, the row centred with margins. No overlay text or captions, no text other than the packaging's own printing, screen content abstract, the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exosignal-hair.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
@@ -51480,7 +51480,7 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Photoreal product shot, 16:9. The matte black landscape carton, closed, in three-quarter view on the left; in front of it five clear glass snap-neck ampoules with colourless liquid, four standing in a row and one lying on its side in front. Lighting: warm gold key from the upper right, cool highlight on the glass necks, matte black background, a soft gold glow behind the box only. Camera: 70 mm, f/5.6, right third empty for numbers. No overlay text, no logos; pack faces clean.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exosignal-hair.webp. Photoreal product shot, 16:9. The matte black landscape carton, closed, in three-quarter view on the left; in front of it five clear glass snap-neck ampoules with colourless liquid, four standing in a row and one lying on its side in front. Lighting: warm gold key from the upper right, cool highlight on the glass necks, matte black background, a soft gold glow behind the box only. Camera: 70 mm, f/5.6, right third empty for numbers. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exosignal-hair.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
@@ -51555,7 +51555,7 @@
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic closing hero, 16:9. The matte black landscape carton on the right third on black satin, five clear snap-neck ampoules lined up in front, a warm gold glow (#C9A24A) behind the box and a thin gold reflection line on the surface; the left two-thirds matte black for the offer and buttons. Camera: 85 mm, eye level, f/4. Quiet, premium, final. No overlay text, no logos; pack faces clean.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exosignal-hair.webp. Photoreal cinematic closing hero, 16:9. The matte black landscape carton on the right third on black satin, five clear snap-neck ampoules lined up in front, a warm gold glow (#C9A24A) behind the box and a thin gold reflection line on the surface; the left two-thirds matte black for the offer and buttons. Camera: 85 mm, eye level, f/4. Quiet, premium, final. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exosignal-hair.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr">
@@ -57405,7 +57405,7 @@
       </c>
       <c r="M93" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product hero, 16:9. A near-square carton, slightly wider than tall, finished in a champagne-gold gradient (pale warm ivory at the top left to deep gold at the right) standing on the right third on a warm cream stone surface; in front of it three vessels: a small amber glass vial with a silver cap, a small turquoise-blue glass vial with a silver cap, and a square clear glass bottle with a tall gold cap holding a pale liquid with fine gold flecks. Background: soft champagne (#F3E4C2) gradient, warm sunlight from the upper left, long soft shadows, subtle warm bloom. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds clear for text. No overlay text, no logos; pack faces clean so the real packshot PNG can be composited.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal cinematic product hero, 16:9. A near-square carton, slightly wider than tall, finished in a champagne-gold gradient (pale warm ivory at the top left to deep gold at the right) standing on the right third on a warm cream stone surface; in front of it three vessels: a small amber glass vial with a silver cap, a small turquoise-blue glass vial with a silver cap, and a square clear glass bottle with a tall gold cap holding a pale liquid with fine gold flecks. Background: soft champagne (#F3E4C2) gradient, warm sunlight from the upper left, long soft shadows, subtle warm bloom. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds clear for text. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N93" s="5" t="inlineStr">
@@ -57555,7 +57555,7 @@
       </c>
       <c r="M95" s="5" t="inlineStr">
         <is>
-          <t>Photoreal macro still life, 16:9. Three vessels in a row on warm cream stone under sunlight: left, a square clear glass bottle with a tall gold cap holding a pale liquid with fine gold flecks; centre, a small amber glass vial with a silver cap; right, a small turquoise-blue glass vial with a silver cap; behind each an out-of-focus macro swirl of its liquid — behind the bottle, a clear oily phase floating over a watery, fleck-filled phase. Lighting: warm champagne (#F3E4C2) backdrop, strong sun from the left, gold flecks sparkling. Camera: 100 mm macro, f/4, vessels sharp. No overlay text, no logos; pack faces clean.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal macro still life, 16:9. Three vessels in a row on warm cream stone under sunlight: left, a square clear glass bottle with a tall gold cap holding a pale liquid with fine gold flecks; centre, a small amber glass vial with a silver cap; right, a small turquoise-blue glass vial with a silver cap; behind each an out-of-focus macro swirl of its liquid — behind the bottle, a clear oily phase floating over a watery, fleck-filled phase. Lighting: warm champagne (#F3E4C2) backdrop, strong sun from the left, gold flecks sparkling. Camera: 100 mm macro, f/4, vessels sharp. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N95" s="5" t="inlineStr">
@@ -57705,7 +57705,7 @@
       </c>
       <c r="M97" s="5" t="inlineStr">
         <is>
-          <t>Photoreal top-down flat lay, 16:9. On warm cream stone, left to right in a straight row with space between: a square clear glass bottle with a tall gold cap and pale gold-flecked liquid, a fan brush, a small amber vial with a silver cap, a small turquoise vial with a silver cap, then a folded translucent pale-blue sheet mask lying in front of a small matte teal carton and a plain white unbranded sunscreen tube. Lighting: sunlight from the upper left, long soft shadows, champagne (#F3E4C2) tone. Camera: overhead, 50 mm, f/8, all sharp. No overlay text, no logos; pack faces clean.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal top-down flat lay, 16:9. On warm cream stone, left to right in a straight row with space between: a square clear glass bottle with a tall gold cap and pale gold-flecked liquid, a fan brush, a small amber vial with a silver cap, a small turquoise vial with a silver cap, then a folded translucent pale-blue sheet mask lying in front of a small matte teal carton and a plain white unbranded sunscreen tube. Lighting: sunlight from the upper left, long soft shadows, champagne (#F3E4C2) tone. Camera: overhead, 50 mm, f/8, all sharp. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N97" s="5" t="inlineStr">
@@ -57780,7 +57780,7 @@
       </c>
       <c r="M98" s="5" t="inlineStr">
         <is>
-          <t>Photoreal product shot, 16:9. The champagne-gold gradient near-square carton, closed, in three-quarter view on the left; beside it on cream stone, laid out neatly: one square clear glass bottle with a tall gold cap and gold-flecked liquid, a row of five small amber vials with silver caps and a row of five small turquoise-blue vials with silver caps. Lighting: warm sunlight from the upper right, soft champagne backdrop, gentle bloom. Camera: 70 mm, f/5.6, everything sharp, right third clear for numbers. No overlay text, no logos; pack faces clean.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal product shot, 16:9. The champagne-gold gradient near-square carton, closed, in three-quarter view on the left; beside it on cream stone, laid out neatly: one square clear glass bottle with a tall gold cap and gold-flecked liquid, a row of five small amber vials with silver caps and a row of five small turquoise-blue vials with silver caps. Lighting: warm sunlight from the upper right, soft champagne backdrop, gentle bloom. Camera: 70 mm, f/5.6, everything sharp, right third clear for numbers. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N98" s="5" t="inlineStr">
@@ -57855,7 +57855,7 @@
       </c>
       <c r="M99" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic closing hero, 16:9. The champagne-gold near-square carton on the right third on cream stone, the three vessels (small amber vial, small turquoise vial, square gold-capped bottle with gold-flecked liquid) in front, warm sunlight from the left, soft bloom, a thin gold reflection line; the left two-thirds clean champagne (#F3E4C2) for the offer and buttons. Camera: 85 mm, eye level, f/4. Warm, calm, final. No overlay text, no logos; pack faces clean.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal cinematic closing hero, 16:9. The champagne-gold near-square carton on the right third on cream stone, the three vessels (small amber vial, small turquoise vial, square gold-capped bottle with gold-flecked liquid) in front, warm sunlight from the left, soft bloom, a thin gold reflection line; the left two-thirds clean champagne (#F3E4C2) for the offer and buttons. Camera: 85 mm, eye level, f/4. Warm, calm, final. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N99" s="5" t="inlineStr">
@@ -57930,7 +57930,7 @@
       </c>
       <c r="M100" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product hero, 16:9. A matte teal (#6FAEB0) portrait-format rectangular carton standing on the right third on a wet pale-aqua stone surface; beside it, floating slightly above the surface, a translucent pale-blue bio-cellulose face mask with eye, nose and mouth cut-outs, folded in half along its vertical centre line so one eye cut-out and half the mouth cut-out show, tiny water droplets on its surface. Background: cool turquoise gradient (#DDF3F3 to #6FAEB0), soft cool key light from the upper left, a cool rim light on the mask edge, reflections in the wet surface. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds clear for text. No overlay text, no logos; pack faces clean so the real packshot PNG can be composited.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exocell-mask.webp. Photoreal cinematic product hero, 16:9. A matte teal (#6FAEB0) portrait-format rectangular carton standing on the right third on a wet pale-aqua stone surface; beside it, floating slightly above the surface, a translucent pale-blue bio-cellulose face mask with eye, nose and mouth cut-outs, folded in half along its vertical centre line so one eye cut-out and half the mouth cut-out show, tiny water droplets on its surface. Background: cool turquoise gradient (#DDF3F3 to #6FAEB0), soft cool key light from the upper left, a cool rim light on the mask edge, reflections in the wet surface. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds clear for text. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exocell-mask.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N100" s="5" t="inlineStr">
@@ -58305,7 +58305,7 @@
       </c>
       <c r="M105" s="5" t="inlineStr">
         <is>
-          <t>Photoreal product shot, 16:9. The matte teal portrait-format carton, closed, in three-quarter view on the left on wet pale-aqua stone; in front of it one unfolded translucent pale-blue bio-cellulose face mask with eye, nose and mouth cut-outs lying flat on the stone, droplets on its surface. Lighting: cool key from the upper right, turquoise gradient backdrop, reflections in the wet stone. Camera: 70 mm, f/5.6, all sharp, right third clear for numbers. No overlay text, no logos; pack face clean.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exocell-mask.webp. Photoreal product shot, 16:9. The matte teal portrait-format carton, closed, in three-quarter view on the left on wet pale-aqua stone; in front of it one unfolded translucent pale-blue bio-cellulose face mask with eye, nose and mouth cut-outs lying flat on the stone, droplets on its surface. Lighting: cool key from the upper right, turquoise gradient backdrop, reflections in the wet stone. Camera: 70 mm, f/5.6, all sharp, right third clear for numbers. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exocell-mask.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N105" s="5" t="inlineStr">
@@ -58380,7 +58380,7 @@
       </c>
       <c r="M106" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic closing hero, 16:9. The matte teal portrait-format carton on the right third on wet pale-aqua stone, the translucent pale-blue mask folded in half floating beside it as in the opening frame, cool key light, a thin cool reflection line on the surface; the left two-thirds clean pale aqua (#DDF3F3) for the offer and buttons. Camera: 85 mm, eye level, f/4. Cool, calm, final. No overlay text, no logos; pack faces clean.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exocell-mask.webp. Photoreal cinematic closing hero, 16:9. The matte teal portrait-format carton on the right third on wet pale-aqua stone, the translucent pale-blue mask folded in half floating beside it as in the opening frame, cool key light, a thin cool reflection line on the surface; the left two-thirds clean pale aqua (#DDF3F3) for the offer and buttons. Camera: 85 mm, eye level, f/4. Cool, calm, final. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exocell-mask.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
         </is>
       </c>
       <c r="N106" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Add the project council plan draft (pre-repair) and the Council sheet
Twelve role memos in four councils merged into seven phases, site changes,
a KPI tree and ten owner questions. The skeptic refuted it on 14 points;
a repair round follows and replaces this draft.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
+++ b/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Make prompt" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Storyboard" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Board" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Council" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -59505,4 +59506,1768 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Council</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Plan item</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Owner role</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Effort</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Спецификация «что после Contact for price»: канал, языки, кто отвечает, срок ответа, что отправляется</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · сейчас</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Решение по обучению (включено или нет, формат); «Training included» → «Training &amp; protocols from MITODERM»</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · сейчас</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Фильтр утверждений «публично / только для профи» и час регуляторного юриста</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · до масштабирования</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>S–M</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Запрос техлистов, срока годности, хранения и MOQ у VM и корейского производителя</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · запрос сейчас</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Построчная смета: фото контейнеров, перевод HE/RU и проверка RTL, перегенерации, часы на заявки</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Ф0</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Политика демо, пробной коробки и стартового комплекта</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>CEO (владелец)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Ф0</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Квалифицирующая форма и очереди по классу SKU (прибор / PRO-кит / домашний уход)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Директор B2B-продаж</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Журнал заявок (дата → ответ → КП → заказ → повтор) и общий дашборд для CEO, специалиста и финансов</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp-шаблон с продуктом и языком, лист ответов на HE/RU только формулировками каталога</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Директор B2B-продаж</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Kit &amp; facts как единица продажи без цены; убрать «one per professional session»</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Единые вторичные CTA и двойной CTA home care на всех 5 страницах</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Директор B2B-продаж</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Порядок волн по роли в выручке; EXOSIGNAL HAIR в волне 1 при условии подтверждения миксом продаж</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Home на четырёх протокольных связках с кнопкой «Enquire about the protocol»</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Директор B2B-продаж</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Цепочка касаний T0 / T+2 / T+7</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Директор B2B-продаж</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Ф4</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>«Where to buy» → «Ask your clinic», затем список партнёрских клиник с их согласием</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Директор B2B-продаж</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Ф3 → Ф5</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Лексикон бренда HE/EN/RU и чёрный список; чистка product-pages.json, .he.json, storyboard.md</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Контент и бренд</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · сейчас</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Решение о бюджете трафика и приоритетном сегменте на 8 недель</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Performance / growth</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Ф0</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Слой измерения: события по блокам, CTA «страница_блок_тип», UTM, скрытые поля, Meta Pixel / GA4</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Performance / growth</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Search Console и замер спроса по базовому списку запросов HE/EN/RU</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Отдельный URL на страницу и язык, SEO-head, JSON-LD, sitemap/robots</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Ф2 · до генерации</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Разделить пилот производства (EXOCELL) и пилот трафика (V-TECH, MICRO BOOST 10%, EXOSIGNAL HAIR + Home-роутер)</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Performance / growth</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>HE и RU для волны 1 и Home до платного трафика</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Контент и бренд</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Хаб Science текстом, PDF noindex, чипы как ссылки</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Правило лиц: только EXOCELL, EXOSIGNAL HAIR, MITOSCAN; на остальных руки, продукт и текстура</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Контент и бренд</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Ф3 · по итогам пилота</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Home care без платного трафика до появления адресата у «Where to buy»</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Performance / growth</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Ретаргет на 3 ключевых кадрах (холодная, тёплая, горячая аудитория)</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Performance / growth</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Ф4</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Слой доказательств Trust: факты каталога, цитаты клиник, пара MITOSCAN</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Контент и бренд</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Ф5 (сбор с Ф0)</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Соц-пакет для клиник 4:5 / 9:16 с подписями HE/RU — опция с апрувом</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Контент и бренд</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Ф5</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Таблица чисел с источником; закрыть конфликты каталога и PDF протоколов; один JSON для сайта и PDF</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Руководитель обучения</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · сейчас</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Реестр утверждений 15×7 с хеджами HE/RU и скриптом проверки</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Медицинский консультант</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · сейчас</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Семь заголовочных правок и кикер «Subject to professional assessment»</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Медицинский консультант</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Ф0</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Запрос пакета доказательств: INCI, аллергены PDRN, pH пилинга, данные под 72 h, срок годности, статус</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Медицинский консультант</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 запрос → Ф5 досье</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Чекбоксы практика в форме: расход, обучение, демо/образец, домашний уход для полки</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Ведущий косметолог</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Карточка протокола в блоке 4: Расход · Интервал · Курс · Финиш</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Ведущий косметолог</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Единая строка финиша и «mandatory» для DERMA RECOVERY на MICRO BOOST 10%</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Руководитель обучения</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Professional notice из трёх строк в блоке 5</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Медицинский консультант</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Правило изображений во всех промптах; исправить сцену нанесения EXOCELL до кадра 0</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Медицинский консультант</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Ф2 · до генерации</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Определение со стр. 5 на каждой экзосомной странице, термин по каталогу</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Медицинский консультант</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Offer «What comes with the kit»: карточки протоколов, обучение, линия специалиста</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Руководитель обучения</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Ф2 тексты → Ф3 публикация</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Строка «что почувствует клиентка» в блоке Feel it</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Ведущий косметолог</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Ссылка на PDF протоколов HE/RU/EN из блока 4 после сверки с каталогом</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Руководитель обучения</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Страница aftercare HE/RU/EN — только после подтверждения источника правил</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Руководитель обучения</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Ф5</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>S–M</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Онбординг: первая процедура с тренером, чек-ины через 72 ч (MICRO BOOST) и 2 недели (V-TECH), скрипт MITOSCAN</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Руководитель обучения</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Ф6</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Путь заявки: реальная отправка формы, wa.me с текстом, якоря #protocol / #kit и «Поделиться»</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Front-end lead</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Ф1 · до любого показа</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Аналитика по блокам и технические события (seq_first_frame_ms, seq_starved, reduced_motion, save_data)</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Front-end lead</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Оболочка сайта: мега-меню, мобильное меню, 7 точек прогресса, «Skip to kit &amp; price»</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>UX-лид</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Логика sticky-кнопки, CTA в шапке на десктопе, подписи над баром</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>UX-лид</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Загрузчик по manifest.json, удалить video.currentTime, исправить reduced-motion</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Front-end lead</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Бюджет веса и экспорт в tools/transitions.py: 40/30 кадров AVIF, hero &lt;img&gt;, Save-Data</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Front-end lead</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Правило RTL, &lt;bdi&gt;, тест-строки; HE-пилот на 3–5 носителях языка</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>UX-лид</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Ф2 · до кадра 0</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Пилот EXOCELL как тест конвейера: правка кадра 0, авто-привязка пакшота, стыки, журнал генераций</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Продюсер видео и кадров</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Ф2 · после апрува №2</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>S–M</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Home из готовых ассетов, без генерации</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>UX-лид</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Science — одна статичная страница; synthetic-exosomes и biospicule убрать из генерации</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>UX-лид</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Съёмка MITOPEN/MITOSCAN (36 кадров по кругу), первичной упаковки BIOSPICULE, EXOSIGNAL SPRAY; пакшоты ≥2000 px</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Продюсер видео и кадров</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Ф3 · до масштабирования</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Пакет 3+2 на 12 страниц, одна сцена на семейство, бюджет с перегенерациями</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Продюсер видео и кадров</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Ф3 → Ф5</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>A/B «кадры против смены стиллов» флагом в манифесте</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Front-end lead</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Ф4</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Роли на масштабе: оператор и листы вариантов, скрипт с лимитом бюджета, версия Kling на семейство</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Продюсер видео и кадров</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Ф5</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Rebuild the EXOCELL key frames on the client's real-use photos
The real sheet is milky-clear on skin with a pale-blue backing film, the
masks come in sealed aqua sachets, and a lighter second box version
exists. Prompts now copy the print from whichever box is attached, the
kit frame shows five sachets, the treatment frame follows the real
clinic application, and a mirror-with-sachet variant is added. Photos
with people stay local; only the box photo is committed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
+++ b/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Old pages (reference)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Make prompt" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Storyboard" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Board" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Council" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Council" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Board" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -58406,6 +58406,1770 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Council</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Plan item</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Owner role</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Effort</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Спецификация «что после Contact for price»: канал, языки, кто отвечает, срок ответа, что отправляется</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · сейчас</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Решение по обучению (включено или нет, формат); «Training included» → «Training &amp; protocols from MITODERM»</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · сейчас</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Фильтр утверждений «публично / только для профи» и час регуляторного юриста</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · до масштабирования</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>S–M</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Запрос техлистов, срока годности, хранения и MOQ у VM и корейского производителя</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · запрос сейчас</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Построчная смета: фото контейнеров, перевод HE/RU и проверка RTL, перегенерации, часы на заявки</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Ф0</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Политика демо, пробной коробки и стартового комплекта</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>CEO (владелец)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Ф0</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Квалифицирующая форма и очереди по классу SKU (прибор / PRO-кит / домашний уход)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Директор B2B-продаж</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Журнал заявок (дата → ответ → КП → заказ → повтор) и общий дашборд для CEO, специалиста и финансов</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp-шаблон с продуктом и языком, лист ответов на HE/RU только формулировками каталога</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Директор B2B-продаж</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Kit &amp; facts как единица продажи без цены; убрать «one per professional session»</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Единые вторичные CTA и двойной CTA home care на всех 5 страницах</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Директор B2B-продаж</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Порядок волн по роли в выручке; EXOSIGNAL HAIR в волне 1 при условии подтверждения миксом продаж</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Home на четырёх протокольных связках с кнопкой «Enquire about the protocol»</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Директор B2B-продаж</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Цепочка касаний T0 / T+2 / T+7</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Директор B2B-продаж</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Ф4</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Совет при CEO</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>«Where to buy» → «Ask your clinic», затем список партнёрских клиник с их согласием</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Директор B2B-продаж</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Ф3 → Ф5</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Лексикон бренда HE/EN/RU и чёрный список; чистка product-pages.json, .he.json, storyboard.md</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Контент и бренд</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · сейчас</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Решение о бюджете трафика и приоритетном сегменте на 8 недель</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Performance / growth</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Ф0</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Слой измерения: события по блокам, CTA «страница_блок_тип», UTM, скрытые поля, Meta Pixel / GA4</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Performance / growth</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Search Console и замер спроса по базовому списку запросов HE/EN/RU</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Отдельный URL на страницу и язык, SEO-head, JSON-LD, sitemap/robots</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Ф2 · до генерации</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Разделить пилот производства (EXOCELL) и пилот трафика (V-TECH, MICRO BOOST 10%, EXOSIGNAL HAIR + Home-роутер)</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Performance / growth</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>HE и RU для волны 1 и Home до платного трафика</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Контент и бренд</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Хаб Science текстом, PDF noindex, чипы как ссылки</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Правило лиц: только EXOCELL, EXOSIGNAL HAIR, MITOSCAN; на остальных руки, продукт и текстура</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Контент и бренд</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Ф3 · по итогам пилота</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Home care без платного трафика до появления адресата у «Where to buy»</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Performance / growth</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Ретаргет на 3 ключевых кадрах (холодная, тёплая, горячая аудитория)</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Performance / growth</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Ф4</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Слой доказательств Trust: факты каталога, цитаты клиник, пара MITOSCAN</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Контент и бренд</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Ф5 (сбор с Ф0)</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Совет при маркетологе</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Соц-пакет для клиник 4:5 / 9:16 с подписями HE/RU — опция с апрувом</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Контент и бренд</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Ф5</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Таблица чисел с источником; закрыть конфликты каталога и PDF протоколов; один JSON для сайта и PDF</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Руководитель обучения</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · сейчас</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Реестр утверждений 15×7 с хеджами HE/RU и скриптом проверки</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Медицинский консультант</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 · сейчас</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Семь заголовочных правок и кикер «Subject to professional assessment»</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Медицинский консультант</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Ф0</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Запрос пакета доказательств: INCI, аллергены PDRN, pH пилинга, данные под 72 h, срок годности, статус</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Медицинский консультант</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Ф0 запрос → Ф5 досье</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Чекбоксы практика в форме: расход, обучение, демо/образец, домашний уход для полки</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Ведущий косметолог</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Карточка протокола в блоке 4: Расход · Интервал · Курс · Финиш</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Ведущий косметолог</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Единая строка финиша и «mandatory» для DERMA RECOVERY на MICRO BOOST 10%</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Руководитель обучения</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Professional notice из трёх строк в блоке 5</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Медицинский консультант</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Правило изображений во всех промптах; исправить сцену нанесения EXOCELL до кадра 0</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Медицинский консультант</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Ф2 · до генерации</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Определение со стр. 5 на каждой экзосомной странице, термин по каталогу</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Медицинский консультант</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Offer «What comes with the kit»: карточки протоколов, обучение, линия специалиста</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Руководитель обучения</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Ф2 тексты → Ф3 публикация</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Строка «что почувствует клиентка» в блоке Feel it</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Ведущий косметолог</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Ссылка на PDF протоколов HE/RU/EN из блока 4 после сверки с каталогом</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Руководитель обучения</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Страница aftercare HE/RU/EN — только после подтверждения источника правил</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Руководитель обучения</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Ф5</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>S–M</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Клинический совет</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Онбординг: первая процедура с тренером, чек-ины через 72 ч (MICRO BOOST) и 2 недели (V-TECH), скрипт MITOSCAN</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Руководитель обучения</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Ф6</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Путь заявки: реальная отправка формы, wa.me с текстом, якоря #protocol / #kit и «Поделиться»</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Front-end lead</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Ф1 · до любого показа</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Аналитика по блокам и технические события (seq_first_frame_ms, seq_starved, reduced_motion, save_data)</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Front-end lead</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Ф1</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Оболочка сайта: мега-меню, мобильное меню, 7 точек прогресса, «Skip to kit &amp; price»</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>UX-лид</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Логика sticky-кнопки, CTA в шапке на десктопе, подписи над баром</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>UX-лид</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Загрузчик по manifest.json, удалить video.currentTime, исправить reduced-motion</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Front-end lead</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Бюджет веса и экспорт в tools/transitions.py: 40/30 кадров AVIF, hero &lt;img&gt;, Save-Data</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Front-end lead</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Ф2</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Правило RTL, &lt;bdi&gt;, тест-строки; HE-пилот на 3–5 носителях языка</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>UX-лид</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Ф2 · до кадра 0</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Пилот EXOCELL как тест конвейера: правка кадра 0, авто-привязка пакшота, стыки, журнал генераций</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Продюсер видео и кадров</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Ф2 · после апрува №2</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>S–M</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Home из готовых ассетов, без генерации</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>UX-лид</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Science — одна статичная страница; synthetic-exosomes и biospicule убрать из генерации</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>UX-лид</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Ф3</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Съёмка MITOPEN/MITOSCAN (36 кадров по кругу), первичной упаковки BIOSPICULE, EXOSIGNAL SPRAY; пакшоты ≥2000 px</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Продюсер видео и кадров</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Ф3 · до масштабирования</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Пакет 3+2 на 12 страниц, одна сцена на семейство, бюджет с перегенерациями</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Продюсер видео и кадров</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Ф3 → Ф5</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>A/B «кадры против смены стиллов» флагом в манифесте</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Front-end lead</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Ф4</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Совет дизайна и технологий</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Роли на масштабе: оператор и листы вариантов, скрипт с лимитом бюджета, версия Kling на семейство</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Продюсер видео и кадров</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Ф5</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -59506,1768 +61270,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F58"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Council</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>Plan item</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>Owner role</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="inlineStr">
-        <is>
-          <t>When</t>
-        </is>
-      </c>
-      <c r="E1" s="6" t="inlineStr">
-        <is>
-          <t>Effort</t>
-        </is>
-      </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>Impact</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Спецификация «что после Contact for price»: канал, языки, кто отвечает, срок ответа, что отправляется</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>COO</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Ф0 · сейчас</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Решение по обучению (включено или нет, формат); «Training included» → «Training &amp; protocols from MITODERM»</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>COO</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Ф0 · сейчас</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Фильтр утверждений «публично / только для профи» и час регуляторного юриста</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>COO</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Ф0 · до масштабирования</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>S–M</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Запрос техлистов, срока годности, хранения и MOQ у VM и корейского производителя</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>COO</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Ф0 · запрос сейчас</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Построчная смета: фото контейнеров, перевод HE/RU и проверка RTL, перегенерации, часы на заявки</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Ф0</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Политика демо, пробной коробки и стартового комплекта</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>CEO (владелец)</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Ф0</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Квалифицирующая форма и очереди по классу SKU (прибор / PRO-кит / домашний уход)</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Директор B2B-продаж</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Ф1</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Журнал заявок (дата → ответ → КП → заказ → повтор) и общий дашборд для CEO, специалиста и финансов</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Ф1</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>WhatsApp-шаблон с продуктом и языком, лист ответов на HE/RU только формулировками каталога</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Директор B2B-продаж</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Ф1</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Kit &amp; facts как единица продажи без цены; убрать «one per professional session»</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Ф2</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Единые вторичные CTA и двойной CTA home care на всех 5 страницах</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Директор B2B-продаж</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Ф2</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Порядок волн по роли в выручке; EXOSIGNAL HAIR в волне 1 при условии подтверждения миксом продаж</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Ф3</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Home на четырёх протокольных связках с кнопкой «Enquire about the protocol»</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Директор B2B-продаж</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Ф3</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Цепочка касаний T0 / T+2 / T+7</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Директор B2B-продаж</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Ф4</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Совет при CEO</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>«Where to buy» → «Ask your clinic», затем список партнёрских клиник с их согласием</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Директор B2B-продаж</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Ф3 → Ф5</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Лексикон бренда HE/EN/RU и чёрный список; чистка product-pages.json, .he.json, storyboard.md</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Контент и бренд</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Ф0 · сейчас</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Решение о бюджете трафика и приоритетном сегменте на 8 недель</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Performance / growth</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Ф0</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Слой измерения: события по блокам, CTA «страница_блок_тип», UTM, скрытые поля, Meta Pixel / GA4</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Performance / growth</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Ф1</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Search Console и замер спроса по базовому списку запросов HE/EN/RU</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>SEO</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Ф1</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Отдельный URL на страницу и язык, SEO-head, JSON-LD, sitemap/robots</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>SEO</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Ф2 · до генерации</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Разделить пилот производства (EXOCELL) и пилот трафика (V-TECH, MICRO BOOST 10%, EXOSIGNAL HAIR + Home-роутер)</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Performance / growth</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Ф3</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>HE и RU для волны 1 и Home до платного трафика</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Контент и бренд</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Ф3</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Хаб Science текстом, PDF noindex, чипы как ссылки</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>SEO</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Ф3</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Правило лиц: только EXOCELL, EXOSIGNAL HAIR, MITOSCAN; на остальных руки, продукт и текстура</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Контент и бренд</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Ф3 · по итогам пилота</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Home care без платного трафика до появления адресата у «Where to buy»</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Performance / growth</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Ф3</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Ретаргет на 3 ключевых кадрах (холодная, тёплая, горячая аудитория)</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Performance / growth</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Ф4</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Слой доказательств Trust: факты каталога, цитаты клиник, пара MITOSCAN</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Контент и бренд</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Ф5 (сбор с Ф0)</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Совет при маркетологе</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Соц-пакет для клиник 4:5 / 9:16 с подписями HE/RU — опция с апрувом</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Контент и бренд</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Ф5</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Таблица чисел с источником; закрыть конфликты каталога и PDF протоколов; один JSON для сайта и PDF</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Руководитель обучения</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Ф0 · сейчас</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>Реестр утверждений 15×7 с хеджами HE/RU и скриптом проверки</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Медицинский консультант</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Ф0 · сейчас</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Семь заголовочных правок и кикер «Subject to professional assessment»</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>Медицинский консультант</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Ф0</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Запрос пакета доказательств: INCI, аллергены PDRN, pH пилинга, данные под 72 h, срок годности, статус</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Медицинский консультант</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Ф0 запрос → Ф5 досье</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>Чекбоксы практика в форме: расход, обучение, демо/образец, домашний уход для полки</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>Ведущий косметолог</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Ф1</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Карточка протокола в блоке 4: Расход · Интервал · Курс · Финиш</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>Ведущий косметолог</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Ф2</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Единая строка финиша и «mandatory» для DERMA RECOVERY на MICRO BOOST 10%</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>Руководитель обучения</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Ф2</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Professional notice из трёх строк в блоке 5</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Медицинский консультант</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Ф2</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Правило изображений во всех промптах; исправить сцену нанесения EXOCELL до кадра 0</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>Медицинский консультант</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Ф2 · до генерации</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Определение со стр. 5 на каждой экзосомной странице, термин по каталогу</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>Медицинский консультант</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Ф2</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F39" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>Offer «What comes with the kit»: карточки протоколов, обучение, линия специалиста</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>Руководитель обучения</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Ф2 тексты → Ф3 публикация</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>Строка «что почувствует клиентка» в блоке Feel it</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>Ведущий косметолог</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Ф3</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>Ссылка на PDF протоколов HE/RU/EN из блока 4 после сверки с каталогом</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>Руководитель обучения</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Ф3</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>Страница aftercare HE/RU/EN — только после подтверждения источника правил</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>Руководитель обучения</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Ф5</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>S–M</t>
-        </is>
-      </c>
-      <c r="F43" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Клинический совет</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>Онбординг: первая процедура с тренером, чек-ины через 72 ч (MICRO BOOST) и 2 недели (V-TECH), скрипт MITOSCAN</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Руководитель обучения</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Ф6</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>Путь заявки: реальная отправка формы, wa.me с текстом, якоря #protocol / #kit и «Поделиться»</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>Front-end lead</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Ф1 · до любого показа</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F45" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>Аналитика по блокам и технические события (seq_first_frame_ms, seq_starved, reduced_motion, save_data)</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>Front-end lead</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Ф1</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F46" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Оболочка сайта: мега-меню, мобильное меню, 7 точек прогресса, «Skip to kit &amp; price»</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>UX-лид</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Ф2</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F47" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Логика sticky-кнопки, CTA в шапке на десктопе, подписи над баром</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>UX-лид</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Ф2</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Загрузчик по manifest.json, удалить video.currentTime, исправить reduced-motion</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>Front-end lead</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Ф2</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F49" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Бюджет веса и экспорт в tools/transitions.py: 40/30 кадров AVIF, hero &lt;img&gt;, Save-Data</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Front-end lead</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Ф2</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>Правило RTL, &lt;bdi&gt;, тест-строки; HE-пилот на 3–5 носителях языка</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>UX-лид</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Ф2 · до кадра 0</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>Пилот EXOCELL как тест конвейера: правка кадра 0, авто-привязка пакшота, стыки, журнал генераций</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>Продюсер видео и кадров</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Ф2 · после апрува №2</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>S–M</t>
-        </is>
-      </c>
-      <c r="F52" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>Home из готовых ассетов, без генерации</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>UX-лид</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Ф3</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F53" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>Science — одна статичная страница; synthetic-exosomes и biospicule убрать из генерации</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>UX-лид</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Ф3</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F54" s="5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Съёмка MITOPEN/MITOSCAN (36 кадров по кругу), первичной упаковки BIOSPICULE, EXOSIGNAL SPRAY; пакшоты ≥2000 px</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>Продюсер видео и кадров</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Ф3 · до масштабирования</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F55" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>Пакет 3+2 на 12 страниц, одна сцена на семейство, бюджет с перегенерациями</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>Продюсер видео и кадров</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Ф3 → Ф5</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F56" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>A/B «кадры против смены стиллов» флагом в манифесте</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>Front-end lead</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Ф4</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F57" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
-        <is>
-          <t>Совет дизайна и технологий</t>
-        </is>
-      </c>
-      <c r="B58" s="5" t="inlineStr">
-        <is>
-          <t>Роли на масштабе: оператор и листы вариантов, скрипт с лимитом бюджета, версия Kling на семейство</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>Продюсер видео и кадров</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Ф5</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F58" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix two garbled phrases in the EXOCELL sachet prompts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
+++ b/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
@@ -61028,7 +61028,7 @@
       </c>
       <c r="M103" s="5" t="inlineStr">
         <is>
-          <t>Branch B. REFERENCE IMAGES: attach the EXOCELL MASK box photo and the treatment photos. Copy the carton exactly from the attached box photo: its colour, the VM monogram with 'VM corporation', the 'EXOCELL' wordmark ('EXO' bold, 'CELL' thin) with letter-spaced 'MASK' beneath, and the small multilingual text block near the bottom — every word spelled exactly as on that box, crisp and legible; add no line that is not on the reference. Photoreal cinematic treatment scene, 16:9, 4K, the same teal light as the hero. A woman in her thirties reclines on a treatment bed, eyes closed, calm, hair under a black disposable cap; a bio-cellulose sheet mask lies smoothly on her face — on skin it turns almost clear and milky, eye and mouth cut-outs sitting precisely, minimal air pockets, a few droplets; a practitioner's hands in black nitrile gloves peel the pale-blue protective backing film away from the mask at the forehead. In the right third, on a black glass side table at shoulder height, the EXOCELL MASK carton, about 35% of the frame height, turned 20 degrees to show its left side panel. CAMERA: 50 mm, slightly above, f/4, face, sheet and carton sharp; the left third darker for text. Realistic skin texture, no redness, no retouched plastic skin. No captions or overlay text, no text other than the packaging's own print, no purple, no extra people.  ||  Branch B alternative (mirror with sachet): REFERENCE IMAGES: attach the sachet photo and the mirror photo. Photoreal portrait, 16:9, 4K, minimal clinic washroom with black walls and the same soft teal light. A woman in her thirties, dark hair pulled back, freshly treated calm skin, faces the camera as if it were her mirror and holds one sealed single-mask sachet copied exactly from the attached sachet photo: pale-aqua foil, the VM monogram and 'EXOCELL MASK' printed on the front at shoulder height on the right, front of the sachet toward the camera and readable. CAMERA: 50 mm, f/2.8, face and sachet sharp; left half dark for text. No captions or overlay text, no text other than the packaging's own print, no mirror frame, no extra objects.</t>
+          <t>Branch B. REFERENCE IMAGES: attach the EXOCELL MASK box photo and the treatment photos. Copy the carton exactly from the attached box photo: its colour, the VM monogram with 'VM corporation', the 'EXOCELL' wordmark ('EXO' bold, 'CELL' thin) with letter-spaced 'MASK' beneath, and the small multilingual text block near the bottom — every word spelled exactly as on that box, crisp and legible; add no line that is not on the reference. Photoreal cinematic treatment scene, 16:9, 4K, the same teal light as the hero. A woman in her thirties reclines on a treatment bed, eyes closed, calm, hair under a black disposable cap; a bio-cellulose sheet mask lies smoothly on her face — on skin it turns almost clear and milky, eye and mouth cut-outs sitting precisely, minimal air pockets, a few droplets; a practitioner's hands in black nitrile gloves peel the pale-blue protective backing film away from the mask at the forehead. In the right third, on a black glass side table at shoulder height, the EXOCELL MASK carton, about 35% of the frame height, turned 20 degrees to show its left side panel. CAMERA: 50 mm, slightly above, f/4, face, sheet and carton sharp; the left third darker for text. Realistic skin texture, no redness, no retouched plastic skin. No captions or overlay text, no text other than the packaging's own print, no purple, no extra people.  ||  Branch B alternative (mirror with sachet): REFERENCE IMAGES: attach the sachet photo and the mirror photo. Photoreal portrait, 16:9, 4K, minimal clinic washroom with black walls and the same soft teal light. A woman in her thirties, dark hair pulled back, freshly treated calm skin, faces the camera as if it were her mirror and holds one sealed single-mask sachet at shoulder height on the right, its front toward the camera and readable; the sachet is copied exactly from the attached sachet photo (pale-aqua foil with the VM monogram and 'EXOCELL MASK' printed on the front). CAMERA: 50 mm, f/2.8, face and sachet sharp; left half dark for text. No captions or overlay text, no text other than the packaging's own print, no mirror frame, no extra objects.</t>
         </is>
       </c>
       <c r="N103" s="5" t="inlineStr">
@@ -61178,7 +61178,7 @@
       </c>
       <c r="M105" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGES: attach the EXOCELL MASK box photo and the sachet photo. Copy the carton exactly from the attached box photo: its colour, the VM monogram with 'VM corporation', the 'EXOCELL' wordmark ('EXO' bold, 'CELL' thin) with letter-spaced 'MASK' beneath, and the small multilingual text block near the bottom — every word spelled exactly as on that box, crisp and legible; add no line that is not on the reference. Photoreal product still life, 16:9, 4K — the same black glass set and teal light as the hero, camera raised about 20 degrees above the counter. The carton stands in the right third at the same scale as the hero (about 45% of the frame height), turned 20 degrees to show its left side panel; in front of it, five sealed single-mask sachets copied exactly from the attached sachet photo: pale-aqua foil, the VM monogram and 'EXOCELL MASK' printed on the front fan out across the glass, the front one slightly lifted; droplets on the glass. Left half empty near-black for numbers. No people, no hands. No captions or overlay text, no text other than the packaging's own print, no extra objects.</t>
+          <t>REFERENCE IMAGES: attach the EXOCELL MASK box photo and the sachet photo. Copy the carton exactly from the attached box photo: its colour, the VM monogram with 'VM corporation', the 'EXOCELL' wordmark ('EXO' bold, 'CELL' thin) with letter-spaced 'MASK' beneath, and the small multilingual text block near the bottom — every word spelled exactly as on that box, crisp and legible; add no line that is not on the reference. Photoreal product still life, 16:9, 4K — the same black glass set and teal light as the hero, camera raised about 20 degrees above the counter. The carton stands in the right third at the same scale as the hero (about 45% of the frame height), turned 20 degrees to show its left side panel; in front of it, five sealed single-mask sachets fan out across the glass, the front one slightly lifted; the sachets are copied exactly from the attached sachet photo (pale-aqua foil with the VM monogram and 'EXOCELL MASK' printed on the front); droplets on the glass. Left half empty near-black for numbers. No people, no hands. No captions or overlay text, no text other than the packaging's own print, no extra objects.</t>
         </is>
       </c>
       <c r="N105" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Generate the EXOCELL pilot frames with the real packaging text
Transcribed every product's packaging print into packaging-text.json and
injected it into all prompts that show a product. With that list GPT
Image 2 renders the EXOCELL carton correctly; four frames (hero, wet
sheet, treatment, kit with sachets) now replace the prototype
placeholders. The hero frame is the desktop hero visual; the still
crossfade is narrowed so the carton never doubles. Adds the proven
prompts and a compositor for the real packshot as a fallback.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
+++ b/mitoderm-catalog/site/mitoderm-site-blocks.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Old pages (reference)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Make prompt" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Council" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Board" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Storyboard" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Storyboard" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Board" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -52187,1114 +52187,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="70" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="inlineStr">
-        <is>
-          <t>Purchase</t>
-        </is>
-      </c>
-      <c r="E1" s="6" t="inlineStr">
-        <is>
-          <t>Truth</t>
-        </is>
-      </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>Brevity</t>
-        </is>
-      </c>
-      <c r="G1" s="6" t="inlineStr">
-        <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="H1" s="6" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-      <c r="I1" s="6" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Meet</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Клиент — косметолог</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E2" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F2" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G2" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>keep</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>Хедер работает: продукт, «вторая кожа», «после процедуры» прослеживаются к спеке и стр. 10. Натяжка — чип «Instant cooling» (в каталоге immediate — про гидратацию, cooling отдельно); сложенная пополам маска — выдуманный элемент, биоцеллюлоза должна читаться как реальный лист.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Meet</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Главный редактор</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G3" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>Строка повторяет eyebrow и hero_sub, чипы повторяют строку — три слоя одного в одном экране. «After every professional treatment» шире каталога (стр. 10: «after professional cosmetic treatments»). Сложенная маска придумана — спорит с реальным пакшотом, где лист раскрыт.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Meet</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>CEO MITODERM</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>«Your second skin» пишет каждая биоцеллюлозная маска на рынке; наш единственный дифференциатор — синтетические экзосомальные структуры VM — задвинут в чип. «After every» — переобещание, каталог говорит «after professional cosmetic treatments».</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Meet</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Маркетинг и конверсия</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Позиционирование и primary CTA на месте, но H1 без имени продукта и без ключа «bio-cellulose mask» — пусто для SEO; имя EXOCELL MASK впервые появляется в последнем блоке. «Every» — усиление спеки. Сложенная маска — осознанно выдуманный элемент, допустимо ради переходов.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Клиент — косметолог</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>Чипы «After V-TECH / EXO-NAD / MICRO BOOST / microneedling» — ровно то, что я проверяю перед заказом, и они прослеживаются (стр. 7, 9, 19). Но покрасневшее лицо с точечными следами на странице про успокоение — риск; маска, висящая в воздухе у лица, странна; «decides how your client walks out» — продающая отсебятина.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Главный редактор</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Слово «after» шесть раз в блоке; второе предложение — риторика, в каталоге нет; чипы дублируют ряд блока 4. Кадр — медицинская иллюстрация, не продукт-герой. Делать типографикой на бирюзе, чипы = ссылки, без генерации.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>CEO MITODERM</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>Четыре чипа — самое сильное B2B-место страницы (маска продаётся как завершение наших же протоколов), но вторая фраза ничем не подтверждена, а румянец и «pinpoint marks» на генеративном лице рискуют выглядеть как осложнение. Уместнее три реальных пакшота протоколов и лист маски.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Маркетинг и конверсия</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>Текст говорит с владельцем клиники на его языке, чипы — правильный внутренний граф ссылок на PRO-страницы. Кадр — самый рискованный на странице (медицина / uncanny valley), продукта в кадре фактически нет. Фраза про «walks out» — риторика, не свойство.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Inside</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Клиент — косметолог</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>Состав честный (все 8 ингредиентов из стр. 10) и это то, что я реально читаю, но строка — перечисление, чипы 3 и 4 составные; «сфера-везикула среди волокон» — клише, которому профессионал не верит; единственный кадр без продукта. Концентраций нет — спрошу у поставщика.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Inside</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Главный редактор</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Состав перечислен трижды (строка, четыре составных чипа, подпись); «adheres with minimal air pockets» повторяется в блоке 4; «soaked» — не из источников (там «active serum»). «Везикула» в макро — псевдонаука. Текстуру дать кропом реального пакшота.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Inside</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>CEO MITODERM</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>Текст дословно из каталога, но блок перегружен; «увеличенная везикула» — научная неточность, которую заметит любой врач: наноразмерные структуры не видны рядом с волокнами целлюлозы. У бренда «where science meets beauty» такого кадра быть не должно.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Inside</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Маркетинг и конверсия</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>Каждое слово из стр. 10 — плюс, но это стена из 14 ингредиентов, здесь владелец клиники начнёт пролистывать; «Full formula ↓» никуда не ведёт. Оставить два дифференциатора (экзосомы, полинуклеотиды), остальное — в раскрывающийся список. Макро без лиц — снимаемый кадр.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Feel it</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Клиент — косметолог</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>Каждое слово из каталога, но семь прилагательных через запятую дублируют четыре чипа, чипы дублируют хедер; ничто не двигает к заказу. Пин «Smoothing &amp; firming» на шее намекает на шею, чего в каталоге нет. Кадр с маской на лице — лучший на странице, оставить.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Feel it</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Главный редактор</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>Строка — весь абзац Key Benefits через точку с запятой и дублирует чипы и заголовок; одна фраза должна остаться одной. Пины держать на лице — каталог шею не упоминает. Единственный кадр с человеком — оставить: маска на лице = продукт на коже.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Feel it</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>CEO MITODERM</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>Эмоциональная вершина страницы и всё по каталогу, но фраза перечисляет семь прилагательных — список, не фраза. В кадре маска «turned nearly invisible» — продукт должен читаться: края, вырезы, голубой оттенок, капли.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Feel it</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Маркетинг и конверсия</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G17" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>Эмоциональный пик и лучший кадр, все слова из каталога. Но четыре клаузы и четыре лейбла повторяют друг друга. На десктопе на пике убеждения нет ни одной кнопки — добавить secondary «Contact for price». Нужен видимый влажный край листа, иначе продукт исчезает из кадра.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Protocol</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Клиент — косметолог</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>Главный блок для косметолога — без времени экспозиции («сколько держать?» — первый вопрос, в каталоге ответа нет); шаг «Remove» обрывается, хотя каталог на стр. 7, 9, 19 даёт финиш EXOCELL → DERMA RECOVERY → солнцезащита. Триптих одной женщины в одном 16:9 генератор держит плохо.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Protocol</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Главный редактор</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>Строка повторяет блок 2 и блок 3; лейбл 2 — предложение, а не ярлык; «Works with» дублирует чипы блока 1. Триптих в одном 16:9 не сгенерируется стабильно, луп капель — лишняя генерация. Одна сцена (маска снята), три шага — типографикой.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Protocol</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>CEO MITODERM</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>Ключевой блок для владельца клиники (как встроить в рабочий процесс), но без времени экспозиции пуст — каталог его не даёт, нужен ответ редактора, не выдумка. Чипы длинные, четвёртый — предложение; триптих с одной женщиной в трёх позах — зона риска по консистентности.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Protocol</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Маркетинг и конверсия</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F21" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G21" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>Самый перегруженный блок: строка из 3 клауз + 4 лейбла + ряд чипов «Works with» + CTA + триптих + луп. Триптих — худшее задание для генератора (разные лица в панелях). «Cleansed skin» есть только в спеке, не в каталоге.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Kit &amp; facts</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Клиент — косметолог</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E22" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F22" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G22" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>«Факты» без фактов: два чипа из четырёх повторяют хедер; нет того, что нужно для заказа — объёма (на коробке 5 × 25 ml, в каталоге нет), хранения, «professional use only»; «one per client» логично, но не написано в источниках. Одноразовая маска на мокром камне читается негигиенично.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Kit &amp; facts</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Главный редактор</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E23" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F23" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G23" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>«One per client» и «one finishing step per protocol» — выводы, не факты; «single-use» есть лишь в спеке; чипы «Bio-cellulose» и «Post-procedure finish» повторяют блок 0. Фактов для закупщика (объём, срок, хранение) нет. Кадр — лучший продуктовый still life страницы, годится как hero и финал.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Kit &amp; facts</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>CEO MITODERM</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E24" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F24" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G24" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>«5 masks per box» — главный B2B-факт (пять клиентов, расчёт себестоимости процедуры), но два чипа из четырёх дословно повторяют блок 0 и место пропадает; сюда просятся «For professional use only» и показания — то, что владелец клиники проверяет перед заказом.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Kit &amp; facts</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Маркетинг и конверсия</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F25" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G25" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>merge</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>Единственный факт для unit-экономики нужен, но блок назван «trust» и доверия не несёт: лейблы повторяют блок 0, «one per client» — вывод, «single-use» только в спеке. Кадр почти дублирует hero, реальный пакшот уже показывает раскрытую маску. Слить в Offer — минус кадр и переход.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Offer</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Клиент — косметолог</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E26" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F26" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G26" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>Всё прослеживается (training — стр. 3, exclusive VM importer — стр. 5); «Add to a V-TECH / EXO-NAD enquiry» — именно так я буду заказывать. Но три уровня CTA + контакты + четыре чипа + логотип — перегруз; «VM» без «Italy» косметологу ничего не говорит; кадр — зеркало блока 0, генерировать не нужно.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Offer</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Главный редактор</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E27" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F27" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G27" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>Строка почти дословно повторяет блок 0 («the soothing finishing step … every …»); «Contact for price» дублирует кнопку, «Finishes every advanced protocol» дублирует строку — живых лейблов два; четыре CTA в блоке «одна фраза». Отдельная генерация не нужна — кадр блока 5.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Offer</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>CEO MITODERM</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E28" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F28" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G28" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>Структура оффера верная для B2B (контакт за ценой, обучение, эксклюзивный импортёр VM), но чип «Contact for price» дублирует кнопку, «every» — переобещание, а главный коммерческий ход «Add to a V-TECH / EXO-NAD enquiry» спрятан во вторую кнопку, хотя маска по каталогу — довесок к этим протоколам.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Offer</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Маркетинг и конверсия</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E29" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F29" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G29" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>rewrite</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>Механика правильная: WhatsApp + форма, вторичный CTA «добавить к запросу» — лучший кросс-селл. Но половина лейблов потрачена впустую (дубли кнопки и строки). Зеркало блока 0 — бесплатный кадр; idle-луп делать CSS. «For professional use only» в каталоге стоит на странице V-TECH, не EXOCELL.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:O106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -53453,7 +52345,7 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/vtech-system.webp. Photoreal cinematic product hero, 16:9. A tall rectangular carton wrapped in mirror-polished gold foil with a thin black band at the top and bottom edges, standing upright on the right third of the frame on a black lacquered surface; in front of it five small amber-brown glass vials with white plastic caps and one flat gold-foil sachet. Background: near-black (#0E0C0A) studio with a soft warm gold glow (#D4A853) only behind the carton and faint gold specks in the air. Lighting: single warm key from the upper left, gold rim light on the carton edges, reflections of the vials in the surface. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds empty for text. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/vtech-system.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/vtech-system.webp. Photoreal cinematic product hero, 16:9. A tall rectangular carton wrapped in mirror-polished gold foil with a thin black band at the top and bottom edges, standing upright on the right third of the frame on a black lacquered surface; in front of it five small amber-brown glass vials with white plastic caps and one flat gold-foil sachet. Background: near-black (#0E0C0A) studio with a soft warm gold glow (#D4A853) only behind the carton and faint gold specks in the air. Lighting: single warm key from the upper left, gold rim light on the carton edges, reflections of the vials in the surface. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds empty for text. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/vtech-system.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL CARTON — mirror-polished gold foil, black bands at top and bottom: top: 'VM' in silver letters; centre: a large black 'V' with a small inverted black triangle above it; lower third: 'V-TECH' letter-spaced (the V drawn as the same V-with-triangle mark), below it letter-spaced 'S Y S T E M' || 5 VIALS — amber glass vials with white flip-off caps, amber label: white V-with-triangle mark; 'V-TECH'; [unreadable] one tiny line under 'V-TECH'; white graduation ticks on the side || GEL MASK SACHET — gold foil sachet with a small white nozzle cap on the left: large black V-with-triangle mark; 'V-TECH' letter-spaced, below it 'G E L   M A S K'; [unreadable] four tiny lines at the bottom.</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
@@ -53528,7 +52420,7 @@
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic close-up, 16:9. A gloved practitioner's hand holds a slim cordless microneedling pen — champagne-gold body, rose-gold grip ring, clear needle cartridge at the tip — just above a woman's cheek; macro view of skin texture with faint dots of temporary micro-channels catching warm light. The woman's face is in soft focus, eyes closed, relaxed. Environment: dark treatment room in black and deep bronze tones, a thin warm gold edge light along the jawline. Camera: 100 mm macro, f/2.8, focus on the pen tip and the skin, the image occupies the left two-thirds and the right third falls to near-black for text. Mood: precise, clinical, luxurious. No overlay text, no logos.</t>
+          <t>Photoreal cinematic close-up, 16:9. A gloved practitioner's hand holds a slim cordless microneedling pen — champagne-gold body, rose-gold grip ring, clear needle cartridge at the tip — just above a woman's cheek; macro view of skin texture with faint dots of temporary micro-channels catching warm light. The woman's face is in soft focus, eyes closed, relaxed. Environment: dark treatment room in black and deep bronze tones, a thin warm gold edge light along the jawline. Camera: 100 mm macro, f/2.8, focus on the pen tip and the skin, the image occupies the left two-thirds and the right third falls to near-black for text. Mood: precise, clinical, luxurious. No overlay text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL CARTON — mirror-polished gold foil, black bands at top and bottom: top: 'VM' in silver letters; centre: a large black 'V' with a small inverted black triangle above it; lower third: 'V-TECH' letter-spaced (the V drawn as the same V-with-triangle mark), below it letter-spaced 'S Y S T E M' || 5 VIALS — amber glass vials with white flip-off caps, amber label: white V-with-triangle mark; 'V-TECH'; [unreadable] one tiny line under 'V-TECH'; white graduation ticks on the side || GEL MASK SACHET — gold foil sachet with a small white nozzle cap on the left: large black V-with-triangle mark; 'V-TECH' letter-spaced, below it 'G E L   M A S K'; [unreadable] four tiny lines at the bottom.</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
@@ -53603,7 +52495,7 @@
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>Photoreal macro, 16:9. An open amber glass vial with its white cap beside it, lying on black slate on the left, a single golden drop suspended at its mouth; centre-right an enlarged translucent golden sphere (an engineered vesicle) floating in dark liquid, its shell catching light, soft strands and particles glowing inside it. Lighting: dark background (#0E0C0A), warm gold backlight (#E8C87E) through the sphere, cool highlights on the glass. Camera: 100 mm macro, f/4, sphere sharp, vial slightly soft. Scientific but warm. No overlay text, no logos, no labels.</t>
+          <t>Photoreal macro, 16:9. An open amber glass vial with its white cap beside it, lying on black slate on the left, a single golden drop suspended at its mouth; centre-right an enlarged translucent golden sphere (an engineered vesicle) floating in dark liquid, its shell catching light, soft strands and particles glowing inside it. Lighting: dark background (#0E0C0A), warm gold backlight (#E8C87E) through the sphere, cool highlights on the glass. Camera: 100 mm macro, f/4, sphere sharp, vial slightly soft. Scientific but warm. No overlay text, no logos, no labels. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL CARTON — mirror-polished gold foil, black bands at top and bottom: top: 'VM' in silver letters; centre: a large black 'V' with a small inverted black triangle above it; lower third: 'V-TECH' letter-spaced (the V drawn as the same V-with-triangle mark), below it letter-spaced 'S Y S T E M' || 5 VIALS — amber glass vials with white flip-off caps, amber label: white V-with-triangle mark; 'V-TECH'; [unreadable] one tiny line under 'V-TECH'; white graduation ticks on the side || GEL MASK SACHET — gold foil sachet with a small white nozzle cap on the left: large black V-with-triangle mark; 'V-TECH' letter-spaced, below it 'G E L   M A S K'; [unreadable] four tiny lines at the bottom.</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
@@ -53678,7 +52570,7 @@
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic portrait, 16:9. A woman in her forties sits in a treatment chair facing the camera as if looking into a mirror, skin slightly flushed and dewy after microneedling; a practitioner's gloved hands press a clear golden gel from a flat gold-foil sachet onto her cheek. Her eyes meet the lens, calm. Environment: dark clinic room with black walls, a warm gold key light from the front-left and a soft gold rim; a hint of the tall gold carton on a shelf behind, out of focus. Camera: 85 mm, f/2, eye level, the woman in the left two-thirds, the right third darker for text. No overlay text, no logos.</t>
+          <t>Photoreal cinematic portrait, 16:9. A woman in her forties sits in a treatment chair facing the camera as if looking into a mirror, skin slightly flushed and dewy after microneedling; a practitioner's gloved hands press a clear golden gel from a flat gold-foil sachet onto her cheek. Her eyes meet the lens, calm. Environment: dark clinic room with black walls, a warm gold key light from the front-left and a soft gold rim; a hint of the tall gold carton on a shelf behind, out of focus. Camera: 85 mm, f/2, eye level, the woman in the left two-thirds, the right third darker for text. No overlay text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL CARTON — mirror-polished gold foil, black bands at top and bottom: top: 'VM' in silver letters; centre: a large black 'V' with a small inverted black triangle above it; lower third: 'V-TECH' letter-spaced (the V drawn as the same V-with-triangle mark), below it letter-spaced 'S Y S T E M' || 5 VIALS — amber glass vials with white flip-off caps, amber label: white V-with-triangle mark; 'V-TECH'; [unreadable] one tiny line under 'V-TECH'; white graduation ticks on the side || GEL MASK SACHET — gold foil sachet with a small white nozzle cap on the left: large black V-with-triangle mark; 'V-TECH' letter-spaced, below it 'G E L   M A S K'; [unreadable] four tiny lines at the bottom.</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
@@ -53753,7 +52645,7 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/vtech-system.webp. Photoreal top-down flat lay, 16:9. On matte black slate, left to right: a slim cordless microneedling pen with a champagne-gold body, rose-gold grip ring and clear needle cartridge; an amber glass vial with a white cap; a flat gold-foil sachet; a folded translucent pale-blue bio-cellulose sheet mask lying in front of a small matte teal carton; and a plain white unbranded sunscreen tube. Items in one straight row with generous black space between them for step numbers. Lighting: a thin warm gold rim light from the top, soft fill, long soft shadows. Camera: directly overhead, 50 mm, f/8, everything sharp. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/vtech-system.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/vtech-system.webp. Photoreal top-down flat lay, 16:9. On matte black slate, left to right: a slim cordless microneedling pen with a champagne-gold body, rose-gold grip ring and clear needle cartridge; an amber glass vial with a white cap; a flat gold-foil sachet; a folded translucent pale-blue bio-cellulose sheet mask lying in front of a small matte teal carton; and a plain white unbranded sunscreen tube. Items in one straight row with generous black space between them for step numbers. Lighting: a thin warm gold rim light from the top, soft fill, long soft shadows. Camera: directly overhead, 50 mm, f/8, everything sharp. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/vtech-system.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL CARTON — mirror-polished gold foil, black bands at top and bottom: top: 'VM' in silver letters; centre: a large black 'V' with a small inverted black triangle above it; lower third: 'V-TECH' letter-spaced (the V drawn as the same V-with-triangle mark), below it letter-spaced 'S Y S T E M' || 5 VIALS — amber glass vials with white flip-off caps, amber label: white V-with-triangle mark; 'V-TECH'; [unreadable] one tiny line under 'V-TECH'; white graduation ticks on the side || GEL MASK SACHET — gold foil sachet with a small white nozzle cap on the left: large black V-with-triangle mark; 'V-TECH' letter-spaced, below it 'G E L   M A S K'; [unreadable] four tiny lines at the bottom.</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
@@ -53828,7 +52720,7 @@
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/vtech-system.webp. Photoreal product shot, 16:9. The tall mirror-gold carton with thin black top and bottom bands, closed, standing in three-quarter view on the left; beside it on black lacquer, neatly in two rows: five amber glass vials with white caps and five flat gold-foil sachets. Lighting: warm gold key from the upper right, black background (#0E0C0A), soft gold glow behind the carton only, crisp reflections in the surface. Camera: 70 mm, slightly above eye level, f/5.6, all items sharp, right third empty for numbers. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/vtech-system.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/vtech-system.webp. Photoreal product shot, 16:9. The tall mirror-gold carton with thin black top and bottom bands, closed, standing in three-quarter view on the left; beside it on black lacquer, neatly in two rows: five amber glass vials with white caps and five flat gold-foil sachets. Lighting: warm gold key from the upper right, black background (#0E0C0A), soft gold glow behind the carton only, crisp reflections in the surface. Camera: 70 mm, slightly above eye level, f/5.6, all items sharp, right third empty for numbers. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/vtech-system.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL CARTON — mirror-polished gold foil, black bands at top and bottom: top: 'VM' in silver letters; centre: a large black 'V' with a small inverted black triangle above it; lower third: 'V-TECH' letter-spaced (the V drawn as the same V-with-triangle mark), below it letter-spaced 'S Y S T E M' || 5 VIALS — amber glass vials with white flip-off caps, amber label: white V-with-triangle mark; 'V-TECH'; [unreadable] one tiny line under 'V-TECH'; white graduation ticks on the side || GEL MASK SACHET — gold foil sachet with a small white nozzle cap on the left: large black V-with-triangle mark; 'V-TECH' letter-spaced, below it 'G E L   M A S K'; [unreadable] four tiny lines at the bottom.</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
@@ -53903,7 +52795,7 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/vtech-system.webp. Photoreal cinematic hero, 16:9, closing frame. The tall mirror-gold carton with thin black top and bottom bands stands on the right third on black lacquer, five amber vials with white caps and the flat gold-foil sachet in front, the set lit by a warm gold glow (#D4A853) behind the carton and a thin gold hairline reflection on the surface; the left two-thirds pure near-black for the offer and buttons. Camera: 85 mm, eye level, f/4. Calm, premium, final. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/vtech-system.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/vtech-system.webp. Photoreal cinematic hero, 16:9, closing frame. The tall mirror-gold carton with thin black top and bottom bands stands on the right third on black lacquer, five amber vials with white caps and the flat gold-foil sachet in front, the set lit by a warm gold glow (#D4A853) behind the carton and a thin gold hairline reflection on the surface; the left two-thirds pure near-black for the offer and buttons. Camera: 85 mm, eye level, f/4. Calm, premium, final. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/vtech-system.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL CARTON — mirror-polished gold foil, black bands at top and bottom: top: 'VM' in silver letters; centre: a large black 'V' with a small inverted black triangle above it; lower third: 'V-TECH' letter-spaced (the V drawn as the same V-with-triangle mark), below it letter-spaced 'S Y S T E M' || 5 VIALS — amber glass vials with white flip-off caps, amber label: white V-with-triangle mark; 'V-TECH'; [unreadable] one tiny line under 'V-TECH'; white graduation ticks on the side || GEL MASK SACHET — gold foil sachet with a small white nozzle cap on the left: large black V-with-triangle mark; 'V-TECH' letter-spaced, below it 'G E L   M A S K'; [unreadable] four tiny lines at the bottom.</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
@@ -53978,7 +52870,7 @@
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exosignal-hair.webp. Photoreal cinematic product hero, 16:9. A matte black landscape carton (wider than tall) standing on the right third on a black satin surface; in front of it five clear glass snap-neck ampoules with colourless liquid standing in a loose row, catching a warm gold edge light (#C9A24A). Background: matte black (#111111), a faint warm gold glow only behind the carton, no haze elsewhere. Lighting: warm key from the upper left, a cool white highlight along the ampoule necks. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds empty for text. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exosignal-hair.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exosignal-hair.webp. Photoreal cinematic product hero, 16:9. A matte black landscape carton (wider than tall) standing on the right third on a black satin surface; in front of it five clear glass snap-neck ampoules with colourless liquid standing in a loose row, catching a warm gold edge light (#C9A24A). Background: matte black (#111111), a faint warm gold glow only behind the carton, no haze elsewhere. Lighting: warm key from the upper left, a cool white highlight along the ampoule necks. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds empty for text. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exosignal-hair.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): FLAT BOX — matte black box, gold and white print: top centre: grey VM monogram, small 'VM corporation'; centre, gold: 'EXOSIGNAL' ('EXO' bold) with letter-spaced 'H A I R' below right; lower block, white: 'EXOSIGNAL HAIR' / 'SIERO NUTRIENTE PER IL CUOIO CAPELLUTO' / 'NOURISHING SCALP SERUM' / 'SÉRUM NOURRISSANT CUIR CHEVELU' / 'SERUM NUTRITIVO PARA EL CUERO CABELLUDO'; 'Net 5 x 5 ml ℮ 5 x 0.17 fl.oz.' || 5 AMPOULES — clear glass ampoules with a white ring at the neck: 'EXOSIGNAL HAIR' printed vertically in black ('EXO' bold).</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
@@ -54128,7 +53020,7 @@
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>Photoreal macro, 16:9. A clear glass snap-neck ampoule with its neck snapped open, tilted, a single clear drop falling from it on the left; centre-right the drop enlarged into a translucent sphere (an engineered vesicle) with glowing strands and particles inside, warm gold (#C9A24A) backlight on matte black (#111111). Camera: 100 mm macro, f/4, sphere sharp, ampoule slightly soft. No overlay text, no logos, no labels.</t>
+          <t>Photoreal macro, 16:9. A clear glass snap-neck ampoule with its neck snapped open, tilted, a single clear drop falling from it on the left; centre-right the drop enlarged into a translucent sphere (an engineered vesicle) with glowing strands and particles inside, warm gold (#C9A24A) backlight on matte black (#111111). Camera: 100 mm macro, f/4, sphere sharp, ampoule slightly soft. No overlay text, no logos, no labels. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): FLAT BOX — matte black box, gold and white print: top centre: grey VM monogram, small 'VM corporation'; centre, gold: 'EXOSIGNAL' ('EXO' bold) with letter-spaced 'H A I R' below right; lower block, white: 'EXOSIGNAL HAIR' / 'SIERO NUTRIENTE PER IL CUOIO CAPELLUTO' / 'NOURISHING SCALP SERUM' / 'SÉRUM NOURRISSANT CUIR CHEVELU' / 'SERUM NUTRITIVO PARA EL CUERO CABELLUDO'; 'Net 5 x 5 ml ℮ 5 x 0.17 fl.oz.' || 5 AMPOULES — clear glass ampoules with a white ring at the neck: 'EXOSIGNAL HAIR' printed vertically in black ('EXO' bold).</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
@@ -54203,7 +53095,7 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic portrait, 16:9. A woman in her thirties with fine, thinning hair sits facing the camera as if into a mirror; behind her a practitioner dressed in black parts her hair and applies a clear serum from a glass snap-neck ampoule along the parting with gloved fingers. Her eyes meet the lens, hopeful and calm. Environment: dark trichology room with matte black walls, a warm gold key light from the front-left, a faint cool glow from a white tablet screen on a stand at the right edge. Camera: 85 mm, f/2, eye level, subject in the left two-thirds, right third dark for text. No overlay text, no logos.</t>
+          <t>Photoreal cinematic portrait, 16:9. A woman in her thirties with fine, thinning hair sits facing the camera as if into a mirror; behind her a practitioner dressed in black parts her hair and applies a clear serum from a glass snap-neck ampoule along the parting with gloved fingers. Her eyes meet the lens, hopeful and calm. Environment: dark trichology room with matte black walls, a warm gold key light from the front-left, a faint cool glow from a white tablet screen on a stand at the right edge. Camera: 85 mm, f/2, eye level, subject in the left two-thirds, right third dark for text. No overlay text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): FLAT BOX — matte black box, gold and white print: top centre: grey VM monogram, small 'VM corporation'; centre, gold: 'EXOSIGNAL' ('EXO' bold) with letter-spaced 'H A I R' below right; lower block, white: 'EXOSIGNAL HAIR' / 'SIERO NUTRIENTE PER IL CUOIO CAPELLUTO' / 'NOURISHING SCALP SERUM' / 'SÉRUM NOURRISSANT CUIR CHEVELU' / 'SERUM NUTRITIVO PARA EL CUERO CABELLUDO'; 'Net 5 x 5 ml ℮ 5 x 0.17 fl.oz.' || 5 AMPOULES — clear glass ampoules with a white ring at the neck: 'EXOSIGNAL HAIR' printed vertically in black ('EXO' bold).</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
@@ -54278,7 +53170,7 @@
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exosignal-hair.webp. Photoreal counter scene, 16:9. On a black satin counter, left to right with space between: a white tablet-style screen on a white stand with a silver cylindrical base, the screen showing an abstract magnified scalp circle, with a corded white handheld scope camera resting in front of it; a slim cordless microneedling pen with a champagne-gold body, rose-gold grip ring and clear needle cartridge; a clear glass snap-neck ampoule standing in a small holder; and a small clear glass spray bottle with a tall gold cap at the far right. Lighting: thin warm gold rim light from above, soft fill, matte black background (#111111). Camera: 50 mm, slightly above eye level, f/8, all items sharp, the row centred with margins. No overlay text or captions, no text other than the packaging's own printing, screen content abstract, the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exosignal-hair.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exosignal-hair.webp. Photoreal counter scene, 16:9. On a black satin counter, left to right with space between: a white tablet-style screen on a white stand with a silver cylindrical base, the screen showing an abstract magnified scalp circle, with a corded white handheld scope camera resting in front of it; a slim cordless microneedling pen with a champagne-gold body, rose-gold grip ring and clear needle cartridge; a clear glass snap-neck ampoule standing in a small holder; and a small clear glass spray bottle with a tall gold cap at the far right. Lighting: thin warm gold rim light from above, soft fill, matte black background (#111111). Camera: 50 mm, slightly above eye level, f/8, all items sharp, the row centred with margins. No overlay text or captions, no text other than the packaging's own printing, screen content abstract, the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exosignal-hair.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): FLAT BOX — matte black box, gold and white print: top centre: grey VM monogram, small 'VM corporation'; centre, gold: 'EXOSIGNAL' ('EXO' bold) with letter-spaced 'H A I R' below right; lower block, white: 'EXOSIGNAL HAIR' / 'SIERO NUTRIENTE PER IL CUOIO CAPELLUTO' / 'NOURISHING SCALP SERUM' / 'SÉRUM NOURRISSANT CUIR CHEVELU' / 'SERUM NUTRITIVO PARA EL CUERO CABELLUDO'; 'Net 5 x 5 ml ℮ 5 x 0.17 fl.oz.' || 5 AMPOULES — clear glass ampoules with a white ring at the neck: 'EXOSIGNAL HAIR' printed vertically in black ('EXO' bold).</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
@@ -54353,7 +53245,7 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exosignal-hair.webp. Photoreal product shot, 16:9. The matte black landscape carton, closed, in three-quarter view on the left; in front of it five clear glass snap-neck ampoules with colourless liquid, four standing in a row and one lying on its side in front. Lighting: warm gold key from the upper right, cool highlight on the glass necks, matte black background, a soft gold glow behind the box only. Camera: 70 mm, f/5.6, right third empty for numbers. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exosignal-hair.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exosignal-hair.webp. Photoreal product shot, 16:9. The matte black landscape carton, closed, in three-quarter view on the left; in front of it five clear glass snap-neck ampoules with colourless liquid, four standing in a row and one lying on its side in front. Lighting: warm gold key from the upper right, cool highlight on the glass necks, matte black background, a soft gold glow behind the box only. Camera: 70 mm, f/5.6, right third empty for numbers. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exosignal-hair.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): FLAT BOX — matte black box, gold and white print: top centre: grey VM monogram, small 'VM corporation'; centre, gold: 'EXOSIGNAL' ('EXO' bold) with letter-spaced 'H A I R' below right; lower block, white: 'EXOSIGNAL HAIR' / 'SIERO NUTRIENTE PER IL CUOIO CAPELLUTO' / 'NOURISHING SCALP SERUM' / 'SÉRUM NOURRISSANT CUIR CHEVELU' / 'SERUM NUTRITIVO PARA EL CUERO CABELLUDO'; 'Net 5 x 5 ml ℮ 5 x 0.17 fl.oz.' || 5 AMPOULES — clear glass ampoules with a white ring at the neck: 'EXOSIGNAL HAIR' printed vertically in black ('EXO' bold).</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
@@ -54428,7 +53320,7 @@
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exosignal-hair.webp. Photoreal cinematic closing hero, 16:9. The matte black landscape carton on the right third on black satin, five clear snap-neck ampoules lined up in front, a warm gold glow (#C9A24A) behind the box and a thin gold reflection line on the surface; the left two-thirds matte black for the offer and buttons. Camera: 85 mm, eye level, f/4. Quiet, premium, final. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exosignal-hair.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exosignal-hair.webp. Photoreal cinematic closing hero, 16:9. The matte black landscape carton on the right third on black satin, five clear snap-neck ampoules lined up in front, a warm gold glow (#C9A24A) behind the box and a thin gold reflection line on the surface; the left two-thirds matte black for the offer and buttons. Camera: 85 mm, eye level, f/4. Quiet, premium, final. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exosignal-hair.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): FLAT BOX — matte black box, gold and white print: top centre: grey VM monogram, small 'VM corporation'; centre, gold: 'EXOSIGNAL' ('EXO' bold) with letter-spaced 'H A I R' below right; lower block, white: 'EXOSIGNAL HAIR' / 'SIERO NUTRIENTE PER IL CUOIO CAPELLUTO' / 'NOURISHING SCALP SERUM' / 'SÉRUM NOURRISSANT CUIR CHEVELU' / 'SERUM NUTRITIVO PARA EL CUERO CABELLUDO'; 'Net 5 x 5 ml ℮ 5 x 0.17 fl.oz.' || 5 AMPOULES — clear glass ampoules with a white ring at the neck: 'EXOSIGNAL HAIR' printed vertically in black ('EXO' bold).</t>
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr">
@@ -54503,7 +53395,7 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product still, 16:9. A tall slim ivory-cream cardboard box (MITODERM MICRO BOOST 10%: ivory box, a deep green horizontal band with gold lettering, a round gold-rimmed window printed with a tangle of thin green needle-like spicules, a small gold monogram at the top) standing upright on a matte deep green (#1E4634) lacquered surface, placed in the right third of the frame; the left two-thirds are an empty dark green gradient falling to near-black green. Lighting: soft warm key from upper left, crisp cool mint rim light along the box's right edge, faint reflection in the surface. In the dark background a sparse out-of-focus drift of microscopic translucent glass-like needles catching mint light. 85 mm lens, f/4, slight low angle, premium cosmetic-campaign look. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal cinematic product still, 16:9. A tall slim ivory-cream cardboard box (MITODERM MICRO BOOST 10%: ivory box, a deep green horizontal band with gold lettering, a round gold-rimmed window printed with a tangle of thin green needle-like spicules, a small gold monogram at the top) standing upright on a matte deep green (#1E4634) lacquered surface, placed in the right third of the frame; the left two-thirds are an empty dark green gradient falling to near-black green. Lighting: soft warm key from upper left, crisp cool mint rim light along the box's right edge, faint reflection in the surface. In the dark background a sparse out-of-focus drift of microscopic translucent glass-like needles catching mint light. 85 mm lens, f/4, slight low angle, premium cosmetic-campaign look. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced dark green, below 'BIOSPICULE PROFESSIONAL'; dark green band with gold text 'MICRO BOOST 10%'; 'SPICULE SERUM'; round medallion in a gold ring with dark green spicules; gold-framed box: 'Concentrated' / 'Spicule System'; between two thin lines: 'PROFESSIONAL TREATMENT'; bottom: '3 ml ℮ 0.10 fl.oz.'.</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
@@ -54728,7 +53620,7 @@
       </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic still, 16:9. A woman in her forties with natural un-retouched skin sits facing the camera as if the camera were a mirror, in a calm clinic room washed in deep green (#1E4634) shadow with a soft mint-tinted light on her face. From behind her, a pair of hands in white nitrile gloves massages a thin translucent serum into her left cheek with fingertips; the skin there is slightly flushed and glossy. Relaxed expression, eyes on the mirror. Subject in the left two-thirds, right third dark green and empty. 50 mm, f/2, shallow focus on the cheek, cinematic grade. No text, no logos, no packaging in frame.</t>
+          <t>Photoreal cinematic still, 16:9. A woman in her forties with natural un-retouched skin sits facing the camera as if the camera were a mirror, in a calm clinic room washed in deep green (#1E4634) shadow with a soft mint-tinted light on her face. From behind her, a pair of hands in white nitrile gloves massages a thin translucent serum into her left cheek with fingertips; the skin there is slightly flushed and glossy. Relaxed expression, eyes on the mirror. Subject in the left two-thirds, right third dark green and empty. 50 mm, f/2, shallow focus on the cheek, cinematic grade. No text, no logos, no packaging in frame. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced dark green, below 'BIOSPICULE PROFESSIONAL'; dark green band with gold text 'MICRO BOOST 10%'; 'SPICULE SERUM'; round medallion in a gold ring with dark green spicules; gold-framed box: 'Concentrated' / 'Spicule System'; between two thin lines: 'PROFESSIONAL TREATMENT'; bottom: '3 ml ℮ 0.10 fl.oz.'.</t>
         </is>
       </c>
       <c r="N19" s="5" t="inlineStr">
@@ -54803,7 +53695,7 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic still, 16:9. A glass shelf in a dark clinic room, deep green (#1E4634) background, cool clinical top light. On the shelf, left to right, evenly spaced with room for captions above each: a small 3 ml syringe without needle lying on a slim ivory box with a deep green band and a round gold-rimmed spicule window, a small 5 ml glass serum ampoule, a flat single-use sheet-mask sachet, and a square ivory cardboard box with a deep green band and a printed white cream swirl. Soft reflections in the glass. 35 mm, f/5.6, everything in focus. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal cinematic still, 16:9. A glass shelf in a dark clinic room, deep green (#1E4634) background, cool clinical top light. On the shelf, left to right, evenly spaced with room for captions above each: a small 3 ml syringe without needle lying on a slim ivory box with a deep green band and a round gold-rimmed spicule window, a small 5 ml glass serum ampoule, a flat single-use sheet-mask sachet, and a square ivory cardboard box with a deep green band and a printed white cream swirl. Soft reflections in the glass. 35 mm, f/5.6, everything in focus. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced dark green, below 'BIOSPICULE PROFESSIONAL'; dark green band with gold text 'MICRO BOOST 10%'; 'SPICULE SERUM'; round medallion in a gold ring with dark green spicules; gold-framed box: 'Concentrated' / 'Spicule System'; between two thin lines: 'PROFESSIONAL TREATMENT'; bottom: '3 ml ℮ 0.10 fl.oz.'.</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
@@ -54878,7 +53770,7 @@
       </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
-          <t>Photoreal overhead flat-lay, 16:9. On a matte deep green (#1E4634) surface: an open ivory MITODERM MICRO BOOST 10% box (ivory, deep green band, round gold-rimmed spicule window) lying flat, and beside it a small 3 ml syringe, cap on, no needle (match the real syringe from a supplied product photo). Soft even top light with one gentle warm highlight, faint shadow. Generous negative space in all four corners. 50 mm from directly above, f/8, crisp. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal overhead flat-lay, 16:9. On a matte deep green (#1E4634) surface: an open ivory MITODERM MICRO BOOST 10% box (ivory, deep green band, round gold-rimmed spicule window) lying flat, and beside it a small 3 ml syringe, cap on, no needle (match the real syringe from a supplied product photo). Soft even top light with one gentle warm highlight, faint shadow. Generous negative space in all four corners. 50 mm from directly above, f/8, crisp. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced dark green, below 'BIOSPICULE PROFESSIONAL'; dark green band with gold text 'MICRO BOOST 10%'; 'SPICULE SERUM'; round medallion in a gold ring with dark green spicules; gold-framed box: 'Concentrated' / 'Spicule System'; between two thin lines: 'PROFESSIONAL TREATMENT'; bottom: '3 ml ℮ 0.10 fl.oz.'.</t>
         </is>
       </c>
       <c r="N21" s="5" t="inlineStr">
@@ -54953,7 +53845,7 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product still, 16:9. The ivory MITODERM MICRO BOOST 10% box (ivory, deep green band, round gold-rimmed spicule window) standing upright in the right third on a deep green (#1E4634) surface, now in warm inviting light: warm key from the left, mint rim on the right, a soft golden glow on the surface behind it. Left two-thirds empty, one step lighter green than the opening frame. 85 mm, f/4. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal cinematic product still, 16:9. The ivory MITODERM MICRO BOOST 10% box (ivory, deep green band, round gold-rimmed spicule window) standing upright in the right third on a deep green (#1E4634) surface, now in warm inviting light: warm key from the left, mint rim on the right, a soft golden glow on the surface behind it. Left two-thirds empty, one step lighter green than the opening frame. 85 mm, f/4. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced dark green, below 'BIOSPICULE PROFESSIONAL'; dark green band with gold text 'MICRO BOOST 10%'; 'SPICULE SERUM'; round medallion in a gold ring with dark green spicules; gold-framed box: 'Concentrated' / 'Spicule System'; between two thin lines: 'PROFESSIONAL TREATMENT'; bottom: '3 ml ℮ 0.10 fl.oz.'.</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
@@ -55028,7 +53920,7 @@
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>Background plate for compositing: a near-black studio tabletop with a faint mirror reflection, deep charcoal-bronze gradient rising to pure black at the top, one warm gold light sweep entering from the upper right, soft volumetric haze, very subtle gold dust suspended in the air, the right third kept empty for a mirror-polished gold sphere jar with a thin seam just below its equator and a black cube box whose front face is mirror-gold foil with a black diagonal wedge at the left edge, photoreal cinematic product photography, 85 mm lens, f/4, low camera at jar height, 16:9, no text, no captions, no logos.</t>
+          <t>Background plate for compositing: a near-black studio tabletop with a faint mirror reflection, deep charcoal-bronze gradient rising to pure black at the top, one warm gold light sweep entering from the upper right, soft volumetric haze, very subtle gold dust suspended in the air, the right third kept empty for a mirror-polished gold sphere jar with a thin seam just below its equator and a black cube box whose front face is mirror-gold foil with a black diagonal wedge at the left edge, photoreal cinematic product photography, 85 mm lens, f/4, low camera at jar height, 16:9, no text, no captions, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): CUBE BOX — mirror gold foil cube with a black diagonal panel on the left side: 'EXOTECH' ('EXO' bold) in black, below it italic letter-spaced 'G E L' || SPHERICAL JAR — polished gold sphere jar with a thin seam: 'EXOTECH' / italic 'GEL' in black.</t>
         </is>
       </c>
       <c r="N23" s="5" t="inlineStr">
@@ -55103,7 +53995,7 @@
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>Cinematic low-key portrait of a woman in her 40s, calm neutral expression, face lit by a single warm gold edge light from the right, deep black background, natural un-retouched skin, shallow depth of field, 85 mm, f/2, dark bronze grade with gold highlights for a black-and-gold page, left third of the frame kept empty and dark for a floating half-open mirror-gold sphere jar, photoreal, 16:9, no text, no logos.</t>
+          <t>Cinematic low-key portrait of a woman in her 40s, calm neutral expression, face lit by a single warm gold edge light from the right, deep black background, natural un-retouched skin, shallow depth of field, 85 mm, f/2, dark bronze grade with gold highlights for a black-and-gold page, left third of the frame kept empty and dark for a floating half-open mirror-gold sphere jar, photoreal, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): CUBE BOX — mirror gold foil cube with a black diagonal panel on the left side: 'EXOTECH' ('EXO' bold) in black, below it italic letter-spaced 'G E L' || SPHERICAL JAR — polished gold sphere jar with a thin seam: 'EXOTECH' / italic 'GEL' in black.</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
@@ -55253,7 +54145,7 @@
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>Medium close-up of a woman in her 40s facing the camera as if it were her bathroom mirror, massaging a thin layer of translucent gel into her cheek with two fingers, eyes meeting the lens, calm evening mood, dark bathroom with one warm gold practical light, a mirror-gold sphere jar open on the shelf beside her with its upper hemisphere resting next to it, black-and-gold grade, 50 mm, f/2.8, photoreal, cinematic, natural skin, 16:9, no text, no logos.</t>
+          <t>Medium close-up of a woman in her 40s facing the camera as if it were her bathroom mirror, massaging a thin layer of translucent gel into her cheek with two fingers, eyes meeting the lens, calm evening mood, dark bathroom with one warm gold practical light, a mirror-gold sphere jar open on the shelf beside her with its upper hemisphere resting next to it, black-and-gold grade, 50 mm, f/2.8, photoreal, cinematic, natural skin, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): CUBE BOX — mirror gold foil cube with a black diagonal panel on the left side: 'EXOTECH' ('EXO' bold) in black, below it italic letter-spaced 'G E L' || SPHERICAL JAR — polished gold sphere jar with a thin seam: 'EXOTECH' / italic 'GEL' in black.</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
@@ -55328,7 +54220,7 @@
       </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
-          <t>A closed mirror-polished gold sphere jar on a dark stone bathroom shelf in soft morning window light from the left, a folded white towel out of focus behind, black background fading to warm bronze, calm daily-ritual mood for a black-and-gold page, 50 mm, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>A closed mirror-polished gold sphere jar on a dark stone bathroom shelf in soft morning window light from the left, a folded white towel out of focus behind, black background fading to warm bronze, calm daily-ritual mood for a black-and-gold page, 50 mm, f/4, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): CUBE BOX — mirror gold foil cube with a black diagonal panel on the left side: 'EXOTECH' ('EXO' bold) in black, below it italic letter-spaced 'G E L' || SPHERICAL JAR — polished gold sphere jar with a thin seam: 'EXOTECH' / italic 'GEL' in black.</t>
         </is>
       </c>
       <c r="N27" s="5" t="inlineStr">
@@ -55403,7 +54295,7 @@
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>Top-down 3/4 view of a black cube box with a mirror-gold foil front face and a black diagonal wedge at its left edge, a mirror-polished gold sphere jar standing in front of it, both on a black reflective surface, warm gold key light from the upper left, deep black surroundings, luxury still-life mood for a black-and-gold page, 50 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Top-down 3/4 view of a black cube box with a mirror-gold foil front face and a black diagonal wedge at its left edge, a mirror-polished gold sphere jar standing in front of it, both on a black reflective surface, warm gold key light from the upper left, deep black surroundings, luxury still-life mood for a black-and-gold page, 50 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): CUBE BOX — mirror gold foil cube with a black diagonal panel on the left side: 'EXOTECH' ('EXO' bold) in black, below it italic letter-spaced 'G E L' || SPHERICAL JAR — polished gold sphere jar with a thin seam: 'EXOTECH' / italic 'GEL' in black.</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
@@ -55478,7 +54370,7 @@
       </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>Mirror-polished gold sphere jar standing beside a black cube box whose front face is mirror-gold foil with a black diagonal wedge at the left edge, both on a black reflective surface, generous warm gold light from the upper right, soft gold haze, deep black surroundings, left half of the frame empty and dark for copy, premium closing shot for a black-and-gold page, 85 mm, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Mirror-polished gold sphere jar standing beside a black cube box whose front face is mirror-gold foil with a black diagonal wedge at the left edge, both on a black reflective surface, generous warm gold light from the upper right, soft gold haze, deep black surroundings, left half of the frame empty and dark for copy, premium closing shot for a black-and-gold page, 85 mm, f/4, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): CUBE BOX — mirror gold foil cube with a black diagonal panel on the left side: 'EXOTECH' ('EXO' bold) in black, below it italic letter-spaced 'G E L' || SPHERICAL JAR — polished gold sphere jar with a thin seam: 'EXOTECH' / italic 'GEL' in black.</t>
         </is>
       </c>
       <c r="N29" s="5" t="inlineStr">
@@ -55553,7 +54445,7 @@
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>Background plate for compositing: a near-black studio with a warm gold rim light from the upper right, a barely visible reflective black surface, a frozen cloud of fine mist droplets suspended in the light at the right third of the frame (where a slim frosted-glass 15 ml spray bottle with a tall polished-gold cap and its tall matte-black rectangular carton will be composited), very faint haze, black-and-gold grade with frosted-white highlights, 85 mm, f/4, low camera, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Background plate for compositing: a near-black studio with a warm gold rim light from the upper right, a barely visible reflective black surface, a frozen cloud of fine mist droplets suspended in the light at the right third of the frame (where a slim frosted-glass 15 ml spray bottle with a tall polished-gold cap and its tall matte-black rectangular carton will be composited), very faint haze, black-and-gold grade with frosted-white highlights, 85 mm, f/4, low camera, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL BOX — matte black box, gold and white print: top: VM monogram; centre, gold: 'EXOSIGNAL' ('EXO' bold), below it letter-spaced 'S P R A Y · H O M E'; lower: 'EXOSIGNAL SPRAY HOME' and [unreadable] four tiny white lines, a small boxed label || SPRAY BOTTLE — white-silver cylinder with a gold cap: VM monogram; 'EXOSIGNAL' running vertically ('EXO' bold); [unreadable] two tiny lines at the bottom.</t>
         </is>
       </c>
       <c r="N30" s="5" t="inlineStr">
@@ -55778,7 +54670,7 @@
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>Medium close-up of a woman in her 30s facing the camera as if it were her bathroom mirror, one hand parting her dark hair to expose the scalp, the other holding a slim frosted-glass spray bottle with a tall polished-gold cap at the parting, calm expression, one warm practical light, dark tiled wall, a tall matte-black carton on the shelf, black-and-gold grade, 50 mm, f/2.8, photoreal, cinematic, natural skin and hair, 16:9, no text, no logos.</t>
+          <t>Medium close-up of a woman in her 30s facing the camera as if it were her bathroom mirror, one hand parting her dark hair to expose the scalp, the other holding a slim frosted-glass spray bottle with a tall polished-gold cap at the parting, calm expression, one warm practical light, dark tiled wall, a tall matte-black carton on the shelf, black-and-gold grade, 50 mm, f/2.8, photoreal, cinematic, natural skin and hair, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL BOX — matte black box, gold and white print: top: VM monogram; centre, gold: 'EXOSIGNAL' ('EXO' bold), below it letter-spaced 'S P R A Y · H O M E'; lower: 'EXOSIGNAL SPRAY HOME' and [unreadable] four tiny white lines, a small boxed label || SPRAY BOTTLE — white-silver cylinder with a gold cap: VM monogram; 'EXOSIGNAL' running vertically ('EXO' bold); [unreadable] two tiny lines at the bottom.</t>
         </is>
       </c>
       <c r="N33" s="5" t="inlineStr">
@@ -55853,7 +54745,7 @@
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>A slim frosted-glass 15 ml spray bottle with a tall polished-gold cap standing on a black stone bathroom shelf beside its tall matte-black rectangular carton, warm morning window light from the left, soft reflection, black background, calm daily-ritual mood for a black-and-gold page, 50 mm, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>A slim frosted-glass 15 ml spray bottle with a tall polished-gold cap standing on a black stone bathroom shelf beside its tall matte-black rectangular carton, warm morning window light from the left, soft reflection, black background, calm daily-ritual mood for a black-and-gold page, 50 mm, f/4, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL BOX — matte black box, gold and white print: top: VM monogram; centre, gold: 'EXOSIGNAL' ('EXO' bold), below it letter-spaced 'S P R A Y · H O M E'; lower: 'EXOSIGNAL SPRAY HOME' and [unreadable] four tiny white lines, a small boxed label || SPRAY BOTTLE — white-silver cylinder with a gold cap: VM monogram; 'EXOSIGNAL' running vertically ('EXO' bold); [unreadable] two tiny lines at the bottom.</t>
         </is>
       </c>
       <c r="N34" s="5" t="inlineStr">
@@ -55928,7 +54820,7 @@
       </c>
       <c r="M35" s="5" t="inlineStr">
         <is>
-          <t>Top-down 3/4 view of a tall matte-black rectangular carton opened at the top, a slim frosted-glass spray bottle with a tall polished-gold cap standing half-inside it, on a black reflective surface, warm gold key light from the upper left, deep black surroundings, precise unboxing mood for a black-and-gold page, 50 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Top-down 3/4 view of a tall matte-black rectangular carton opened at the top, a slim frosted-glass spray bottle with a tall polished-gold cap standing half-inside it, on a black reflective surface, warm gold key light from the upper left, deep black surroundings, precise unboxing mood for a black-and-gold page, 50 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL BOX — matte black box, gold and white print: top: VM monogram; centre, gold: 'EXOSIGNAL' ('EXO' bold), below it letter-spaced 'S P R A Y · H O M E'; lower: 'EXOSIGNAL SPRAY HOME' and [unreadable] four tiny white lines, a small boxed label || SPRAY BOTTLE — white-silver cylinder with a gold cap: VM monogram; 'EXOSIGNAL' running vertically ('EXO' bold); [unreadable] two tiny lines at the bottom.</t>
         </is>
       </c>
       <c r="N35" s="5" t="inlineStr">
@@ -56003,7 +54895,7 @@
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>A slim frosted-glass 15 ml spray bottle with a tall polished-gold cap standing beside its tall matte-black rectangular carton on a black reflective surface, a fine frozen mist above the cap, bright warm gold rim light from the upper right, deep black surroundings, left half of the frame empty and dark for copy, premium closing shot for a black-and-gold page, 85 mm, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>A slim frosted-glass 15 ml spray bottle with a tall polished-gold cap standing beside its tall matte-black rectangular carton on a black reflective surface, a fine frozen mist above the cap, bright warm gold rim light from the upper right, deep black surroundings, left half of the frame empty and dark for copy, premium closing shot for a black-and-gold page, 85 mm, f/4, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL BOX — matte black box, gold and white print: top: VM monogram; centre, gold: 'EXOSIGNAL' ('EXO' bold), below it letter-spaced 'S P R A Y · H O M E'; lower: 'EXOSIGNAL SPRAY HOME' and [unreadable] four tiny white lines, a small boxed label || SPRAY BOTTLE — white-silver cylinder with a gold cap: VM monogram; 'EXOSIGNAL' running vertically ('EXO' bold); [unreadable] two tiny lines at the bottom.</t>
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr">
@@ -56078,7 +54970,7 @@
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product still, 16:9. A slim ivory-cream cardboard box (MITODERM CELL RENEW 1.5%: ivory, a muted deep green horizontal band with gold lettering, a round thin-gold-rimmed window printed with green needle-like spicules, a small gold monogram at the top) standing in the right third on a pale stone bathroom shelf, soft daylight from a window on the left, a deep green (#1E4634) wall behind that lightens to sage near the light. A few water droplets on the shelf, gentle reflections. 85 mm, f/2.8, shallow, calm and fresh. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal cinematic product still, 16:9. A slim ivory-cream cardboard box (MITODERM CELL RENEW 1.5%: ivory, a muted deep green horizontal band with gold lettering, a round thin-gold-rimmed window printed with green needle-like spicules, a small gold monogram at the top) standing in the right third on a pale stone bathroom shelf, soft daylight from a window on the left, a deep green (#1E4634) wall behind that lightens to sage near the light. A few water droplets on the shelf, gentle reflections. 85 mm, f/2.8, shallow, calm and fresh. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, medium green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; medium green band with gold text 'CELL RENEW' / '1.5%'; 'BIOSPICULE' / 'SERUM'; round medallion in a green ring with dark green spicules; gold-framed box: 'ADVANCED' / 'BIOSPICULE TECHNOLOGY'; bottom: '30 ml ℮ 1.0 fl.oz.'.</t>
         </is>
       </c>
       <c r="N37" s="5" t="inlineStr">
@@ -56303,7 +55195,7 @@
       </c>
       <c r="M40" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic still, 16:9. A woman in her thirties facing the camera as if it were her bathroom mirror, window light from the left, deep green (#1E4634) shadowed wall behind, fresh un-retouched skin slightly flushed on the cheek where two fingertips massage a translucent serum in a small circle. Hair tied back, calm face, eyes on the mirror. Subject in the left two-thirds, right third dark green. 50 mm, f/2, shallow focus on the fingertips. No text, no logos, no visible packaging.</t>
+          <t>Photoreal cinematic still, 16:9. A woman in her thirties facing the camera as if it were her bathroom mirror, window light from the left, deep green (#1E4634) shadowed wall behind, fresh un-retouched skin slightly flushed on the cheek where two fingertips massage a translucent serum in a small circle. Hair tied back, calm face, eyes on the mirror. Subject in the left two-thirds, right third dark green. 50 mm, f/2, shallow focus on the fingertips. No text, no logos, no visible packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, medium green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; medium green band with gold text 'CELL RENEW' / '1.5%'; 'BIOSPICULE' / 'SERUM'; round medallion in a green ring with dark green spicules; gold-framed box: 'ADVANCED' / 'BIOSPICULE TECHNOLOGY'; bottom: '30 ml ℮ 1.0 fl.oz.'.</t>
         </is>
       </c>
       <c r="N40" s="5" t="inlineStr">
@@ -56378,7 +55270,7 @@
       </c>
       <c r="M41" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic still, 16:9. A pale stone bathroom shelf in window light, deep green (#1E4634) wall behind. Left to right, evenly spaced with room for captions above: a slim ivory box with a muted deep green band and a round thin-gold-rimmed spicule window (CELL RENEW 1.5%), a square ivory box with a deep green band and a printed white cream swirl (DERMA RECOVERY CREAM), and an unbranded plain white sunscreen tube. Soft window light from the left, clean reflections. 35 mm, f/5.6, all in focus. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal cinematic still, 16:9. A pale stone bathroom shelf in window light, deep green (#1E4634) wall behind. Left to right, evenly spaced with room for captions above: a slim ivory box with a muted deep green band and a round thin-gold-rimmed spicule window (CELL RENEW 1.5%), a square ivory box with a deep green band and a printed white cream swirl (DERMA RECOVERY CREAM), and an unbranded plain white sunscreen tube. Soft window light from the left, clean reflections. 35 mm, f/5.6, all in focus. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, medium green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; medium green band with gold text 'CELL RENEW' / '1.5%'; 'BIOSPICULE' / 'SERUM'; round medallion in a green ring with dark green spicules; gold-framed box: 'ADVANCED' / 'BIOSPICULE TECHNOLOGY'; bottom: '30 ml ℮ 1.0 fl.oz.'.</t>
         </is>
       </c>
       <c r="N41" s="5" t="inlineStr">
@@ -56453,7 +55345,7 @@
       </c>
       <c r="M42" s="5" t="inlineStr">
         <is>
-          <t>Photoreal overhead flat-lay, 16:9. On a pale stone surface tinted by deep green (#1E4634) shadow at the edges: the slim ivory MITODERM CELL RENEW 1.5% box (ivory, muted deep green band, round thin-gold-rimmed spicule window) lying flat, beside it a single translucent drop of serum catching the light. Soft daylight, generous negative space in all four corners. 50 mm from directly above, f/8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal overhead flat-lay, 16:9. On a pale stone surface tinted by deep green (#1E4634) shadow at the edges: the slim ivory MITODERM CELL RENEW 1.5% box (ivory, muted deep green band, round thin-gold-rimmed spicule window) lying flat, beside it a single translucent drop of serum catching the light. Soft daylight, generous negative space in all four corners. 50 mm from directly above, f/8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, medium green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; medium green band with gold text 'CELL RENEW' / '1.5%'; 'BIOSPICULE' / 'SERUM'; round medallion in a green ring with dark green spicules; gold-framed box: 'ADVANCED' / 'BIOSPICULE TECHNOLOGY'; bottom: '30 ml ℮ 1.0 fl.oz.'.</t>
         </is>
       </c>
       <c r="N42" s="5" t="inlineStr">
@@ -56528,7 +55420,7 @@
       </c>
       <c r="M43" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product still, 16:9. The ivory MITODERM CELL RENEW 1.5% box standing upright in the right third on a pale stone shelf, warm daylight from the left, mint rim light on the right; slightly behind and out of focus a second identical-format ivory box with a deep green band (CELLULAR AGE DEFENSE 2.5%). Deep green (#1E4634) wall softening to sage. Left two-thirds empty. 85 mm, f/2.8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal cinematic product still, 16:9. The ivory MITODERM CELL RENEW 1.5% box standing upright in the right third on a pale stone shelf, warm daylight from the left, mint rim light on the right; slightly behind and out of focus a second identical-format ivory box with a deep green band (CELLULAR AGE DEFENSE 2.5%). Deep green (#1E4634) wall softening to sage. Left two-thirds empty. 85 mm, f/2.8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, medium green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; medium green band with gold text 'CELL RENEW' / '1.5%'; 'BIOSPICULE' / 'SERUM'; round medallion in a green ring with dark green spicules; gold-framed box: 'ADVANCED' / 'BIOSPICULE TECHNOLOGY'; bottom: '30 ml ℮ 1.0 fl.oz.'.</t>
         </is>
       </c>
       <c r="N43" s="5" t="inlineStr">
@@ -56603,7 +55495,7 @@
       </c>
       <c r="M44" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product still, 16:9. A slim ivory-cream cardboard box (MITODERM CELLULAR AGE DEFENSE 2.5%: ivory, a deep green horizontal band with gold lettering, a round thin-gold-rimmed window printed with green needle-like spicules, a small gold monogram at the top) standing upright in the right third on a dark polished vanity, evening mood: warm lamp key light from the upper left, cool mint rim light on the right, deep green (#1E4634) to near-black background. Behind the box five faint golden hair-thin threads of light drift upward, out of focus. 85 mm, f/2.8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal cinematic product still, 16:9. A slim ivory-cream cardboard box (MITODERM CELLULAR AGE DEFENSE 2.5%: ivory, a deep green horizontal band with gold lettering, a round thin-gold-rimmed window printed with green needle-like spicules, a small gold monogram at the top) standing upright in the right third on a dark polished vanity, evening mood: warm lamp key light from the upper left, cool mint rim light on the right, deep green (#1E4634) to near-black background. Behind the box five faint golden hair-thin threads of light drift upward, out of focus. 85 mm, f/2.8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; dark green band with gold text 'CELLULAR AGE' / 'DEFENSE 2.5%'; 'BIOSPICULE' / 'SERUM'; round medallion in a dark green ring with dark green spicules; gold-framed box: 'ADVANCED' / 'BIOSPICULE TECHNOLOGY'; bottom: '30 ml ℮ 1.0 fl.oz.'.</t>
         </is>
       </c>
       <c r="N44" s="5" t="inlineStr">
@@ -56828,7 +55720,7 @@
       </c>
       <c r="M47" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic still, 16:9. A woman in her fifties facing the camera as if it were her vanity mirror at night, warm lamp light from the left, deep green (#1E4634) shadowed room, natural un-retouched skin, two fingertips drawing a translucent serum upward along her jawline, the skin there faintly flushed. Composed, confident expression. Subject in the left two-thirds, right third dark. 50 mm, f/2, focus on the fingertips. No text, no logos, no visible packaging.</t>
+          <t>Photoreal cinematic still, 16:9. A woman in her fifties facing the camera as if it were her vanity mirror at night, warm lamp light from the left, deep green (#1E4634) shadowed room, natural un-retouched skin, two fingertips drawing a translucent serum upward along her jawline, the skin there faintly flushed. Composed, confident expression. Subject in the left two-thirds, right third dark. 50 mm, f/2, focus on the fingertips. No text, no logos, no visible packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; dark green band with gold text 'CELLULAR AGE' / 'DEFENSE 2.5%'; 'BIOSPICULE' / 'SERUM'; round medallion in a dark green ring with dark green spicules; gold-framed box: 'ADVANCED' / 'BIOSPICULE TECHNOLOGY'; bottom: '30 ml ℮ 1.0 fl.oz.'.</t>
         </is>
       </c>
       <c r="N47" s="5" t="inlineStr">
@@ -56903,7 +55795,7 @@
       </c>
       <c r="M48" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic still, 16:9. A dark polished vanity at night, deep green (#1E4634) wall, warm lamp light from the left with a cool mint edge light. Left to right, evenly spaced with room for captions above: a slim ivory box with a deep green band and a round thin-gold-rimmed spicule window (CELLULAR AGE DEFENSE 2.5%), a square ivory box with a deep green band and a printed white cream swirl (DERMA RECOVERY CREAM), an unbranded plain white sunscreen tube; slightly behind and out of focus a second slim ivory box of the same format (CELL RENEW 1.5%). 35 mm, f/5.6. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal cinematic still, 16:9. A dark polished vanity at night, deep green (#1E4634) wall, warm lamp light from the left with a cool mint edge light. Left to right, evenly spaced with room for captions above: a slim ivory box with a deep green band and a round thin-gold-rimmed spicule window (CELLULAR AGE DEFENSE 2.5%), a square ivory box with a deep green band and a printed white cream swirl (DERMA RECOVERY CREAM), an unbranded plain white sunscreen tube; slightly behind and out of focus a second slim ivory box of the same format (CELL RENEW 1.5%). 35 mm, f/5.6. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; dark green band with gold text 'CELLULAR AGE' / 'DEFENSE 2.5%'; 'BIOSPICULE' / 'SERUM'; round medallion in a dark green ring with dark green spicules; gold-framed box: 'ADVANCED' / 'BIOSPICULE TECHNOLOGY'; bottom: '30 ml ℮ 1.0 fl.oz.'.</t>
         </is>
       </c>
       <c r="N48" s="5" t="inlineStr">
@@ -56978,7 +55870,7 @@
       </c>
       <c r="M49" s="5" t="inlineStr">
         <is>
-          <t>Photoreal overhead flat-lay, 16:9. On a dark polished surface tinted deep green (#1E4634): the slim ivory MITODERM CELLULAR AGE DEFENSE 2.5% box (ivory, deep green band, round thin-gold-rimmed spicule window) lying flat, a single translucent drop of serum beside it catching warm lamp light, and five hair-thin golden light threads resting in a neat line on the surface. Generous negative space in the corners. 50 mm from directly above, f/8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal overhead flat-lay, 16:9. On a dark polished surface tinted deep green (#1E4634): the slim ivory MITODERM CELLULAR AGE DEFENSE 2.5% box (ivory, deep green band, round thin-gold-rimmed spicule window) lying flat, a single translucent drop of serum beside it catching warm lamp light, and five hair-thin golden light threads resting in a neat line on the surface. Generous negative space in the corners. 50 mm from directly above, f/8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; dark green band with gold text 'CELLULAR AGE' / 'DEFENSE 2.5%'; 'BIOSPICULE' / 'SERUM'; round medallion in a dark green ring with dark green spicules; gold-framed box: 'ADVANCED' / 'BIOSPICULE TECHNOLOGY'; bottom: '30 ml ℮ 1.0 fl.oz.'.</t>
         </is>
       </c>
       <c r="N49" s="5" t="inlineStr">
@@ -57053,7 +55945,7 @@
       </c>
       <c r="M50" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product still, 16:9. The ivory MITODERM CELLULAR AGE DEFENSE 2.5% box standing upright in the right third on a dark polished vanity, warm lamp light from the left, mint rim light on the right, a soft golden glow on the surface; slightly behind and out of focus a square ivory box with a deep green band (DERMA RECOVERY CREAM). Deep green (#1E4634) background. Left two-thirds empty. 85 mm, f/2.8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal cinematic product still, 16:9. The ivory MITODERM CELLULAR AGE DEFENSE 2.5% box standing upright in the right third on a dark polished vanity, warm lamp light from the left, mint rim light on the right, a soft golden glow on the surface; slightly behind and out of focus a square ivory box with a deep green band (DERMA RECOVERY CREAM). Deep green (#1E4634) background. Left two-thirds empty. 85 mm, f/2.8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TALL SLIM BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; dark green band with gold text 'CELLULAR AGE' / 'DEFENSE 2.5%'; 'BIOSPICULE' / 'SERUM'; round medallion in a dark green ring with dark green spicules; gold-framed box: 'ADVANCED' / 'BIOSPICULE TECHNOLOGY'; bottom: '30 ml ℮ 1.0 fl.oz.'.</t>
         </is>
       </c>
       <c r="N50" s="5" t="inlineStr">
@@ -57128,7 +56020,7 @@
       </c>
       <c r="M51" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product still, 16:9. A square ivory-cream cardboard box (MITODERM DERMA RECOVERY CREAM: ivory, a deep green horizontal band with gold lettering, a printed soft swirl of white cream below it, a small gold monogram at the top) standing in the right third on a smooth ivory surface, soft diffused daylight from the left, deep green (#1E4634) background. Behind it, out of focus, a slow spiralling swirl of white cream suspended in the air. Calm, comforting, premium. 85 mm, f/2.8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal cinematic product still, 16:9. A square ivory-cream cardboard box (MITODERM DERMA RECOVERY CREAM: ivory, a deep green horizontal band with gold lettering, a printed soft swirl of white cream below it, a small gold monogram at the top) standing in the right third on a smooth ivory surface, soft diffused daylight from the left, deep green (#1E4634) background. Behind it, out of focus, a slow spiralling swirl of white cream suspended in the air. Calm, comforting, premium. 85 mm, f/2.8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; dark green band with gold text 'DERMA RECOVERY' / 'CREAM'; 'SNAIL COLLAGEN'; white cream swirl illustration; gold-framed box: 'Daily nourishing collagen cream' / 'for healthy-looking glow'; bottom: '50 ml ℮ 1.69 fl.oz.'.</t>
         </is>
       </c>
       <c r="N51" s="5" t="inlineStr">
@@ -57353,7 +56245,7 @@
       </c>
       <c r="M54" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic still, 16:9. A woman in her forties the day after a cosmetic treatment, facing the camera as if it were her bathroom mirror, soft diffused morning light from the left, deep green (#1E4634) shadowed room. Her skin is natural and slightly pink; with two fingertips she smooths a small amount of white cream over her cheek, half of it already blended. Relaxed, relieved expression. Subject in the left two-thirds, right third dark. 50 mm, f/2, focus on the fingertips. No text, no logos, no visible packaging.</t>
+          <t>Photoreal cinematic still, 16:9. A woman in her forties the day after a cosmetic treatment, facing the camera as if it were her bathroom mirror, soft diffused morning light from the left, deep green (#1E4634) shadowed room. Her skin is natural and slightly pink; with two fingertips she smooths a small amount of white cream over her cheek, half of it already blended. Relaxed, relieved expression. Subject in the left two-thirds, right third dark. 50 mm, f/2, focus on the fingertips. No text, no logos, no visible packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; dark green band with gold text 'DERMA RECOVERY' / 'CREAM'; 'SNAIL COLLAGEN'; white cream swirl illustration; gold-framed box: 'Daily nourishing collagen cream' / 'for healthy-looking glow'; bottom: '50 ml ℮ 1.69 fl.oz.'.</t>
         </is>
       </c>
       <c r="N54" s="5" t="inlineStr">
@@ -57428,7 +56320,7 @@
       </c>
       <c r="M55" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic still, 16:9. A pale shelf against a deep green (#1E4634) wall, soft diffused light from the left. Left to right, evenly spaced with room for captions above: a tall slim ivory box with a deep green band and a round gold-rimmed spicule window (MICRO BOOST 10%), two slim ivory boxes with deep green bands and round thin-gold-rimmed spicule windows (CELL RENEW 1.5%, CELLULAR AGE DEFENSE 2.5%), and at the end a square ivory box with a deep green band and a printed white cream swirl (DERMA RECOVERY CREAM). All MITODERM family packaging, no other brands. 35 mm, f/5.6, all in focus. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal cinematic still, 16:9. A pale shelf against a deep green (#1E4634) wall, soft diffused light from the left. Left to right, evenly spaced with room for captions above: a tall slim ivory box with a deep green band and a round gold-rimmed spicule window (MICRO BOOST 10%), two slim ivory boxes with deep green bands and round thin-gold-rimmed spicule windows (CELL RENEW 1.5%, CELLULAR AGE DEFENSE 2.5%), and at the end a square ivory box with a deep green band and a printed white cream swirl (DERMA RECOVERY CREAM). All MITODERM family packaging, no other brands. 35 mm, f/5.6, all in focus. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; dark green band with gold text 'DERMA RECOVERY' / 'CREAM'; 'SNAIL COLLAGEN'; white cream swirl illustration; gold-framed box: 'Daily nourishing collagen cream' / 'for healthy-looking glow'; bottom: '50 ml ℮ 1.69 fl.oz.'.</t>
         </is>
       </c>
       <c r="N55" s="5" t="inlineStr">
@@ -57503,7 +56395,7 @@
       </c>
       <c r="M56" s="5" t="inlineStr">
         <is>
-          <t>Photoreal overhead flat-lay, 16:9. On a smooth ivory surface shaded deep green (#1E4634) at the edges: the square ivory MITODERM DERMA RECOVERY CREAM box (ivory, deep green band, printed white cream swirl) lying flat, and beside it a small smooth dollop of white cream. Soft diffused light, generous negative space in the four corners. 50 mm from directly above, f/8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal overhead flat-lay, 16:9. On a smooth ivory surface shaded deep green (#1E4634) at the edges: the square ivory MITODERM DERMA RECOVERY CREAM box (ivory, deep green band, printed white cream swirl) lying flat, and beside it a small smooth dollop of white cream. Soft diffused light, generous negative space in the four corners. 50 mm from directly above, f/8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; dark green band with gold text 'DERMA RECOVERY' / 'CREAM'; 'SNAIL COLLAGEN'; white cream swirl illustration; gold-framed box: 'Daily nourishing collagen cream' / 'for healthy-looking glow'; bottom: '50 ml ℮ 1.69 fl.oz.'.</t>
         </is>
       </c>
       <c r="N56" s="5" t="inlineStr">
@@ -57578,7 +56470,7 @@
       </c>
       <c r="M57" s="5" t="inlineStr">
         <is>
-          <t>Photoreal cinematic product still, 16:9. The square ivory MITODERM DERMA RECOVERY CREAM box standing upright in the right third on a smooth ivory surface, warm diffused light from the left, mint rim light on the right; slightly behind and out of focus a tall slim ivory box with a deep green band (MICRO BOOST 10%). Deep green (#1E4634) background. Left two-thirds empty. 85 mm, f/2.8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging.</t>
+          <t>Photoreal cinematic product still, 16:9. The square ivory MITODERM DERMA RECOVERY CREAM box standing upright in the right third on a smooth ivory surface, warm diffused light from the left, mint rim light on the right; slightly behind and out of focus a tall slim ivory box with a deep green band (MICRO BOOST 10%). Deep green (#1E4634) background. Left two-thirds empty. 85 mm, f/2.8. No people. No added text or overlays, no invented logos; only the printing that exists on the real packaging. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): BOX — ivory box, dark green and gold print: top: gold M monogram; 'MITODERM' letter-spaced, below 'BIOSPICULE SYSTEM'; dark green band with gold text 'DERMA RECOVERY' / 'CREAM'; 'SNAIL COLLAGEN'; white cream swirl illustration; gold-framed box: 'Daily nourishing collagen cream' / 'for healthy-looking glow'; bottom: '50 ml ℮ 1.69 fl.oz.'.</t>
         </is>
       </c>
       <c r="N57" s="5" t="inlineStr">
@@ -57653,7 +56545,7 @@
       </c>
       <c r="M58" s="5" t="inlineStr">
         <is>
-          <t>Background plate for compositing: a warm champagne-gold brushed-metal studio surface with a soft horizon gradient from pale champagne to deeper sand, one large soft key light from the upper left and a subtle warm rim from the right, faint metallic sheen, the right third kept empty for a slender champagne-gold cordless microneedling pen with a ribbed rose-copper adjustment ring, a small rose-copper button near the top and a clear needle cartridge at the tip, precision-instrument mood, 85 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Background plate for compositing: a warm champagne-gold brushed-metal studio surface with a soft horizon gradient from pale champagne to deeper sand, one large soft key light from the upper left and a subtle warm rim from the right, faint metallic sheen, the right third kept empty for a slender champagne-gold cordless microneedling pen with a ribbed rose-copper adjustment ring, a small rose-copper button near the top and a clear needle cartridge at the tip, precision-instrument mood, 85 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): MICRONEEDLING PEN — champagne-gold metal body, rose-gold knurled grip ring and button, clear needle cartridge: 'MITOPEN' printed vertically in white along the body; a small engraved V near the top cone.</t>
         </is>
       </c>
       <c r="N58" s="5" t="inlineStr">
@@ -57803,7 +56695,7 @@
       </c>
       <c r="M60" s="5" t="inlineStr">
         <is>
-          <t>Extreme macro of the tip of a slender champagne-gold cordless microneedling pen: a clear plastic needle cartridge with fine needle tips just extended, a ribbed rose-copper adjustment ring in the foreground, brushed champagne-metal barrel receding out of focus, warm soft key light with a cool rim to separate the clear plastic, champagne-beige background, precision-instrument mood, 100 mm macro, f/5.6, photoreal, cinematic, 16:9, no text, no numbers, no logos.</t>
+          <t>Extreme macro of the tip of a slender champagne-gold cordless microneedling pen: a clear plastic needle cartridge with fine needle tips just extended, a ribbed rose-copper adjustment ring in the foreground, brushed champagne-metal barrel receding out of focus, warm soft key light with a cool rim to separate the clear plastic, champagne-beige background, precision-instrument mood, 100 mm macro, f/5.6, photoreal, cinematic, 16:9, no text, no numbers, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): MICRONEEDLING PEN — champagne-gold metal body, rose-gold knurled grip ring and button, clear needle cartridge: 'MITOPEN' printed vertically in white along the body; a small engraved V near the top cone.</t>
         </is>
       </c>
       <c r="N60" s="5" t="inlineStr">
@@ -57878,7 +56770,7 @@
       </c>
       <c r="M61" s="5" t="inlineStr">
         <is>
-          <t>Aesthetic-clinic treatment scene: a practitioner in white nitrile gloves holding a slender champagne-gold cordless microneedling pen with a ribbed rose-copper ring, gliding it across the cheek of a reclined calm client whose eyes look toward the camera, warm soft clinical light, champagne and cream room tones, shallow depth of field on the pen and cheek, 50 mm, f/2.8, photoreal, cinematic, natural skin, 16:9, no text, no logos.</t>
+          <t>Aesthetic-clinic treatment scene: a practitioner in white nitrile gloves holding a slender champagne-gold cordless microneedling pen with a ribbed rose-copper ring, gliding it across the cheek of a reclined calm client whose eyes look toward the camera, warm soft clinical light, champagne and cream room tones, shallow depth of field on the pen and cheek, 50 mm, f/2.8, photoreal, cinematic, natural skin, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): MICRONEEDLING PEN — champagne-gold metal body, rose-gold knurled grip ring and button, clear needle cartridge: 'MITOPEN' printed vertically in white along the body; a small engraved V near the top cone.</t>
         </is>
       </c>
       <c r="N61" s="5" t="inlineStr">
@@ -57953,7 +56845,7 @@
       </c>
       <c r="M62" s="5" t="inlineStr">
         <is>
-          <t>Top-down view of a clinic treatment tray on a warm champagne-beige surface: a slender champagne-gold cordless microneedling pen with a ribbed rose-copper ring lying centred, empty space left and right of the pen for product packshots, white gauze and a glass dish at the edges, soft even clinical light, precise calm mood for a champagne-metal page, 50 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Top-down view of a clinic treatment tray on a warm champagne-beige surface: a slender champagne-gold cordless microneedling pen with a ribbed rose-copper ring lying centred, empty space left and right of the pen for product packshots, white gauze and a glass dish at the edges, soft even clinical light, precise calm mood for a champagne-metal page, 50 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): MICRONEEDLING PEN — champagne-gold metal body, rose-gold knurled grip ring and button, clear needle cartridge: 'MITOPEN' printed vertically in white along the body; a small engraved V near the top cone.</t>
         </is>
       </c>
       <c r="N62" s="5" t="inlineStr">
@@ -58028,7 +56920,7 @@
       </c>
       <c r="M63" s="5" t="inlineStr">
         <is>
-          <t>A slender champagne-gold cordless microneedling pen with a ribbed rose-copper ring and clear needle cartridge standing upright on a round brushed-champagne metal plinth, 3/4 view, warm soft key light from the upper left and a thin cool rim light, champagne-beige gradient background, left half of the frame empty for stat tiles, precision-instrument mood, 85 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>A slender champagne-gold cordless microneedling pen with a ribbed rose-copper ring and clear needle cartridge standing upright on a round brushed-champagne metal plinth, 3/4 view, warm soft key light from the upper left and a thin cool rim light, champagne-beige gradient background, left half of the frame empty for stat tiles, precision-instrument mood, 85 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): MICRONEEDLING PEN — champagne-gold metal body, rose-gold knurled grip ring and button, clear needle cartridge: 'MITOPEN' printed vertically in white along the body; a small engraved V near the top cone.</t>
         </is>
       </c>
       <c r="N63" s="5" t="inlineStr">
@@ -58103,7 +56995,7 @@
       </c>
       <c r="M64" s="5" t="inlineStr">
         <is>
-          <t>A slender champagne-gold cordless microneedling pen with a ribbed rose-copper ring resting at a 20° diagonal on a warm champagne brushed-metal surface, bright soft key light from the upper left, warm rim from the right, faint metallic sheen, left half of the frame empty for copy, premium closing shot for a champagne-metal page, 85 mm, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>A slender champagne-gold cordless microneedling pen with a ribbed rose-copper ring resting at a 20° diagonal on a warm champagne brushed-metal surface, bright soft key light from the upper left, warm rim from the right, faint metallic sheen, left half of the frame empty for copy, premium closing shot for a champagne-metal page, 85 mm, f/4, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): MICRONEEDLING PEN — champagne-gold metal body, rose-gold knurled grip ring and button, clear needle cartridge: 'MITOPEN' printed vertically in white along the body; a small engraved V near the top cone.</t>
         </is>
       </c>
       <c r="N64" s="5" t="inlineStr">
@@ -58178,7 +57070,7 @@
       </c>
       <c r="M65" s="5" t="inlineStr">
         <is>
-          <t>Background plate for compositing: a bright clinical white studio with a seamless white-to-pale-blue gradient, soft overhead daylight and a faint cool blue reflected glow on a white glossy tabletop at the right third of the frame (where a white tablet-style diagnostic monitor on a low stand, a white handheld scan probe with a coiled cable and a brushed-silver cylindrical base will be composited), subtle depth haze, 85 mm, f/5.6, low camera at table height, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>Background plate for compositing: a bright clinical white studio with a seamless white-to-pale-blue gradient, soft overhead daylight and a faint cool blue reflected glow on a white glossy tabletop at the right third of the frame (where a white tablet-style diagnostic monitor on a low stand, a white handheld scan probe with a coiled cable and a brushed-silver cylindrical base will be composited), subtle depth haze, 85 mm, f/5.6, low camera at table height, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TABLET — white tablet on a white stand, black screen: on screen: a teal-to-purple target logo, 'Mitoscan' in white, below 'By Mitoderm Ltd' || HANDHELD SCANNER — white handset with a black oval panel, white coiled cable: on the panel: 'Mitoscan' / 'By Mitoderm Ltd' in white || BASE — brushed silver cylinder with chrome ends: small chrome badge 'Mitoscan'.</t>
         </is>
       </c>
       <c r="N65" s="5" t="inlineStr">
@@ -58253,7 +57145,7 @@
       </c>
       <c r="M66" s="5" t="inlineStr">
         <is>
-          <t>Bright consultation room in an aesthetic clinic, white walls, daylight from a large window on the left, a white tablet-style diagnostic monitor on a low stand turned toward an empty white client chair, a white handheld scan probe resting on the desk, cool blue glow on the wall from the screen, clean white-and-blue grade, calm honest mood, 35 mm, f/4, photoreal, cinematic, 16:9, no text, no logos, screen content blurred.</t>
+          <t>Bright consultation room in an aesthetic clinic, white walls, daylight from a large window on the left, a white tablet-style diagnostic monitor on a low stand turned toward an empty white client chair, a white handheld scan probe resting on the desk, cool blue glow on the wall from the screen, clean white-and-blue grade, calm honest mood, 35 mm, f/4, photoreal, cinematic, 16:9, no text, no logos, screen content blurred. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TABLET — white tablet on a white stand, black screen: on screen: a teal-to-purple target logo, 'Mitoscan' in white, below 'By Mitoderm Ltd' || HANDHELD SCANNER — white handset with a black oval panel, white coiled cable: on the panel: 'Mitoscan' / 'By Mitoderm Ltd' in white || BASE — brushed silver cylinder with chrome ends: small chrome badge 'Mitoscan'.</t>
         </is>
       </c>
       <c r="N66" s="5" t="inlineStr">
@@ -58403,7 +57295,7 @@
       </c>
       <c r="M68" s="5" t="inlineStr">
         <is>
-          <t>Aesthetic-clinic consultation: a practitioner in a white coat holds a white handheld scan probe against the parting of a seated client's dark hair and points to a white tablet-style monitor showing an abstract magnified scalp image, the client looking at the screen with interest, bright daylight room, cool blue screen glow on their faces, white-and-blue grade, 35 mm, f/2.8, photoreal, cinematic, natural skin and hair, 16:9, no text, no logos.</t>
+          <t>Aesthetic-clinic consultation: a practitioner in a white coat holds a white handheld scan probe against the parting of a seated client's dark hair and points to a white tablet-style monitor showing an abstract magnified scalp image, the client looking at the screen with interest, bright daylight room, cool blue screen glow on their faces, white-and-blue grade, 35 mm, f/2.8, photoreal, cinematic, natural skin and hair, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TABLET — white tablet on a white stand, black screen: on screen: a teal-to-purple target logo, 'Mitoscan' in white, below 'By Mitoderm Ltd' || HANDHELD SCANNER — white handset with a black oval panel, white coiled cable: on the panel: 'Mitoscan' / 'By Mitoderm Ltd' in white || BASE — brushed silver cylinder with chrome ends: small chrome badge 'Mitoscan'.</t>
         </is>
       </c>
       <c r="N68" s="5" t="inlineStr">
@@ -58478,7 +57370,7 @@
       </c>
       <c r="M69" s="5" t="inlineStr">
         <is>
-          <t>Top-down view of a white clinic desk: a white tablet-style diagnostic monitor on a low stand glowing faintly blue, a white handheld scan probe with a coiled cable docked beside it, a brushed-silver cylindrical base unit, empty white space along the bottom of the frame for three cards, soft even daylight, clean white-and-blue grade, 50 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos, screen content blurred.</t>
+          <t>Top-down view of a white clinic desk: a white tablet-style diagnostic monitor on a low stand glowing faintly blue, a white handheld scan probe with a coiled cable docked beside it, a brushed-silver cylindrical base unit, empty white space along the bottom of the frame for three cards, soft even daylight, clean white-and-blue grade, 50 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos, screen content blurred. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TABLET — white tablet on a white stand, black screen: on screen: a teal-to-purple target logo, 'Mitoscan' in white, below 'By Mitoderm Ltd' || HANDHELD SCANNER — white handset with a black oval panel, white coiled cable: on the panel: 'Mitoscan' / 'By Mitoderm Ltd' in white || BASE — brushed silver cylinder with chrome ends: small chrome badge 'Mitoscan'.</t>
         </is>
       </c>
       <c r="N69" s="5" t="inlineStr">
@@ -58553,7 +57445,7 @@
       </c>
       <c r="M70" s="5" t="inlineStr">
         <is>
-          <t>A white tablet-style diagnostic monitor on a low white stand showing an abstract magnified scalp image, a white handheld scan probe with a coiled white cable docked at its right, a brushed-silver cylindrical base unit with chrome ends in front, all on a white plinth, 3/4 view, soft daylight with a cool blue screen glow, white-to-pale-blue background, left half of the frame empty for stat tiles, 85 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>A white tablet-style diagnostic monitor on a low white stand showing an abstract magnified scalp image, a white handheld scan probe with a coiled white cable docked at its right, a brushed-silver cylindrical base unit with chrome ends in front, all on a white plinth, 3/4 view, soft daylight with a cool blue screen glow, white-to-pale-blue background, left half of the frame empty for stat tiles, 85 mm, f/5.6, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TABLET — white tablet on a white stand, black screen: on screen: a teal-to-purple target logo, 'Mitoscan' in white, below 'By Mitoderm Ltd' || HANDHELD SCANNER — white handset with a black oval panel, white coiled cable: on the panel: 'Mitoscan' / 'By Mitoderm Ltd' in white || BASE — brushed silver cylinder with chrome ends: small chrome badge 'Mitoscan'.</t>
         </is>
       </c>
       <c r="N70" s="5" t="inlineStr">
@@ -58628,7 +57520,7 @@
       </c>
       <c r="M71" s="5" t="inlineStr">
         <is>
-          <t>A white tablet-style diagnostic monitor on a low stand glowing cool blue with an abstract magnified scalp image, a white handheld scan probe docked at its right and a brushed-silver cylindrical base in front, on a white glossy tabletop, bright soft daylight, white-to-pale-blue gradient background, left half of the frame empty for copy, premium closing shot for a white-and-blue page, 85 mm, f/4, photoreal, cinematic, 16:9, no text, no logos.</t>
+          <t>A white tablet-style diagnostic monitor on a low stand glowing cool blue with an abstract magnified scalp image, a white handheld scan probe docked at its right and a brushed-silver cylindrical base in front, on a white glossy tabletop, bright soft daylight, white-to-pale-blue gradient background, left half of the frame empty for copy, premium closing shot for a white-and-blue page, 85 mm, f/4, photoreal, cinematic, 16:9, no text, no logos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): TABLET — white tablet on a white stand, black screen: on screen: a teal-to-purple target logo, 'Mitoscan' in white, below 'By Mitoderm Ltd' || HANDHELD SCANNER — white handset with a black oval panel, white coiled cable: on the panel: 'Mitoscan' / 'By Mitoderm Ltd' in white || BASE — brushed silver cylinder with chrome ends: small chrome badge 'Mitoscan'.</t>
         </is>
       </c>
       <c r="N71" s="5" t="inlineStr">
@@ -60278,7 +59170,7 @@
       </c>
       <c r="M93" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal cinematic product hero, 16:9. A near-square carton, slightly wider than tall, finished in a champagne-gold gradient (pale warm ivory at the top left to deep gold at the right) standing on the right third on a warm cream stone surface; in front of it three vessels: a small amber glass vial with a silver cap, a small turquoise-blue glass vial with a silver cap, and a square clear glass bottle with a tall gold cap holding a pale liquid with fine gold flecks. Background: soft champagne (#F3E4C2) gradient, warm sunlight from the upper left, long soft shadows, subtle warm bloom. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds clear for text. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal cinematic product hero, 16:9. A near-square carton, slightly wider than tall, finished in a champagne-gold gradient (pale warm ivory at the top left to deep gold at the right) standing on the right third on a warm cream stone surface; in front of it three vessels: a small amber glass vial with a silver cap, a small turquoise-blue glass vial with a silver cap, and a square clear glass bottle with a tall gold cap holding a pale liquid with fine gold flecks. Background: soft champagne (#F3E4C2) gradient, warm sunlight from the upper left, long soft shadows, subtle warm bloom. Camera: 85 mm, eye level, f/4, product sharp, left two-thirds clear for text. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): SQUARE BOX — brushed gold gradient box with a thin lid line near the bottom, black print: top centre: VM monogram, 'VM corporation'; centre: 'EXO-NAD' ('EXO-' thin, 'NAD' bold); below: letter-spaced 'SKIN LONGEVITY PEELING' || PEEL BOTTLE — clear square glass bottle with a gold cap, gold flakes in the liquid: 'EXO-NAD'; 'SKIN LONGEVITY PEELING' || AMBER VIAL — amber glass vial, silver crimp cap: VM monogram; 'PH NORMALIZER' bold white || TEAL VIAL — blue-teal glass vial, silver crimp cap: VM monogram; 'LONGEVITY SERUM' bold white.</t>
         </is>
       </c>
       <c r="N93" s="5" t="inlineStr">
@@ -60428,7 +59320,7 @@
       </c>
       <c r="M95" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal macro still life, 16:9. Three vessels in a row on warm cream stone under sunlight: left, a square clear glass bottle with a tall gold cap holding a pale liquid with fine gold flecks; centre, a small amber glass vial with a silver cap; right, a small turquoise-blue glass vial with a silver cap; behind each an out-of-focus macro swirl of its liquid — behind the bottle, a clear oily phase floating over a watery, fleck-filled phase. Lighting: warm champagne (#F3E4C2) backdrop, strong sun from the left, gold flecks sparkling. Camera: 100 mm macro, f/4, vessels sharp. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal macro still life, 16:9. Three vessels in a row on warm cream stone under sunlight: left, a square clear glass bottle with a tall gold cap holding a pale liquid with fine gold flecks; centre, a small amber glass vial with a silver cap; right, a small turquoise-blue glass vial with a silver cap; behind each an out-of-focus macro swirl of its liquid — behind the bottle, a clear oily phase floating over a watery, fleck-filled phase. Lighting: warm champagne (#F3E4C2) backdrop, strong sun from the left, gold flecks sparkling. Camera: 100 mm macro, f/4, vessels sharp. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): SQUARE BOX — brushed gold gradient box with a thin lid line near the bottom, black print: top centre: VM monogram, 'VM corporation'; centre: 'EXO-NAD' ('EXO-' thin, 'NAD' bold); below: letter-spaced 'SKIN LONGEVITY PEELING' || PEEL BOTTLE — clear square glass bottle with a gold cap, gold flakes in the liquid: 'EXO-NAD'; 'SKIN LONGEVITY PEELING' || AMBER VIAL — amber glass vial, silver crimp cap: VM monogram; 'PH NORMALIZER' bold white || TEAL VIAL — blue-teal glass vial, silver crimp cap: VM monogram; 'LONGEVITY SERUM' bold white.</t>
         </is>
       </c>
       <c r="N95" s="5" t="inlineStr">
@@ -60578,7 +59470,7 @@
       </c>
       <c r="M97" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal top-down flat lay, 16:9. On warm cream stone, left to right in a straight row with space between: a square clear glass bottle with a tall gold cap and pale gold-flecked liquid, a fan brush, a small amber vial with a silver cap, a small turquoise vial with a silver cap, then a folded translucent pale-blue sheet mask lying in front of a small matte teal carton and a plain white unbranded sunscreen tube. Lighting: sunlight from the upper left, long soft shadows, champagne (#F3E4C2) tone. Camera: overhead, 50 mm, f/8, all sharp. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal top-down flat lay, 16:9. On warm cream stone, left to right in a straight row with space between: a square clear glass bottle with a tall gold cap and pale gold-flecked liquid, a fan brush, a small amber vial with a silver cap, a small turquoise vial with a silver cap, then a folded translucent pale-blue sheet mask lying in front of a small matte teal carton and a plain white unbranded sunscreen tube. Lighting: sunlight from the upper left, long soft shadows, champagne (#F3E4C2) tone. Camera: overhead, 50 mm, f/8, all sharp. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): SQUARE BOX — brushed gold gradient box with a thin lid line near the bottom, black print: top centre: VM monogram, 'VM corporation'; centre: 'EXO-NAD' ('EXO-' thin, 'NAD' bold); below: letter-spaced 'SKIN LONGEVITY PEELING' || PEEL BOTTLE — clear square glass bottle with a gold cap, gold flakes in the liquid: 'EXO-NAD'; 'SKIN LONGEVITY PEELING' || AMBER VIAL — amber glass vial, silver crimp cap: VM monogram; 'PH NORMALIZER' bold white || TEAL VIAL — blue-teal glass vial, silver crimp cap: VM monogram; 'LONGEVITY SERUM' bold white.</t>
         </is>
       </c>
       <c r="N97" s="5" t="inlineStr">
@@ -60653,7 +59545,7 @@
       </c>
       <c r="M98" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal product shot, 16:9. The champagne-gold gradient near-square carton, closed, in three-quarter view on the left; beside it on cream stone, laid out neatly: one square clear glass bottle with a tall gold cap and gold-flecked liquid, a row of five small amber vials with silver caps and a row of five small turquoise-blue vials with silver caps. Lighting: warm sunlight from the upper right, soft champagne backdrop, gentle bloom. Camera: 70 mm, f/5.6, everything sharp, right third clear for numbers. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal product shot, 16:9. The champagne-gold gradient near-square carton, closed, in three-quarter view on the left; beside it on cream stone, laid out neatly: one square clear glass bottle with a tall gold cap and gold-flecked liquid, a row of five small amber vials with silver caps and a row of five small turquoise-blue vials with silver caps. Lighting: warm sunlight from the upper right, soft champagne backdrop, gentle bloom. Camera: 70 mm, f/5.6, everything sharp, right third clear for numbers. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): SQUARE BOX — brushed gold gradient box with a thin lid line near the bottom, black print: top centre: VM monogram, 'VM corporation'; centre: 'EXO-NAD' ('EXO-' thin, 'NAD' bold); below: letter-spaced 'SKIN LONGEVITY PEELING' || PEEL BOTTLE — clear square glass bottle with a gold cap, gold flakes in the liquid: 'EXO-NAD'; 'SKIN LONGEVITY PEELING' || AMBER VIAL — amber glass vial, silver crimp cap: VM monogram; 'PH NORMALIZER' bold white || TEAL VIAL — blue-teal glass vial, silver crimp cap: VM monogram; 'LONGEVITY SERUM' bold white.</t>
         </is>
       </c>
       <c r="N98" s="5" t="inlineStr">
@@ -60728,7 +59620,7 @@
       </c>
       <c r="M99" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal cinematic closing hero, 16:9. The champagne-gold near-square carton on the right third on cream stone, the three vessels (small amber vial, small turquoise vial, square gold-capped bottle with gold-flecked liquid) in front, warm sunlight from the left, soft bloom, a thin gold reflection line; the left two-thirds clean champagne (#F3E4C2) for the offer and buttons. Camera: 85 mm, eye level, f/4. Warm, calm, final. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible.</t>
+          <t>REFERENCE IMAGE: attach the product photo mitoderm-catalog/protocols/assets/img/exo-nad.webp. Photoreal cinematic closing hero, 16:9. The champagne-gold near-square carton on the right third on cream stone, the three vessels (small amber vial, small turquoise vial, square gold-capped bottle with gold-flecked liquid) in front, warm sunlight from the left, soft bloom, a thin gold reflection line; the left two-thirds clean champagne (#F3E4C2) for the offer and buttons. Camera: 85 mm, eye level, f/4. Warm, calm, final. No overlay text or captions; no text other than the packaging's own printing; the packaging reproduced exactly from the attached packshot photo (mitoderm-catalog/protocols/assets/img/exo-nad.webp): same colours, wordmark and every printed word spelled as on the pack, crisp and legible. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): SQUARE BOX — brushed gold gradient box with a thin lid line near the bottom, black print: top centre: VM monogram, 'VM corporation'; centre: 'EXO-NAD' ('EXO-' thin, 'NAD' bold); below: letter-spaced 'SKIN LONGEVITY PEELING' || PEEL BOTTLE — clear square glass bottle with a gold cap, gold flakes in the liquid: 'EXO-NAD'; 'SKIN LONGEVITY PEELING' || AMBER VIAL — amber glass vial, silver crimp cap: VM monogram; 'PH NORMALIZER' bold white || TEAL VIAL — blue-teal glass vial, silver crimp cap: VM monogram; 'LONGEVITY SERUM' bold white.</t>
         </is>
       </c>
       <c r="N99" s="5" t="inlineStr">
@@ -60803,7 +59695,7 @@
       </c>
       <c r="M100" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGES: attach the EXOCELL MASK box photo. Copy the carton exactly from the attached box photo: its colour, the VM monogram with 'VM corporation', the 'EXOCELL' wordmark ('EXO' bold, 'CELL' thin) with letter-spaced 'MASK' beneath, and the small multilingual text block near the bottom — every word spelled exactly as on that box, crisp and legible; add no line that is not on the reference. Photoreal cinematic product hero, 16:9, 4K. SET (identical in every key frame): a polished black glass counter in a near-black studio (#0b0f10), no haze. CARTON: upright on the glass in the right third, about 45% of the frame height, turned about 20 degrees so its left side panel shows (three-quarter view). SHEET: in front of the carton and to its left, not touching it, one unfolded bio-cellulose face mask: a thin, wet, translucent milky-white film with a faint aqua tint, eye, nose and mouth cut-outs, fine water droplets, lying almost flat on the glass with its upper edge lifted a few centimetres toward the camera. LIGHT (identical in every key frame): one soft teal (#6fb7ba) key from the upper left, a faint neutral fill from the front, a thin teal rim on the sheet edge, the carton softly reflected in the glass. CAMERA: 85 mm, eye level, f/8, carton and sheet sharp; the left half of the frame empty near-black for text. No people, no hands. No captions or overlay text, no text other than the packaging's own print, no extra objects.</t>
+          <t>REFERENCE IMAGES: attach the EXOCELL MASK box photo. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): CARTON (MAIN PHOTO VERSION) — matte muted-teal portrait carton (#5ca0a5), dark navy print: top centre: VM monogram, below it small 'VM corporation'; centre: 'EXOCELL' in wide-spaced capitals ('EXO' bold, 'CELL' thin), below it letter-spaced 'M A S K'; below the middle, light italic pale aqua, two lines: 'Your Second Skin' / 'For Exo Bio-Regeneration'; small block, first line bold: 'Professional facial moisturizing mask' / 'Maschera viso idratante ad uso professionale' / 'Mascarilla hidratante facial profesional' / 'Masque hydratant visage professionnel'; bottom two lines: '5 face masks – maschere viso - máscaras facial - masques facial' / 'Net 5 x 25 ml ℮ 5 x 0.84 fl.oz'; left side panel: 'EXOCELL' and 'MASK' running vertically, grey || SHEET MASK — translucent milky-white bio-cellulose, faint aqua tint, eye, nose and mouth cut-outs, a small slit at the right jaw; pale-blue protective film. Photoreal cinematic product hero, 16:9, 4K. SET (identical in every key frame): a polished black glass counter in a near-black studio (#0b0f10), no haze. CARTON: upright on the glass in the right third, about 45% of the frame height, turned about 20 degrees so its left side panel shows (three-quarter view). SHEET: in front of the carton and to its left, not touching it, one unfolded bio-cellulose face mask: a thin, wet, translucent milky-white film with a faint aqua tint, eye, nose and mouth cut-outs, fine water droplets, lying almost flat on the glass with its upper edge lifted a few centimetres toward the camera. LIGHT (identical in every key frame): one soft teal (#6fb7ba) key from the upper left, a faint neutral fill from the front, a thin teal rim on the sheet edge, the carton softly reflected in the glass. CAMERA: 85 mm, eye level, f/8, carton and sheet sharp; the left half of the frame empty near-black for text. No people, no hands. No captions or overlay text, no text other than the packaging's own print, no extra objects.</t>
         </is>
       </c>
       <c r="N100" s="5" t="inlineStr">
@@ -60953,7 +59845,7 @@
       </c>
       <c r="M102" s="5" t="inlineStr">
         <is>
-          <t>Branch A only. REFERENCE IMAGES: attach the EXOCELL MASK box photo and the hero frame. Photoreal macro still, 16:9, 4K — the same set and light as the hero, nothing moved. CAMERA: 100 mm macro, f/4, pushed in close to the sheet on the black glass: in focus, the lifted edge of the translucent milky-white bio-cellulose film (faint aqua tint) and one eye cut-out, its fine fibrous translucency and water droplets catching the teal light; the carton stands where it stood, softly out of focus at the right edge, its print as on the box photo. No people, no hands. No captions or overlay text, no text other than the packaging's own print, no floating fibres, no vesicle or particle illustrations.</t>
+          <t>Branch A only. REFERENCE IMAGES: attach the EXOCELL MASK box photo and the hero frame. Photoreal macro still, 16:9, 4K — the same set and light as the hero, nothing moved. CAMERA: 100 mm macro, f/4, pushed in close to the sheet on the black glass: in focus, the lifted edge of the translucent milky-white bio-cellulose film (faint aqua tint) and one eye cut-out, its fine fibrous translucency and water droplets catching the teal light; the carton stands where it stood, softly out of focus at the right edge, its print as on the box photo. No people, no hands. No captions or overlay text, no text other than the packaging's own print, no floating fibres, no vesicle or particle illustrations. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): CARTON (MAIN PHOTO VERSION) — matte muted-teal portrait carton (#5ca0a5), dark navy print: top centre: VM monogram, below it small 'VM corporation'; centre: 'EXOCELL' in wide-spaced capitals ('EXO' bold, 'CELL' thin), below it letter-spaced 'M A S K'; below the middle, light italic pale aqua, two lines: 'Your Second Skin' / 'For Exo Bio-Regeneration'; small block, first line bold: 'Professional facial moisturizing mask' / 'Maschera viso idratante ad uso professionale' / 'Mascarilla hidratante facial profesional' / 'Masque hydratant visage professionnel'; bottom two lines: '5 face masks – maschere viso - máscaras facial - masques facial' / 'Net 5 x 25 ml ℮ 5 x 0.84 fl.oz'; left side panel: 'EXOCELL' and 'MASK' running vertically, grey || SHEET MASK — translucent milky-white bio-cellulose, faint aqua tint, eye, nose and mouth cut-outs, a small slit at the right jaw; pale-blue protective film.</t>
         </is>
       </c>
       <c r="N102" s="5" t="inlineStr">
@@ -61028,7 +59920,7 @@
       </c>
       <c r="M103" s="5" t="inlineStr">
         <is>
-          <t>Branch B. REFERENCE IMAGES: attach the EXOCELL MASK box photo and the treatment photos. Copy the carton exactly from the attached box photo: its colour, the VM monogram with 'VM corporation', the 'EXOCELL' wordmark ('EXO' bold, 'CELL' thin) with letter-spaced 'MASK' beneath, and the small multilingual text block near the bottom — every word spelled exactly as on that box, crisp and legible; add no line that is not on the reference. Photoreal cinematic treatment scene, 16:9, 4K, the same teal light as the hero. A woman in her thirties reclines on a treatment bed, eyes closed, calm, hair under a black disposable cap; a bio-cellulose sheet mask lies smoothly on her face — on skin it turns almost clear and milky, eye and mouth cut-outs sitting precisely, minimal air pockets, a few droplets; a practitioner's hands in black nitrile gloves peel the pale-blue protective backing film away from the mask at the forehead. In the right third, on a black glass side table at shoulder height, the EXOCELL MASK carton, about 35% of the frame height, turned 20 degrees to show its left side panel. CAMERA: 50 mm, slightly above, f/4, face, sheet and carton sharp; the left third darker for text. Realistic skin texture, no redness, no retouched plastic skin. No captions or overlay text, no text other than the packaging's own print, no purple, no extra people.  ||  Branch B alternative (mirror with sachet): REFERENCE IMAGES: attach the sachet photo and the mirror photo. Photoreal portrait, 16:9, 4K, minimal clinic washroom with black walls and the same soft teal light. A woman in her thirties, dark hair pulled back, freshly treated calm skin, faces the camera as if it were her mirror and holds one sealed single-mask sachet at shoulder height on the right, its front toward the camera and readable; the sachet is copied exactly from the attached sachet photo (pale-aqua foil with the VM monogram and 'EXOCELL MASK' printed on the front). CAMERA: 50 mm, f/2.8, face and sachet sharp; left half dark for text. No captions or overlay text, no text other than the packaging's own print, no mirror frame, no extra objects.</t>
+          <t>Branch B. REFERENCE IMAGES: attach the EXOCELL MASK box photo and the treatment photos. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): CARTON (MAIN PHOTO VERSION) — matte muted-teal portrait carton (#5ca0a5), dark navy print: top centre: VM monogram, below it small 'VM corporation'; centre: 'EXOCELL' in wide-spaced capitals ('EXO' bold, 'CELL' thin), below it letter-spaced 'M A S K'; below the middle, light italic pale aqua, two lines: 'Your Second Skin' / 'For Exo Bio-Regeneration'; small block, first line bold: 'Professional facial moisturizing mask' / 'Maschera viso idratante ad uso professionale' / 'Mascarilla hidratante facial profesional' / 'Masque hydratant visage professionnel'; bottom two lines: '5 face masks – maschere viso - máscaras facial - masques facial' / 'Net 5 x 25 ml ℮ 5 x 0.84 fl.oz'; left side panel: 'EXOCELL' and 'MASK' running vertically, grey || SHEET MASK — translucent milky-white bio-cellulose, faint aqua tint, eye, nose and mouth cut-outs, a small slit at the right jaw; pale-blue protective film. Photoreal cinematic treatment scene, 16:9, 4K, the same teal light as the hero. A woman in her thirties reclines on a treatment bed, eyes closed, calm, hair under a black disposable cap; a bio-cellulose sheet mask lies smoothly on her face — on skin it turns almost clear and milky, eye and mouth cut-outs sitting precisely, minimal air pockets, a few droplets; a practitioner's hands in black nitrile gloves peel the pale-blue protective backing film away from the mask at the forehead. In the right third, on a black glass side table at shoulder height, the EXOCELL MASK carton, about 35% of the frame height, turned 20 degrees to show its left side panel. CAMERA: 50 mm, slightly above, f/4, face, sheet and carton sharp; the left third darker for text. Realistic skin texture, no redness, no retouched plastic skin. No captions or overlay text, no text other than the packaging's own print, no purple, no extra people.  ||  Branch B alternative (mirror with sachet): REFERENCE IMAGES: attach the sachet photo and the mirror photo. Photoreal portrait, 16:9, 4K, minimal clinic washroom with black walls and the same soft teal light. A woman in her thirties, dark hair pulled back, freshly treated calm skin, faces the camera as if it were her mirror and holds one sealed single-mask sachet at shoulder height on the right, its front toward the camera and readable; the sachet is copied exactly from the attached sachet photo (pale-aqua foil with the VM monogram and 'EXOCELL MASK' printed on the front). CAMERA: 50 mm, f/2.8, face and sachet sharp; left half dark for text. No captions or overlay text, no text other than the packaging's own print, no mirror frame, no extra objects. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): SINGLE-MASK SACHET — pale aqua foil sachet: VM monogram top centre; 'EXOCELL' / letter-spaced 'MASK'; [unreadable] two tiny lines near the bottom.</t>
         </is>
       </c>
       <c r="N103" s="5" t="inlineStr">
@@ -61178,7 +60070,7 @@
       </c>
       <c r="M105" s="5" t="inlineStr">
         <is>
-          <t>REFERENCE IMAGES: attach the EXOCELL MASK box photo and the sachet photo. Copy the carton exactly from the attached box photo: its colour, the VM monogram with 'VM corporation', the 'EXOCELL' wordmark ('EXO' bold, 'CELL' thin) with letter-spaced 'MASK' beneath, and the small multilingual text block near the bottom — every word spelled exactly as on that box, crisp and legible; add no line that is not on the reference. Photoreal product still life, 16:9, 4K — the same black glass set and teal light as the hero, camera raised about 20 degrees above the counter. The carton stands in the right third at the same scale as the hero (about 45% of the frame height), turned 20 degrees to show its left side panel; in front of it, five sealed single-mask sachets fan out across the glass, the front one slightly lifted; the sachets are copied exactly from the attached sachet photo (pale-aqua foil with the VM monogram and 'EXOCELL MASK' printed on the front); droplets on the glass. Left half empty near-black for numbers. No people, no hands. No captions or overlay text, no text other than the packaging's own print, no extra objects.</t>
+          <t>REFERENCE IMAGES: attach the EXOCELL MASK box photo and the sachet photo. PACKAGING TEXT — reproduce exactly as listed, every word spelled exactly as written here, crisp and legible, nothing added or translated (lines marked [unreadable] are tiny grey lines, not words): CARTON (MAIN PHOTO VERSION) — matte muted-teal portrait carton (#5ca0a5), dark navy print: top centre: VM monogram, below it small 'VM corporation'; centre: 'EXOCELL' in wide-spaced capitals ('EXO' bold, 'CELL' thin), below it letter-spaced 'M A S K'; below the middle, light italic pale aqua, two lines: 'Your Second Skin' / 'For Exo Bio-Regeneration'; small block, first line bold: 'Professional facial moisturizing mask' / 'Maschera viso idratante ad uso professionale' / 'Mascarilla hidratante facial profesional' / 'Masque hydratant visage professionnel'; bottom two lines: '5 face masks – maschere viso - máscaras facial - masques facial' / 'Net 5 x 25 ml ℮ 5 x 0.84 fl.oz'; left side panel: 'EXOCELL' and 'MASK' running vertically, grey || SINGLE-MASK SACHET — pale aqua foil sachet: VM monogram top centre; 'EXOCELL' / letter-spaced 'MASK'; [unreadable] two tiny lines near the bottom || SHEET MASK — translucent milky-white bio-cellulose, faint aqua tint, eye, nose and mouth cut-outs, a small slit at the right jaw; pale-blue protective film. Photoreal product still life, 16:9, 4K — the same black glass set and teal light as the hero, camera raised about 20 degrees above the counter. The carton stands in the right third at the same scale as the hero (about 45% of the frame height), turned 20 degrees to show its left side panel; in front of it, five sealed single-mask sachets fan out across the glass, the front one slightly lifted; the sachets are copied exactly from the attached sachet photo (pale-aqua foil with the VM monogram and 'EXOCELL MASK' printed on the front); droplets on the glass. Left half empty near-black for numbers. No people, no hands. No captions or overlay text, no text other than the packaging's own print, no extra objects.</t>
         </is>
       </c>
       <c r="N105" s="5" t="inlineStr">
@@ -61264,6 +60156,1114 @@
       <c r="O106" s="5" t="inlineStr">
         <is>
           <t>Packshot small (≈35 vh) above the headline; two full-width buttons; contact row; sticky bar becomes the primary button.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Block</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Purchase</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Truth</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Brevity</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Meet</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Хедер работает: продукт, «вторая кожа», «после процедуры» прослеживаются к спеке и стр. 10. Натяжка — чип «Instant cooling» (в каталоге immediate — про гидратацию, cooling отдельно); сложенная пополам маска — выдуманный элемент, биоцеллюлоза должна читаться как реальный лист.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Meet</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Строка повторяет eyebrow и hero_sub, чипы повторяют строку — три слоя одного в одном экране. «After every professional treatment» шире каталога (стр. 10: «after professional cosmetic treatments»). Сложенная маска придумана — спорит с реальным пакшотом, где лист раскрыт.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Meet</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>«Your second skin» пишет каждая биоцеллюлозная маска на рынке; наш единственный дифференциатор — синтетические экзосомальные структуры VM — задвинут в чип. «After every» — переобещание, каталог говорит «after professional cosmetic treatments».</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Meet</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Позиционирование и primary CTA на месте, но H1 без имени продукта и без ключа «bio-cellulose mask» — пусто для SEO; имя EXOCELL MASK впервые появляется в последнем блоке. «Every» — усиление спеки. Сложенная маска — осознанно выдуманный элемент, допустимо ради переходов.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Чипы «After V-TECH / EXO-NAD / MICRO BOOST / microneedling» — ровно то, что я проверяю перед заказом, и они прослеживаются (стр. 7, 9, 19). Но покрасневшее лицо с точечными следами на странице про успокоение — риск; маска, висящая в воздухе у лица, странна; «decides how your client walks out» — продающая отсебятина.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Слово «after» шесть раз в блоке; второе предложение — риторика, в каталоге нет; чипы дублируют ряд блока 4. Кадр — медицинская иллюстрация, не продукт-герой. Делать типографикой на бирюзе, чипы = ссылки, без генерации.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Четыре чипа — самое сильное B2B-место страницы (маска продаётся как завершение наших же протоколов), но вторая фраза ничем не подтверждена, а румянец и «pinpoint marks» на генеративном лице рискуют выглядеть как осложнение. Уместнее три реальных пакшота протоколов и лист маски.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Текст говорит с владельцем клиники на его языке, чипы — правильный внутренний граф ссылок на PRO-страницы. Кадр — самый рискованный на странице (медицина / uncanny valley), продукта в кадре фактически нет. Фраза про «walks out» — риторика, не свойство.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Inside</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Состав честный (все 8 ингредиентов из стр. 10) и это то, что я реально читаю, но строка — перечисление, чипы 3 и 4 составные; «сфера-везикула среди волокон» — клише, которому профессионал не верит; единственный кадр без продукта. Концентраций нет — спрошу у поставщика.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Inside</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Состав перечислен трижды (строка, четыре составных чипа, подпись); «adheres with minimal air pockets» повторяется в блоке 4; «soaked» — не из источников (там «active serum»). «Везикула» в макро — псевдонаука. Текстуру дать кропом реального пакшота.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Inside</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Текст дословно из каталога, но блок перегружен; «увеличенная везикула» — научная неточность, которую заметит любой врач: наноразмерные структуры не видны рядом с волокнами целлюлозы. У бренда «where science meets beauty» такого кадра быть не должно.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Inside</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Каждое слово из стр. 10 — плюс, но это стена из 14 ингредиентов, здесь владелец клиники начнёт пролистывать; «Full formula ↓» никуда не ведёт. Оставить два дифференциатора (экзосомы, полинуклеотиды), остальное — в раскрывающийся список. Макро без лиц — снимаемый кадр.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Feel it</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Каждое слово из каталога, но семь прилагательных через запятую дублируют четыре чипа, чипы дублируют хедер; ничто не двигает к заказу. Пин «Smoothing &amp; firming» на шее намекает на шею, чего в каталоге нет. Кадр с маской на лице — лучший на странице, оставить.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Feel it</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Строка — весь абзац Key Benefits через точку с запятой и дублирует чипы и заголовок; одна фраза должна остаться одной. Пины держать на лице — каталог шею не упоминает. Единственный кадр с человеком — оставить: маска на лице = продукт на коже.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Feel it</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Эмоциональная вершина страницы и всё по каталогу, но фраза перечисляет семь прилагательных — список, не фраза. В кадре маска «turned nearly invisible» — продукт должен читаться: края, вырезы, голубой оттенок, капли.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Feel it</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Эмоциональный пик и лучший кадр, все слова из каталога. Но четыре клаузы и четыре лейбла повторяют друг друга. На десктопе на пике убеждения нет ни одной кнопки — добавить secondary «Contact for price». Нужен видимый влажный край листа, иначе продукт исчезает из кадра.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Главный блок для косметолога — без времени экспозиции («сколько держать?» — первый вопрос, в каталоге ответа нет); шаг «Remove» обрывается, хотя каталог на стр. 7, 9, 19 даёт финиш EXOCELL → DERMA RECOVERY → солнцезащита. Триптих одной женщины в одном 16:9 генератор держит плохо.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Строка повторяет блок 2 и блок 3; лейбл 2 — предложение, а не ярлык; «Works with» дублирует чипы блока 1. Триптих в одном 16:9 не сгенерируется стабильно, луп капель — лишняя генерация. Одна сцена (маска снята), три шага — типографикой.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Ключевой блок для владельца клиники (как встроить в рабочий процесс), но без времени экспозиции пуст — каталог его не даёт, нужен ответ редактора, не выдумка. Чипы длинные, четвёртый — предложение; триптих с одной женщиной в трёх позах — зона риска по консистентности.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Самый перегруженный блок: строка из 3 клауз + 4 лейбла + ряд чипов «Works with» + CTA + триптих + луп. Триптих — худшее задание для генератора (разные лица в панелях). «Cleansed skin» есть только в спеке, не в каталоге.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Kit &amp; facts</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>«Факты» без фактов: два чипа из четырёх повторяют хедер; нет того, что нужно для заказа — объёма (на коробке 5 × 25 ml, в каталоге нет), хранения, «professional use only»; «one per client» логично, но не написано в источниках. Одноразовая маска на мокром камне читается негигиенично.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Kit &amp; facts</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>«One per client» и «one finishing step per protocol» — выводы, не факты; «single-use» есть лишь в спеке; чипы «Bio-cellulose» и «Post-procedure finish» повторяют блок 0. Фактов для закупщика (объём, срок, хранение) нет. Кадр — лучший продуктовый still life страницы, годится как hero и финал.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Kit &amp; facts</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>«5 masks per box» — главный B2B-факт (пять клиентов, расчёт себестоимости процедуры), но два чипа из четырёх дословно повторяют блок 0 и место пропадает; сюда просятся «For professional use only» и показания — то, что владелец клиники проверяет перед заказом.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Kit &amp; facts</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Единственный факт для unit-экономики нужен, но блок назван «trust» и доверия не несёт: лейблы повторяют блок 0, «one per client» — вывод, «single-use» только в спеке. Кадр почти дублирует hero, реальный пакшот уже показывает раскрытую маску. Слить в Offer — минус кадр и переход.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Клиент — косметолог</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Всё прослеживается (training — стр. 3, exclusive VM importer — стр. 5); «Add to a V-TECH / EXO-NAD enquiry» — именно так я буду заказывать. Но три уровня CTA + контакты + четыре чипа + логотип — перегруз; «VM» без «Italy» косметологу ничего не говорит; кадр — зеркало блока 0, генерировать не нужно.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Главный редактор</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>Строка почти дословно повторяет блок 0 («the soothing finishing step … every …»); «Contact for price» дублирует кнопку, «Finishes every advanced protocol» дублирует строку — живых лейблов два; четыре CTA в блоке «одна фраза». Отдельная генерация не нужна — кадр блока 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>CEO MITODERM</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Структура оффера верная для B2B (контакт за ценой, обучение, эксклюзивный импортёр VM), но чип «Contact for price» дублирует кнопку, «every» — переобещание, а главный коммерческий ход «Add to a V-TECH / EXO-NAD enquiry» спрятан во вторую кнопку, хотя маска по каталогу — довесок к этим протоколам.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Маркетинг и конверсия</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>rewrite</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Механика правильная: WhatsApp + форма, вторичный CTA «добавить к запросу» — лучший кросс-селл. Но половина лейблов потрачена впустую (дубли кнопки и строки). Зеркало блока 0 — бесплатный кадр; idle-луп делать CSS. «For professional use only» в каталоге стоит на странице V-TECH, не EXOCELL.</t>
         </is>
       </c>
     </row>

</xml_diff>